<commit_message>
Adapt extractor to new Excel templates and workflow runner updates
</commit_message>
<xml_diff>
--- a/output/shocapp_da_ordinare.xlsx
+++ b/output/shocapp_da_ordinare.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C82"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,29 +434,29 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>BACIO DEL PRINCIPE</v>
+        <v>GIANDUIA VARIEGATA</v>
       </c>
       <c r="B4" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C4" t="str">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>BANANA E LIME</v>
+        <v>BACIO DEL PRINCIPE</v>
       </c>
       <c r="B5" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C5" t="str">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>CACHI</v>
+        <v>BANANA E LIME</v>
       </c>
       <c r="B6" t="str">
         <v>Da Ordinare</v>
@@ -467,7 +467,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>CIOCCOLATO</v>
+        <v>BASILICO NOCI E MIELE</v>
       </c>
       <c r="B7" t="str">
         <v>Da Ordinare</v>
@@ -478,7 +478,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>CIOCCOLATO AL LATTE gelato</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="B8" t="str">
         <v>Da Ordinare</v>
@@ -489,7 +489,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>CIOCCOLATO AL PIMENTO</v>
+        <v>CAFFE'</v>
       </c>
       <c r="B9" t="str">
         <v>Da Ordinare</v>
@@ -500,117 +500,117 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>CIOCCOLATO E ARANCIA</v>
+        <v>CACHI</v>
       </c>
       <c r="B10" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C10" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>CIOCCOLATO KENTUCKY</v>
+        <v>CIOCCOLATO</v>
       </c>
       <c r="B11" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C11" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
+        <v>CIOCCOLATO AL LATTE gelato</v>
       </c>
       <c r="B12" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C12" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>CIOCCOLATO AL PIMENTO</v>
       </c>
       <c r="B13" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C13" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CIOCCOLATO VENEZUELA</v>
+        <v>CIOCCOLATO E ARANCIA</v>
       </c>
       <c r="B14" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C14" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>COCCO CREMA</v>
+        <v>CIOCCOLATO KENTUCKY</v>
       </c>
       <c r="B15" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C15" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CREMA  PASTICCIERA PARISI</v>
+        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
       </c>
       <c r="B16" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C16" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>CREMA CANNELLA</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="B17" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C17" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>CREMA FRAGOLE E MANDORLE</v>
+        <v>CIOCCOLATO VENEZUELA</v>
       </c>
       <c r="B18" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C18" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CREMA VANIGLIA</v>
+        <v>COCCO CREMA</v>
       </c>
       <c r="B19" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C19" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
+        <v>CREMA  PASTICCIERA PARISI</v>
       </c>
       <c r="B20" t="str">
         <v>Da Ordinare</v>
@@ -621,18 +621,18 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>FIORDILATTE</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="B21" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C21" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>FRAGOLA</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="B22" t="str">
         <v>Da Ordinare</v>
@@ -643,18 +643,18 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>LEMON CURD</v>
+        <v>CREMA FRAGOLE E MANDORLE</v>
       </c>
       <c r="B23" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C23" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>LIMONE</v>
+        <v>CREMA VANIGLIA</v>
       </c>
       <c r="B24" t="str">
         <v>Da Ordinare</v>
@@ -665,29 +665,29 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
       </c>
       <c r="B25" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C25" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>FIORDILATTE</v>
       </c>
       <c r="B26" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C26" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>FRAGOLA</v>
       </c>
       <c r="B27" t="str">
         <v>Da Ordinare</v>
@@ -698,7 +698,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>MELA MANDORLA E CANNELLA</v>
+        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
       </c>
       <c r="B28" t="str">
         <v>Da Ordinare</v>
@@ -709,18 +709,18 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>MORA</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B29" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C29" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>LATTE MENTA E CIOCCOLATO</v>
       </c>
       <c r="B30" t="str">
         <v>Da Ordinare</v>
@@ -731,7 +731,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>NOCCIOLA</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="B31" t="str">
         <v>Da Ordinare</v>
@@ -742,18 +742,18 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>LIMONE</v>
       </c>
       <c r="B32" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C32" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>PASSION FRUIT</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B33" t="str">
         <v>Da Ordinare</v>
@@ -764,51 +764,51 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>PERA</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B34" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C34" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>PERE BELLE HELENE</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B35" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C35" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="B36" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C36" t="str">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="B37" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C37" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>MELA MANDORLA E CANNELLA</v>
       </c>
       <c r="B38" t="str">
         <v>Da Ordinare</v>
@@ -819,18 +819,18 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>STRACCIATELLA</v>
+        <v>MORA</v>
       </c>
       <c r="B39" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C39" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>TIRAMISU'</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B40" t="str">
         <v>Da Ordinare</v>
@@ -841,7 +841,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>CIOCCOLATO WASABI</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B41" t="str">
         <v>Da Ordinare</v>
@@ -852,18 +852,18 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
       </c>
       <c r="B42" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C42" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>PENSIERO</v>
+        <v>PAPAYA</v>
       </c>
       <c r="B43" t="str">
         <v>Da Ordinare</v>
@@ -874,7 +874,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="B44" t="str">
         <v>Da Ordinare</v>
@@ -885,29 +885,29 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>PERE BELLE HELENE</v>
       </c>
       <c r="B45" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C45" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>MONT BLANC</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="B46" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C46" t="str">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ZABAIONE AL SAKE'</v>
+        <v>POLLICINA</v>
       </c>
       <c r="B47" t="str">
         <v>Da Ordinare</v>
@@ -918,40 +918,40 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B48" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C48" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="B49" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C49" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>SACHER TORTE</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B50" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C50" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>CASTAGNA AL WHISKY</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B51" t="str">
         <v>Da Ordinare</v>
@@ -962,128 +962,128 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B52" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C52" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ALBICOCCA</v>
+        <v>CIOCCOLATO WASABI</v>
       </c>
       <c r="B53" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C53" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ANANAS E ZENZERO</v>
+        <v>ZABAIONE GELATO</v>
       </c>
       <c r="B54" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C54" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>BASILICO NOCI E MIELE</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
       </c>
       <c r="B55" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C55" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>BIANCANEVE</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B56" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C56" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>CAFFE'</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="B57" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C57" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>AVOCADO LIME E VINO BIANCO</v>
       </c>
       <c r="B58" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C58" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>CIOCCOLATO CRUDO DEL PERU'</v>
+        <v>ZABAIONE AL SAKE'</v>
       </c>
       <c r="B59" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C59" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>CREMA AGNESE</v>
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
       </c>
       <c r="B60" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C60" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
+        <v>SACHER TORTE</v>
       </c>
       <c r="B61" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C61" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
+        <v>CASTAGNA AL WHISKY</v>
       </c>
       <c r="B62" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C62" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
       </c>
       <c r="B63" t="str">
         <v>Da Ordinare</v>
@@ -1094,7 +1094,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>LATTE MENTA E CIOCCOLATO</v>
+        <v>ALBICOCCA</v>
       </c>
       <c r="B64" t="str">
         <v>Da Ordinare</v>
@@ -1105,18 +1105,18 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>ANANAS E ZENZERO</v>
       </c>
       <c r="B65" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C65" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>MIRTILLO</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="B66" t="str">
         <v>Da Ordinare</v>
@@ -1127,7 +1127,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>NOCCIOLA AL FRUTTOSIO</v>
+        <v>CIOCCOLATO CRUDO DEL PERU'</v>
       </c>
       <c r="B67" t="str">
         <v>Da Ordinare</v>
@@ -1138,18 +1138,18 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="B68" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C68" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>POLLICINA</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="B69" t="str">
         <v>Da Ordinare</v>
@@ -1160,7 +1160,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>SEADAS</v>
+        <v>NOCCIOLA AL FRUTTOSIO</v>
       </c>
       <c r="B70" t="str">
         <v>Da Ordinare</v>
@@ -1171,7 +1171,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>YOGURT</v>
+        <v>PERA</v>
       </c>
       <c r="B71" t="str">
         <v>Da Ordinare</v>
@@ -1182,7 +1182,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="B72" t="str">
         <v>Da Ordinare</v>
@@ -1193,7 +1193,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>SACRIPANTE</v>
+        <v>SEADAS</v>
       </c>
       <c r="B73" t="str">
         <v>Da Ordinare</v>
@@ -1204,18 +1204,18 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>CIOCCOLATA CALDA FONDENTE</v>
+        <v>YOGURT</v>
       </c>
       <c r="B74" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C74" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>SEMIFREDDO  TIRAMISU</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B75" t="str">
         <v>Da Ordinare</v>
@@ -1226,29 +1226,84 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>CREMA MASCARPONE</v>
+        <v>ROSA KARKADE E ARANCIA</v>
       </c>
       <c r="B76" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C76" t="str">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+        <v>SEMIFREDDO  TIRAMISU</v>
       </c>
       <c r="B77" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C77" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>MONT BLANC</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C78" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>TORTA CAPRESE</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C79" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>EVERGREEN  BRONTE VEGAN</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C80" t="str">
         <v>3</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C81" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>CREMA MASCARPONE</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C82" t="str">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C77"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C82"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly SHOCAPP data 2026-03-22
</commit_message>
<xml_diff>
--- a/output/shocapp_da_ordinare.xlsx
+++ b/output/shocapp_da_ordinare.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C105"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,7 +412,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>AMARENA</v>
+        <v>ALBICOCCA</v>
       </c>
       <c r="B2" t="str">
         <v>Da Ordinare</v>
@@ -423,62 +423,62 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ARACHIDI COCCO E CIOCCOLATO</v>
+        <v>AMARENA</v>
       </c>
       <c r="B3" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C3" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>GIANDUIA VARIEGATA</v>
+        <v>ANANAS E ZENZERO</v>
       </c>
       <c r="B4" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C4" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>BACIO DEL PRINCIPE</v>
+        <v>GIANDUIA VARIEGATA</v>
       </c>
       <c r="B5" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C5" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BANANA E LIME</v>
+        <v>BACIO DEL PRINCIPE</v>
       </c>
       <c r="B6" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C6" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>BASILICO NOCI E MIELE</v>
+        <v>BANANA E LIME</v>
       </c>
       <c r="B7" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C7" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>BIANCANEVE</v>
+        <v>BASILICO NOCI E MIELE</v>
       </c>
       <c r="B8" t="str">
         <v>Da Ordinare</v>
@@ -489,18 +489,18 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>CAFFE'</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="B9" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C9" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>CACHI</v>
+        <v>CAFFE'</v>
       </c>
       <c r="B10" t="str">
         <v>Da Ordinare</v>
@@ -511,13 +511,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>CIOCCOLATO</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="B11" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C11" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -544,7 +544,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CIOCCOLATO E ARANCIA</v>
+        <v>CIOCCOLATO CRUDO DEL PERU'</v>
       </c>
       <c r="B14" t="str">
         <v>Da Ordinare</v>
@@ -555,40 +555,40 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CIOCCOLATO KENTUCKY</v>
+        <v>CIOCCOLATO E ARANCIA</v>
       </c>
       <c r="B15" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C15" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
+        <v>CIOCCOLATO KENTUCKY</v>
       </c>
       <c r="B16" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C16" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
       </c>
       <c r="B17" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C17" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>CIOCCOLATO VENEZUELA</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="B18" t="str">
         <v>Da Ordinare</v>
@@ -599,7 +599,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>COCCO CREMA</v>
+        <v>CIOCCOLATO VENEZUELA</v>
       </c>
       <c r="B19" t="str">
         <v>Da Ordinare</v>
@@ -610,7 +610,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CREMA  PASTICCIERA PARISI</v>
+        <v>COCCO CREMA</v>
       </c>
       <c r="B20" t="str">
         <v>Da Ordinare</v>
@@ -621,7 +621,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
+        <v>CREMA  PASTICCIERA PARISI</v>
       </c>
       <c r="B21" t="str">
         <v>Da Ordinare</v>
@@ -632,7 +632,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CREMA CANNELLA</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="B22" t="str">
         <v>Da Ordinare</v>
@@ -643,7 +643,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>CREMA FRAGOLE E MANDORLE</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="B23" t="str">
         <v>Da Ordinare</v>
@@ -654,7 +654,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>CREMA VANIGLIA</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="B24" t="str">
         <v>Da Ordinare</v>
@@ -665,7 +665,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
+        <v>CREMA FRAGOLE E MANDORLE</v>
       </c>
       <c r="B25" t="str">
         <v>Da Ordinare</v>
@@ -676,7 +676,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>FIORDILATTE</v>
+        <v>ESTASI</v>
       </c>
       <c r="B26" t="str">
         <v>Da Ordinare</v>
@@ -693,34 +693,34 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C27" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B28" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C28" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>LATTE MENTA E CIOCCOLATO</v>
       </c>
       <c r="B29" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C29" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>LATTE MENTA E CIOCCOLATO</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="B30" t="str">
         <v>Da Ordinare</v>
@@ -731,29 +731,29 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>LEMON CURD</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B31" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C31" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>LIMONE</v>
+        <v>MELA MANDORLA E CANNELLA</v>
       </c>
       <c r="B32" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C32" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>LIQUIRIZIA</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="B33" t="str">
         <v>Da Ordinare</v>
@@ -764,7 +764,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>PERA</v>
       </c>
       <c r="B34" t="str">
         <v>Da Ordinare</v>
@@ -775,7 +775,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>PERE BELLE HELENE</v>
       </c>
       <c r="B35" t="str">
         <v>Da Ordinare</v>
@@ -786,7 +786,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="B36" t="str">
         <v>Da Ordinare</v>
@@ -797,29 +797,29 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="B37" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C37" t="str">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>MELA MANDORLA E CANNELLA</v>
+        <v>POLLICINA</v>
       </c>
       <c r="B38" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C38" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>MORA</v>
+        <v>PUNCH PARADISE</v>
       </c>
       <c r="B39" t="str">
         <v>Da Ordinare</v>
@@ -830,7 +830,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B40" t="str">
         <v>Da Ordinare</v>
@@ -841,7 +841,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>NOCCIOLA</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="B41" t="str">
         <v>Da Ordinare</v>
@@ -852,7 +852,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>SEADAS</v>
       </c>
       <c r="B42" t="str">
         <v>Da Ordinare</v>
@@ -863,18 +863,18 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>PAPAYA</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B43" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C43" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>PASSION FRUIT</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B44" t="str">
         <v>Da Ordinare</v>
@@ -885,29 +885,29 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>PERE BELLE HELENE</v>
+        <v>CIOCCOLATO WASABI</v>
       </c>
       <c r="B45" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C45" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>YOGURT</v>
       </c>
       <c r="B46" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C46" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>POLLICINA</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
       </c>
       <c r="B47" t="str">
         <v>Da Ordinare</v>
@@ -918,7 +918,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>PENSIERO</v>
       </c>
       <c r="B48" t="str">
         <v>Da Ordinare</v>
@@ -929,40 +929,40 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B49" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C49" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>STRACCIATELLA</v>
+        <v>BUONGIORNO AMORE</v>
       </c>
       <c r="B50" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C50" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>TIRAMISU'</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B51" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C51" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>UVA E NOCI</v>
+        <v>CARROT CAKE</v>
       </c>
       <c r="B52" t="str">
         <v>Da Ordinare</v>
@@ -973,29 +973,29 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>CIOCCOLATO WASABI</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="B53" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C53" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>MONT BLANC</v>
       </c>
       <c r="B54" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C54" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+        <v>ZABAIONE AL SAKE'</v>
       </c>
       <c r="B55" t="str">
         <v>Da Ordinare</v>
@@ -1006,7 +1006,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>SACHER TORTE</v>
       </c>
       <c r="B56" t="str">
         <v>Da Ordinare</v>
@@ -1017,18 +1017,18 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
       </c>
       <c r="B57" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C57" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>AVOCADO LIME E VINO BIANCO</v>
+        <v>PISTACCHIO LARNAKA , CIPRO</v>
       </c>
       <c r="B58" t="str">
         <v>Da Ordinare</v>
@@ -1039,7 +1039,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ZABAIONE AL SAKE'</v>
+        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
       </c>
       <c r="B59" t="str">
         <v>Da Ordinare</v>
@@ -1050,7 +1050,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+        <v>ZABAIONE NEW</v>
       </c>
       <c r="B60" t="str">
         <v>Da Ordinare</v>
@@ -1061,29 +1061,29 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>SACHER TORTE</v>
+        <v>ANGURIA</v>
       </c>
       <c r="B61" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C61" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>CASTAGNA AL WHISKY</v>
+        <v>ARACHIDI COCCO E CIOCCOLATO</v>
       </c>
       <c r="B62" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C62" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+        <v>BAKLAVA</v>
       </c>
       <c r="B63" t="str">
         <v>Da Ordinare</v>
@@ -1094,7 +1094,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>ALBICOCCA</v>
+        <v>CACHI</v>
       </c>
       <c r="B64" t="str">
         <v>Da Ordinare</v>
@@ -1105,18 +1105,18 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>ANANAS E ZENZERO</v>
+        <v>CIOCCOLATO</v>
       </c>
       <c r="B65" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C65" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
       </c>
       <c r="B66" t="str">
         <v>Da Ordinare</v>
@@ -1127,18 +1127,18 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>CIOCCOLATO CRUDO DEL PERU'</v>
+        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
       </c>
       <c r="B67" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C67" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>CREMA AGNESE</v>
+        <v>FIORDILATTE</v>
       </c>
       <c r="B68" t="str">
         <v>Da Ordinare</v>
@@ -1149,29 +1149,29 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>MIRTILLO</v>
+        <v>GIANDUIA</v>
       </c>
       <c r="B69" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C69" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>NOCCIOLA AL FRUTTOSIO</v>
+        <v>LIMONE</v>
       </c>
       <c r="B70" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C70" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>PERA</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B71" t="str">
         <v>Da Ordinare</v>
@@ -1182,7 +1182,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B72" t="str">
         <v>Da Ordinare</v>
@@ -1193,40 +1193,40 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>SEADAS</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="B73" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C73" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>YOGURT</v>
+        <v>MANDORLA TOSTATA</v>
       </c>
       <c r="B74" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C74" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>SACRIPANTE</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="B75" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C75" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>ROSA KARKADE E ARANCIA</v>
+        <v>MORA</v>
       </c>
       <c r="B76" t="str">
         <v>Da Ordinare</v>
@@ -1237,40 +1237,40 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>SEMIFREDDO  TIRAMISU</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B77" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C77" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>MONT BLANC</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B78" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C78" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>TORTA CAPRESE</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="B79" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C79" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B80" t="str">
         <v>Da Ordinare</v>
@@ -1281,40 +1281,40 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+        <v>ZABAIONE GELATO</v>
       </c>
       <c r="B81" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C81" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>CREMA MASCARPONE</v>
+        <v>FIOR DI CIOCCOLATO</v>
       </c>
       <c r="B82" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C82" t="str">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>PENSIERO</v>
+        <v>AVOCADO LIME E VINO BIANCO</v>
       </c>
       <c r="B83" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C83" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>CIOCCOLATA CALDA FONDENTE</v>
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
       </c>
       <c r="B84" t="str">
         <v>Da Ordinare</v>
@@ -1325,18 +1325,18 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>BAKLAVA</v>
+        <v>EVERGREEN  BRONTE VEGAN</v>
       </c>
       <c r="B85" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C85" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>CASTAGNA E MIRTO</v>
+        <v>CASTAGNA AL WHISKY</v>
       </c>
       <c r="B86" t="str">
         <v>Da Ordinare</v>
@@ -1347,40 +1347,40 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>ESTASI</v>
+        <v>CREMA MASCARPONE</v>
       </c>
       <c r="B87" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C87" t="str">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>FICHI</v>
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
       </c>
       <c r="B88" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C88" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>RICOTTA, MIELE E COCCO</v>
+        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
       </c>
       <c r="B89" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C89" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>UVA FRAGOLA E ZENZERO</v>
+        <v>NOCCIOLA AL FRUTTOSIO</v>
       </c>
       <c r="B90" t="str">
         <v>Da Ordinare</v>
@@ -1391,7 +1391,7 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>CARROT CAKE</v>
+        <v>ROSA KARKADE E ARANCIA</v>
       </c>
       <c r="B91" t="str">
         <v>Da Ordinare</v>
@@ -1402,18 +1402,18 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
+        <v>TORTA CAPRESE</v>
       </c>
       <c r="B92" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C92" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>GIANDUIA</v>
+        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
       </c>
       <c r="B93" t="str">
         <v>Da Ordinare</v>
@@ -1424,7 +1424,7 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>BUONGIORNO AMORE</v>
+        <v>CIOCCOLATA CALDA FONDENTE</v>
       </c>
       <c r="B94" t="str">
         <v>Da Ordinare</v>
@@ -1435,7 +1435,7 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
+        <v>SEMIFREDDO  TIRAMISU</v>
       </c>
       <c r="B95" t="str">
         <v>Da Ordinare</v>
@@ -1446,7 +1446,7 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>COCONUT RICE CAKE</v>
+        <v>CASTAGNA E MIRTO</v>
       </c>
       <c r="B96" t="str">
         <v>Da Ordinare</v>
@@ -1457,29 +1457,29 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>CASTAGNACCIO</v>
+        <v>CREMA VANIGLIA</v>
       </c>
       <c r="B97" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C97" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>TORRONE SALATO</v>
+        <v>FICHI</v>
       </c>
       <c r="B98" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C98" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>MANDARINO</v>
+        <v>RICOTTA, MIELE E COCCO</v>
       </c>
       <c r="B99" t="str">
         <v>Da Ordinare</v>
@@ -1490,18 +1490,73 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>GELATO DI PANETTONE</v>
+        <v>UVA FRAGOLA E ZENZERO</v>
       </c>
       <c r="B100" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C100" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C101" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
+      </c>
+      <c r="B102" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C102" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>COCONUT RICE CAKE</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C103" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>CASTAGNACCIO</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C104" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>TORRONE SALATO</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C105" t="str">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C100"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C105"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly SHOCAPP data 2026-03-29
</commit_message>
<xml_diff>
--- a/output/shocapp_da_ordinare.xlsx
+++ b/output/shocapp_da_ordinare.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C104"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,7 +412,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ALBICOCCA</v>
+        <v>AMARENA</v>
       </c>
       <c r="B2" t="str">
         <v>Da Ordinare</v>
@@ -423,24 +423,24 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>AMARENA</v>
+        <v>ANANAS E ZENZERO</v>
       </c>
       <c r="B3" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C3" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ANANAS E ZENZERO</v>
+        <v>ANGURIA</v>
       </c>
       <c r="B4" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C4" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -462,7 +462,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C6" t="str">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -473,45 +473,45 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C7" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>BASILICO NOCI E MIELE</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="B8" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C8" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>BIANCANEVE</v>
+        <v>CAFFE'</v>
       </c>
       <c r="B9" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C9" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>CAFFE'</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="B10" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C10" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>CIOCCOLATO CRUDO DEL PERU'</v>
       </c>
       <c r="B11" t="str">
         <v>Da Ordinare</v>
@@ -522,18 +522,18 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CIOCCOLATO AL LATTE gelato</v>
+        <v>CIOCCOLATO E ARANCIA</v>
       </c>
       <c r="B12" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C12" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>CIOCCOLATO AL PIMENTO</v>
+        <v>CIOCCOLATO KENTUCKY</v>
       </c>
       <c r="B13" t="str">
         <v>Da Ordinare</v>
@@ -544,18 +544,18 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CIOCCOLATO CRUDO DEL PERU'</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="B14" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C14" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CIOCCOLATO E ARANCIA</v>
+        <v>COCCO CREMA</v>
       </c>
       <c r="B15" t="str">
         <v>Da Ordinare</v>
@@ -566,7 +566,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CIOCCOLATO KENTUCKY</v>
+        <v>CREMA  PASTICCIERA PARISI</v>
       </c>
       <c r="B16" t="str">
         <v>Da Ordinare</v>
@@ -577,18 +577,18 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="B17" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C17" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="B18" t="str">
         <v>Da Ordinare</v>
@@ -599,7 +599,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CIOCCOLATO VENEZUELA</v>
+        <v>CREMA FRAGOLE E MANDORLE</v>
       </c>
       <c r="B19" t="str">
         <v>Da Ordinare</v>
@@ -610,7 +610,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>COCCO CREMA</v>
+        <v>CREMA VANIGLIA</v>
       </c>
       <c r="B20" t="str">
         <v>Da Ordinare</v>
@@ -621,18 +621,18 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>CREMA  PASTICCIERA PARISI</v>
+        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
       </c>
       <c r="B21" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C21" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CREMA AGNESE</v>
+        <v>FIORDILATTE</v>
       </c>
       <c r="B22" t="str">
         <v>Da Ordinare</v>
@@ -643,62 +643,62 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
+        <v>FRAGOLA</v>
       </c>
       <c r="B23" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C23" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>CREMA CANNELLA</v>
+        <v>GIANDUIA</v>
       </c>
       <c r="B24" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C24" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>CREMA FRAGOLE E MANDORLE</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B25" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C25" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ESTASI</v>
+        <v>LATTE MENTA E CIOCCOLATO</v>
       </c>
       <c r="B26" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C26" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>FRAGOLA</v>
+        <v>LIMONE</v>
       </c>
       <c r="B27" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C27" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B28" t="str">
         <v>Da Ordinare</v>
@@ -709,7 +709,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>LATTE MENTA E CIOCCOLATO</v>
+        <v>MANDARINO</v>
       </c>
       <c r="B29" t="str">
         <v>Da Ordinare</v>
@@ -720,40 +720,40 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>LEMON CURD</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B30" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C30" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="B31" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C31" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>MELA MANDORLA E CANNELLA</v>
+        <v>MANDORLA TOSTATA</v>
       </c>
       <c r="B32" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C32" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>MIRTILLO</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="B33" t="str">
         <v>Da Ordinare</v>
@@ -764,51 +764,51 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>PERA</v>
+        <v>MELA MANDORLA E CANNELLA</v>
       </c>
       <c r="B34" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C34" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>PERE BELLE HELENE</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="B35" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C35" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B36" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C36" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B37" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C37" t="str">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>POLLICINA</v>
+        <v>NOCCIOLA AL FRUTTOSIO</v>
       </c>
       <c r="B38" t="str">
         <v>Da Ordinare</v>
@@ -819,29 +819,29 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>PUNCH PARADISE</v>
+        <v>PERA</v>
       </c>
       <c r="B39" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C39" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="B40" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C40" t="str">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>PUNCH PARADISE</v>
       </c>
       <c r="B41" t="str">
         <v>Da Ordinare</v>
@@ -852,29 +852,29 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>SEADAS</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B42" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C42" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>STRACCIATELLA</v>
+        <v>RICOTTA, MIELE E COCCO</v>
       </c>
       <c r="B43" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C43" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>UVA E NOCI</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="B44" t="str">
         <v>Da Ordinare</v>
@@ -885,7 +885,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>CIOCCOLATO WASABI</v>
+        <v>SEADAS</v>
       </c>
       <c r="B45" t="str">
         <v>Da Ordinare</v>
@@ -896,18 +896,18 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>YOGURT</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B46" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C46" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B47" t="str">
         <v>Da Ordinare</v>
@@ -918,7 +918,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>PENSIERO</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B48" t="str">
         <v>Da Ordinare</v>
@@ -929,7 +929,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>SACRIPANTE</v>
+        <v>CIOCCOLATO WASABI</v>
       </c>
       <c r="B49" t="str">
         <v>Da Ordinare</v>
@@ -940,29 +940,29 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>BUONGIORNO AMORE</v>
+        <v>YOGURT</v>
       </c>
       <c r="B50" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C50" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>PENSIERO</v>
       </c>
       <c r="B51" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C51" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>CARROT CAKE</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B52" t="str">
         <v>Da Ordinare</v>
@@ -973,51 +973,51 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>BUONGIORNO AMORE</v>
       </c>
       <c r="B53" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C53" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>MONT BLANC</v>
+        <v>CARROT CAKE</v>
       </c>
       <c r="B54" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C54" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ZABAIONE AL SAKE'</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="B55" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C55" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>SACHER TORTE</v>
+        <v>FIOR DI CIOCCOLATO</v>
       </c>
       <c r="B56" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C56" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+        <v>AVOCADO LIME E VINO BIANCO</v>
       </c>
       <c r="B57" t="str">
         <v>Da Ordinare</v>
@@ -1028,7 +1028,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>PISTACCHIO LARNAKA , CIPRO</v>
+        <v>MONT BLANC</v>
       </c>
       <c r="B58" t="str">
         <v>Da Ordinare</v>
@@ -1039,7 +1039,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
+        <v>PASTIERA NAPOLETANA</v>
       </c>
       <c r="B59" t="str">
         <v>Da Ordinare</v>
@@ -1050,7 +1050,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ZABAIONE NEW</v>
+        <v>ZABAIONE AL SAKE'</v>
       </c>
       <c r="B60" t="str">
         <v>Da Ordinare</v>
@@ -1061,106 +1061,106 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ANGURIA</v>
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
       </c>
       <c r="B61" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C61" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ARACHIDI COCCO E CIOCCOLATO</v>
+        <v>EVERGREEN  BRONTE VEGAN</v>
       </c>
       <c r="B62" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C62" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>BAKLAVA</v>
+        <v>SACHER TORTE</v>
       </c>
       <c r="B63" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C63" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>CACHI</v>
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
       </c>
       <c r="B64" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C64" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>CIOCCOLATO</v>
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
       </c>
       <c r="B65" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C65" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
+        <v>PISTACCHIO LARNAKA , CIPRO</v>
       </c>
       <c r="B66" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C66" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
+        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
       </c>
       <c r="B67" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C67" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>FIORDILATTE</v>
+        <v>ZABAIONE NEW</v>
       </c>
       <c r="B68" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C68" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>GIANDUIA</v>
+        <v>ALBICOCCA</v>
       </c>
       <c r="B69" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C69" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>LIMONE</v>
+        <v>ARACHIDI COCCO E CIOCCOLATO</v>
       </c>
       <c r="B70" t="str">
         <v>Da Ordinare</v>
@@ -1171,7 +1171,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>LIQUIRIZIA</v>
+        <v>BASILICO NOCI E MIELE</v>
       </c>
       <c r="B71" t="str">
         <v>Da Ordinare</v>
@@ -1182,7 +1182,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>CACHI</v>
       </c>
       <c r="B72" t="str">
         <v>Da Ordinare</v>
@@ -1193,29 +1193,29 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>CIOCCOLATO</v>
       </c>
       <c r="B73" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C73" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>MANDORLA TOSTATA</v>
+        <v>CIOCCOLATO AL LATTE gelato</v>
       </c>
       <c r="B74" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C74" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>CIOCCOLATO VENEZUELA</v>
       </c>
       <c r="B75" t="str">
         <v>Da Ordinare</v>
@@ -1226,62 +1226,62 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>MORA</v>
+        <v>ESTASI</v>
       </c>
       <c r="B76" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C76" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
       </c>
       <c r="B77" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C77" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>NOCCIOLA</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B78" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C78" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>PASSION FRUIT</v>
+        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
       </c>
       <c r="B79" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C79" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>TIRAMISU'</v>
+        <v>PAPAYA</v>
       </c>
       <c r="B80" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C80" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>PERE BELLE HELENE</v>
       </c>
       <c r="B81" t="str">
         <v>Da Ordinare</v>
@@ -1292,18 +1292,18 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>FIOR DI CIOCCOLATO</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="B82" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C82" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>AVOCADO LIME E VINO BIANCO</v>
+        <v>POLLICINA</v>
       </c>
       <c r="B83" t="str">
         <v>Da Ordinare</v>
@@ -1314,18 +1314,18 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+        <v>ZABAIONE GELATO</v>
       </c>
       <c r="B84" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C84" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
       </c>
       <c r="B85" t="str">
         <v>Da Ordinare</v>
@@ -1336,29 +1336,29 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>CASTAGNA AL WHISKY</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B86" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C86" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>CREMA MASCARPONE</v>
+        <v>ROSA KARKADE E ARANCIA</v>
       </c>
       <c r="B87" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C87" t="str">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+        <v>CASTAGNA AL WHISKY</v>
       </c>
       <c r="B88" t="str">
         <v>Da Ordinare</v>
@@ -1369,18 +1369,18 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
+        <v>CREMA MASCARPONE</v>
       </c>
       <c r="B89" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C89" t="str">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>NOCCIOLA AL FRUTTOSIO</v>
+        <v>COCONUT RICE CAKE</v>
       </c>
       <c r="B90" t="str">
         <v>Da Ordinare</v>
@@ -1391,7 +1391,7 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>ROSA KARKADE E ARANCIA</v>
+        <v>MORA</v>
       </c>
       <c r="B91" t="str">
         <v>Da Ordinare</v>
@@ -1402,18 +1402,18 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>TORTA CAPRESE</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="B92" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C92" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>BAKLAVA</v>
       </c>
       <c r="B93" t="str">
         <v>Da Ordinare</v>
@@ -1424,7 +1424,7 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>CIOCCOLATA CALDA FONDENTE</v>
+        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
       </c>
       <c r="B94" t="str">
         <v>Da Ordinare</v>
@@ -1435,7 +1435,7 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>SEMIFREDDO  TIRAMISU</v>
+        <v>TORTA CAPRESE</v>
       </c>
       <c r="B95" t="str">
         <v>Da Ordinare</v>
@@ -1446,7 +1446,7 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>CASTAGNA E MIRTO</v>
+        <v>CIOCCOLATA CALDA FONDENTE</v>
       </c>
       <c r="B96" t="str">
         <v>Da Ordinare</v>
@@ -1457,7 +1457,7 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>CREMA VANIGLIA</v>
+        <v>SEMIFREDDO  TIRAMISU</v>
       </c>
       <c r="B97" t="str">
         <v>Da Ordinare</v>
@@ -1468,7 +1468,7 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>FICHI</v>
+        <v>CASTAGNA E MIRTO</v>
       </c>
       <c r="B98" t="str">
         <v>Da Ordinare</v>
@@ -1479,7 +1479,7 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>RICOTTA, MIELE E COCCO</v>
+        <v>FICHI</v>
       </c>
       <c r="B99" t="str">
         <v>Da Ordinare</v>
@@ -1512,7 +1512,7 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="B102" t="str">
         <v>Da Ordinare</v>
@@ -1523,7 +1523,7 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>COCONUT RICE CAKE</v>
+        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
       </c>
       <c r="B103" t="str">
         <v>Da Ordinare</v>
@@ -1543,20 +1543,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" t="str">
-        <v>TORRONE SALATO</v>
-      </c>
-      <c r="B105" t="str">
-        <v>Da Ordinare</v>
-      </c>
-      <c r="C105" t="str">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C105"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C104"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly SHOCAPP data 2026-04-05
</commit_message>
<xml_diff>
--- a/output/shocapp_da_ordinare.xlsx
+++ b/output/shocapp_da_ordinare.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C103"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,7 +412,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>AMARENA</v>
+        <v>ANANAS E ZENZERO</v>
       </c>
       <c r="B2" t="str">
         <v>Da Ordinare</v>
@@ -423,7 +423,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ANANAS E ZENZERO</v>
+        <v>ANGURIA</v>
       </c>
       <c r="B3" t="str">
         <v>Da Ordinare</v>
@@ -434,13 +434,13 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ANGURIA</v>
+        <v>ARACHIDI COCCO E CIOCCOLATO</v>
       </c>
       <c r="B4" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C4" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -451,7 +451,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C5" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -462,7 +462,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C6" t="str">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -478,40 +478,40 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>BIANCANEVE</v>
+        <v>BASILICO NOCI E MIELE</v>
       </c>
       <c r="B8" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C8" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>CAFFE'</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="B9" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C9" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>CASTAGNA E MIRTO</v>
       </c>
       <c r="B10" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C10" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>CIOCCOLATO CRUDO DEL PERU'</v>
+        <v>CIOCCOLATO AL LATTE gelato</v>
       </c>
       <c r="B11" t="str">
         <v>Da Ordinare</v>
@@ -522,7 +522,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CIOCCOLATO E ARANCIA</v>
+        <v>CIOCCOLATO CRUDO DEL PERU'</v>
       </c>
       <c r="B12" t="str">
         <v>Da Ordinare</v>
@@ -533,57 +533,57 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>CIOCCOLATO KENTUCKY</v>
+        <v>CIOCCOLATO E ARANCIA</v>
       </c>
       <c r="B13" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C13" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>CIOCCOLATO KENTUCKY</v>
       </c>
       <c r="B14" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C14" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>COCCO CREMA</v>
+        <v>CIOCCOLATO VENEZUELA</v>
       </c>
       <c r="B15" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C15" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CREMA  PASTICCIERA PARISI</v>
+        <v>CIOCCOLATO ROSEMARY</v>
       </c>
       <c r="B16" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C16" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>CREMA AGNESE</v>
+        <v>COCCO CREMA</v>
       </c>
       <c r="B17" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C17" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -599,29 +599,29 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CREMA FRAGOLE E MANDORLE</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="B19" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C19" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CREMA VANIGLIA</v>
+        <v>CREMA FRAGOLE E MANDORLE</v>
       </c>
       <c r="B20" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C20" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
+        <v>CREMA VANIGLIA</v>
       </c>
       <c r="B21" t="str">
         <v>Da Ordinare</v>
@@ -632,7 +632,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>FIORDILATTE</v>
+        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
       </c>
       <c r="B22" t="str">
         <v>Da Ordinare</v>
@@ -643,95 +643,95 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>FRAGOLA</v>
+        <v>ESTASI</v>
       </c>
       <c r="B23" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C23" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>GIANDUIA</v>
+        <v>FIORDILATTE</v>
       </c>
       <c r="B24" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C24" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>FRAGOLA</v>
       </c>
       <c r="B25" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C25" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>LATTE MENTA E CIOCCOLATO</v>
+        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
       </c>
       <c r="B26" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C26" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>LIMONE</v>
+        <v>GIANDUIA</v>
       </c>
       <c r="B27" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C27" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>LIQUIRIZIA</v>
+        <v>LATTE MENTA E CIOCCOLATO</v>
       </c>
       <c r="B28" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C28" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>MANDARINO</v>
+        <v>LIMONE</v>
       </c>
       <c r="B29" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C29" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B30" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C30" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B31" t="str">
         <v>Da Ordinare</v>
@@ -742,18 +742,18 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>MANDORLA TOSTATA</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B32" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C32" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="B33" t="str">
         <v>Da Ordinare</v>
@@ -764,7 +764,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>MELA MANDORLA E CANNELLA</v>
+        <v>MANDORLA TOSTATA</v>
       </c>
       <c r="B34" t="str">
         <v>Da Ordinare</v>
@@ -775,29 +775,29 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>MIRTILLO</v>
+        <v>MELA MANDORLA E CANNELLA</v>
       </c>
       <c r="B35" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C35" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="B36" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C36" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>NOCCIOLA</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B37" t="str">
         <v>Da Ordinare</v>
@@ -808,7 +808,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>NOCCIOLA AL FRUTTOSIO</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B38" t="str">
         <v>Da Ordinare</v>
@@ -819,40 +819,40 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>PERA</v>
+        <v>NOCCIOLA AL FRUTTOSIO</v>
       </c>
       <c r="B39" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C39" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
       </c>
       <c r="B40" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C40" t="str">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>PUNCH PARADISE</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="B41" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C41" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>PERA</v>
       </c>
       <c r="B42" t="str">
         <v>Da Ordinare</v>
@@ -863,51 +863,51 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>RICOTTA, MIELE E COCCO</v>
+        <v>PERE BELLE HELENE</v>
       </c>
       <c r="B43" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C43" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="B44" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C44" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>SEADAS</v>
+        <v>POLLICINA</v>
       </c>
       <c r="B45" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C45" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>STRACCIATELLA</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B46" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C46" t="str">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>TIRAMISU'</v>
+        <v>RICOTTA, MIELE E COCCO</v>
       </c>
       <c r="B47" t="str">
         <v>Da Ordinare</v>
@@ -918,51 +918,51 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>UVA E NOCI</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="B48" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C48" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>CIOCCOLATO WASABI</v>
+        <v>SEADAS</v>
       </c>
       <c r="B49" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C49" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>YOGURT</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B50" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C50" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>PENSIERO</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B51" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C51" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>SACRIPANTE</v>
+        <v>YOGURT</v>
       </c>
       <c r="B52" t="str">
         <v>Da Ordinare</v>
@@ -973,7 +973,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>BUONGIORNO AMORE</v>
+        <v>PENSIERO</v>
       </c>
       <c r="B53" t="str">
         <v>Da Ordinare</v>
@@ -984,40 +984,40 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>CARROT CAKE</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B54" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C54" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B55" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C55" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>FIOR DI CIOCCOLATO</v>
+        <v>CARROT CAKE</v>
       </c>
       <c r="B56" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C56" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>AVOCADO LIME E VINO BIANCO</v>
+        <v>FIOR DI CIOCCOLATO</v>
       </c>
       <c r="B57" t="str">
         <v>Da Ordinare</v>
@@ -1028,7 +1028,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>MONT BLANC</v>
+        <v>ROSA KARKADE E ARANCIA</v>
       </c>
       <c r="B58" t="str">
         <v>Da Ordinare</v>
@@ -1039,18 +1039,18 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>PASTIERA NAPOLETANA</v>
+        <v>AVOCADO LIME E VINO BIANCO</v>
       </c>
       <c r="B59" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C59" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ZABAIONE AL SAKE'</v>
+        <v>MONT BLANC</v>
       </c>
       <c r="B60" t="str">
         <v>Da Ordinare</v>
@@ -1061,7 +1061,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
       </c>
       <c r="B61" t="str">
         <v>Da Ordinare</v>
@@ -1072,7 +1072,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
+        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
       </c>
       <c r="B62" t="str">
         <v>Da Ordinare</v>
@@ -1083,7 +1083,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>SACHER TORTE</v>
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
       </c>
       <c r="B63" t="str">
         <v>Da Ordinare</v>
@@ -1094,18 +1094,18 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+        <v>SACHER TORTE</v>
       </c>
       <c r="B64" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C64" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
       </c>
       <c r="B65" t="str">
         <v>Da Ordinare</v>
@@ -1116,7 +1116,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>PISTACCHIO LARNAKA , CIPRO</v>
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
       </c>
       <c r="B66" t="str">
         <v>Da Ordinare</v>
@@ -1127,18 +1127,18 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
+        <v>COCONUT RICE CAKE</v>
       </c>
       <c r="B67" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C67" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>ZABAIONE NEW</v>
+        <v>PISTACCHIO LARNAKA , CIPRO</v>
       </c>
       <c r="B68" t="str">
         <v>Da Ordinare</v>
@@ -1149,7 +1149,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>ALBICOCCA</v>
+        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
       </c>
       <c r="B69" t="str">
         <v>Da Ordinare</v>
@@ -1160,18 +1160,18 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>ARACHIDI COCCO E CIOCCOLATO</v>
+        <v>ZABAIONE NEW</v>
       </c>
       <c r="B70" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C70" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>BASILICO NOCI E MIELE</v>
+        <v>ALBICOCCA</v>
       </c>
       <c r="B71" t="str">
         <v>Da Ordinare</v>
@@ -1182,7 +1182,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>CACHI</v>
+        <v>AMARENA</v>
       </c>
       <c r="B72" t="str">
         <v>Da Ordinare</v>
@@ -1193,62 +1193,62 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>CIOCCOLATO</v>
+        <v>CAFFE'</v>
       </c>
       <c r="B73" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C73" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>CIOCCOLATO AL LATTE gelato</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="B74" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C74" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>CIOCCOLATO VENEZUELA</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="B75" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C75" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>ESTASI</v>
+        <v>CREMA  PASTICCIERA PARISI</v>
       </c>
       <c r="B76" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C76" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="B77" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C77" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B78" t="str">
         <v>Da Ordinare</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="B79" t="str">
         <v>Da Ordinare</v>
@@ -1270,18 +1270,18 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>PAPAYA</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="B80" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C80" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>PERE BELLE HELENE</v>
+        <v>PAPAYA</v>
       </c>
       <c r="B81" t="str">
         <v>Da Ordinare</v>
@@ -1292,29 +1292,29 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="B82" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C82" t="str">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>POLLICINA</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B83" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C83" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>BUONGIORNO AMORE</v>
       </c>
       <c r="B84" t="str">
         <v>Da Ordinare</v>
@@ -1325,117 +1325,117 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="B85" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C85" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>CIOCCOLATA CALDA FONDENTE</v>
       </c>
       <c r="B86" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C86" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>ROSA KARKADE E ARANCIA</v>
+        <v>PASTIERA NAPOLETANA</v>
       </c>
       <c r="B87" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C87" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>CASTAGNA AL WHISKY</v>
+        <v>ZABAIONE AL SAKE'</v>
       </c>
       <c r="B88" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C88" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>CREMA MASCARPONE</v>
+        <v>TORTA CAPRESE</v>
       </c>
       <c r="B89" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C89" t="str">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>COCONUT RICE CAKE</v>
+        <v>EVERGREEN  BRONTE VEGAN</v>
       </c>
       <c r="B90" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C90" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>MORA</v>
+        <v>CREMA MASCARPONE</v>
       </c>
       <c r="B91" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C91" t="str">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>PASSION FRUIT</v>
+        <v>CACHI</v>
       </c>
       <c r="B92" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C92" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>BAKLAVA</v>
+        <v>CIOCCOLATO</v>
       </c>
       <c r="B93" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C93" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
       </c>
       <c r="B94" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C94" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>TORTA CAPRESE</v>
+        <v>CASTAGNA AL WHISKY</v>
       </c>
       <c r="B95" t="str">
         <v>Da Ordinare</v>
@@ -1446,7 +1446,7 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>CIOCCOLATA CALDA FONDENTE</v>
+        <v>MORA</v>
       </c>
       <c r="B96" t="str">
         <v>Da Ordinare</v>
@@ -1457,18 +1457,18 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>SEMIFREDDO  TIRAMISU</v>
+        <v>ZABAIONE GELATO</v>
       </c>
       <c r="B97" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C97" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>CASTAGNA E MIRTO</v>
+        <v>BAKLAVA</v>
       </c>
       <c r="B98" t="str">
         <v>Da Ordinare</v>
@@ -1479,7 +1479,7 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>FICHI</v>
+        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
       </c>
       <c r="B99" t="str">
         <v>Da Ordinare</v>
@@ -1490,7 +1490,7 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>UVA FRAGOLA E ZENZERO</v>
+        <v>SEMIFREDDO  TIRAMISU</v>
       </c>
       <c r="B100" t="str">
         <v>Da Ordinare</v>
@@ -1501,7 +1501,7 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
+        <v>FICHI</v>
       </c>
       <c r="B101" t="str">
         <v>Da Ordinare</v>
@@ -1512,7 +1512,7 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>CREMA CANNELLA</v>
+        <v>UVA FRAGOLA E ZENZERO</v>
       </c>
       <c r="B102" t="str">
         <v>Da Ordinare</v>
@@ -1523,29 +1523,18 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
+        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
       </c>
       <c r="B103" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C103" t="str">
         <v>1</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="str">
-        <v>CASTAGNACCIO</v>
-      </c>
-      <c r="B104" t="str">
-        <v>Da Ordinare</v>
-      </c>
-      <c r="C104" t="str">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C104"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C103"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly SHOCAPP data 2026-04-12
</commit_message>
<xml_diff>
--- a/output/shocapp_da_ordinare.xlsx
+++ b/output/shocapp_da_ordinare.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C111"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,18 +412,18 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ANANAS E ZENZERO</v>
+        <v>AMARENA</v>
       </c>
       <c r="B2" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C2" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ANGURIA</v>
+        <v>ANANAS E ZENZERO</v>
       </c>
       <c r="B3" t="str">
         <v>Da Ordinare</v>
@@ -434,7 +434,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ARACHIDI COCCO E CIOCCOLATO</v>
+        <v>GIANDUIA VARIEGATA</v>
       </c>
       <c r="B4" t="str">
         <v>Da Ordinare</v>
@@ -445,24 +445,24 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>GIANDUIA VARIEGATA</v>
+        <v>BACIO DEL PRINCIPE</v>
       </c>
       <c r="B5" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C5" t="str">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BACIO DEL PRINCIPE</v>
+        <v>BAKLAVA</v>
       </c>
       <c r="B6" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C6" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -473,7 +473,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C7" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -495,12 +495,12 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C9" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>CASTAGNA E MIRTO</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="B10" t="str">
         <v>Da Ordinare</v>
@@ -517,7 +517,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C11" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -528,7 +528,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C12" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -561,7 +561,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C15" t="str">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -583,12 +583,12 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C17" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
+        <v>CREMA  PASTICCIERA PARISI</v>
       </c>
       <c r="B18" t="str">
         <v>Da Ordinare</v>
@@ -599,29 +599,29 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CREMA CANNELLA</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="B19" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C19" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CREMA FRAGOLE E MANDORLE</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="B20" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C20" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>CREMA VANIGLIA</v>
+        <v>CREMA FRAGOLE E MANDORLE</v>
       </c>
       <c r="B21" t="str">
         <v>Da Ordinare</v>
@@ -632,7 +632,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
+        <v>CREMA VANIGLIA</v>
       </c>
       <c r="B22" t="str">
         <v>Da Ordinare</v>
@@ -643,7 +643,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ESTASI</v>
+        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
       </c>
       <c r="B23" t="str">
         <v>Da Ordinare</v>
@@ -671,29 +671,29 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C25" t="str">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
+        <v>GIANDUIA</v>
       </c>
       <c r="B26" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C26" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>GIANDUIA</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B27" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C27" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -715,7 +715,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C29" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
@@ -726,7 +726,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C30" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -737,7 +737,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C31" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -748,7 +748,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C32" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -764,18 +764,18 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>MANDORLA TOSTATA</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="B34" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C34" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>MELA MANDORLA E CANNELLA</v>
+        <v>MELONE</v>
       </c>
       <c r="B35" t="str">
         <v>Da Ordinare</v>
@@ -797,7 +797,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>MOJITO ALLA AMARENA</v>
       </c>
       <c r="B37" t="str">
         <v>Da Ordinare</v>
@@ -808,7 +808,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>NOCCIOLA</v>
+        <v>MORA</v>
       </c>
       <c r="B38" t="str">
         <v>Da Ordinare</v>
@@ -819,40 +819,40 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>NOCCIOLA AL FRUTTOSIO</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B39" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C39" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B40" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C40" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>PASSION FRUIT</v>
+        <v>NOCCIOLA AL FRUTTOSIO</v>
       </c>
       <c r="B41" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C41" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>PERA</v>
+        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
       </c>
       <c r="B42" t="str">
         <v>Da Ordinare</v>
@@ -863,7 +863,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>PERE BELLE HELENE</v>
+        <v>PERA</v>
       </c>
       <c r="B43" t="str">
         <v>Da Ordinare</v>
@@ -874,7 +874,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>PERE BELLE HELENE</v>
       </c>
       <c r="B44" t="str">
         <v>Da Ordinare</v>
@@ -885,7 +885,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>POLLICINA</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="B45" t="str">
         <v>Da Ordinare</v>
@@ -896,18 +896,18 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="B46" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C46" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>RICOTTA, MIELE E COCCO</v>
+        <v>PUNCH PARADISE</v>
       </c>
       <c r="B47" t="str">
         <v>Da Ordinare</v>
@@ -918,18 +918,18 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B48" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C48" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>SEADAS</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="B49" t="str">
         <v>Da Ordinare</v>
@@ -940,29 +940,29 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>STRACCIATELLA</v>
+        <v>SEADAS</v>
       </c>
       <c r="B50" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C50" t="str">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>TIRAMISU'</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B51" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C51" t="str">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>YOGURT</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B52" t="str">
         <v>Da Ordinare</v>
@@ -973,18 +973,18 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>PENSIERO</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B53" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C53" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>SACRIPANTE</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
       </c>
       <c r="B54" t="str">
         <v>Da Ordinare</v>
@@ -995,29 +995,29 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>PENSIERO</v>
       </c>
       <c r="B55" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C55" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>CARROT CAKE</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B56" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C56" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>FIOR DI CIOCCOLATO</v>
+        <v>BUONGIORNO AMORE</v>
       </c>
       <c r="B57" t="str">
         <v>Da Ordinare</v>
@@ -1028,7 +1028,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ROSA KARKADE E ARANCIA</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B58" t="str">
         <v>Da Ordinare</v>
@@ -1039,29 +1039,29 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>AVOCADO LIME E VINO BIANCO</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="B59" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C59" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>MONT BLANC</v>
+        <v>AVOCADO LIME E VINO BIANCO</v>
       </c>
       <c r="B60" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C60" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
+        <v>MONT BLANC</v>
       </c>
       <c r="B61" t="str">
         <v>Da Ordinare</v>
@@ -1072,7 +1072,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
+        <v>COCCO</v>
       </c>
       <c r="B62" t="str">
         <v>Da Ordinare</v>
@@ -1083,7 +1083,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
       </c>
       <c r="B63" t="str">
         <v>Da Ordinare</v>
@@ -1094,7 +1094,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>SACHER TORTE</v>
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
       </c>
       <c r="B64" t="str">
         <v>Da Ordinare</v>
@@ -1105,57 +1105,57 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+        <v>EVERGREEN  BRONTE VEGAN</v>
       </c>
       <c r="B65" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C65" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+        <v>SACHER TORTE</v>
       </c>
       <c r="B66" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C66" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>COCONUT RICE CAKE</v>
+        <v>CASTAGNA AL WHISKY</v>
       </c>
       <c r="B67" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C67" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>PISTACCHIO LARNAKA , CIPRO</v>
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
       </c>
       <c r="B68" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C68" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
       </c>
       <c r="B69" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C69" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -1171,24 +1171,24 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>ALBICOCCA</v>
+        <v>ANGURIA</v>
       </c>
       <c r="B71" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C71" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>AMARENA</v>
+        <v>ARACHIDI COCCO E CIOCCOLATO</v>
       </c>
       <c r="B72" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C72" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73">
@@ -1199,45 +1199,45 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C73" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>CASTAGNA E MIRTO</v>
       </c>
       <c r="B74" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C74" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>CIOCCOLATO AL PIMENTO</v>
       </c>
       <c r="B75" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C75" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>CREMA  PASTICCIERA PARISI</v>
+        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
       </c>
       <c r="B76" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C76" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>CREMA AGNESE</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="B77" t="str">
         <v>Da Ordinare</v>
@@ -1248,73 +1248,73 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="B78" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C78" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>LEMON CURD</v>
+        <v>ESTASI</v>
       </c>
       <c r="B79" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C79" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
       </c>
       <c r="B80" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C80" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>PAPAYA</v>
+        <v>MANDARINO</v>
       </c>
       <c r="B81" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C81" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>MELA MANDORLA E CANNELLA</v>
       </c>
       <c r="B82" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C82" t="str">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>UVA E NOCI</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="B83" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C83" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>BUONGIORNO AMORE</v>
+        <v>POLLICINA</v>
       </c>
       <c r="B84" t="str">
         <v>Da Ordinare</v>
@@ -1325,18 +1325,18 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>RICOTTA, MIELE E COCCO</v>
       </c>
       <c r="B85" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C85" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>CIOCCOLATA CALDA FONDENTE</v>
+        <v>CIOCCOLATO WASABI</v>
       </c>
       <c r="B86" t="str">
         <v>Da Ordinare</v>
@@ -1347,40 +1347,40 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>PASTIERA NAPOLETANA</v>
+        <v>YOGURT</v>
       </c>
       <c r="B87" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C87" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>ZABAIONE AL SAKE'</v>
+        <v>CARROT CAKE</v>
       </c>
       <c r="B88" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C88" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>TORTA CAPRESE</v>
+        <v>FIOR DI CIOCCOLATO</v>
       </c>
       <c r="B89" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C89" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
+        <v>ROSA KARKADE E ARANCIA</v>
       </c>
       <c r="B90" t="str">
         <v>Da Ordinare</v>
@@ -1391,18 +1391,18 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>CREMA MASCARPONE</v>
+        <v>PASTIERA NAPOLETANA</v>
       </c>
       <c r="B91" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C91" t="str">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>CACHI</v>
+        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
       </c>
       <c r="B92" t="str">
         <v>Da Ordinare</v>
@@ -1413,18 +1413,18 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>CIOCCOLATO</v>
+        <v>CREMA MASCARPONE</v>
       </c>
       <c r="B93" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C93" t="str">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+        <v>COCONUT RICE CAKE</v>
       </c>
       <c r="B94" t="str">
         <v>Da Ordinare</v>
@@ -1435,18 +1435,18 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>CASTAGNA AL WHISKY</v>
+        <v>PISTACCHIO LARNAKA , CIPRO</v>
       </c>
       <c r="B95" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C95" t="str">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>MORA</v>
+        <v>ALBICOCCA</v>
       </c>
       <c r="B96" t="str">
         <v>Da Ordinare</v>
@@ -1457,29 +1457,29 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="B97" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C97" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>BAKLAVA</v>
+        <v>PAPAYA</v>
       </c>
       <c r="B98" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C98" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
+        <v>CIOCCOLATA CALDA FONDENTE</v>
       </c>
       <c r="B99" t="str">
         <v>Da Ordinare</v>
@@ -1490,7 +1490,7 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>SEMIFREDDO  TIRAMISU</v>
+        <v>ZABAIONE AL SAKE'</v>
       </c>
       <c r="B100" t="str">
         <v>Da Ordinare</v>
@@ -1501,7 +1501,7 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>FICHI</v>
+        <v>TORTA CAPRESE</v>
       </c>
       <c r="B101" t="str">
         <v>Da Ordinare</v>
@@ -1512,29 +1512,117 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>UVA FRAGOLA E ZENZERO</v>
+        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
       </c>
       <c r="B102" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C102" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
+        <v>CACHI</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C103" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>CIOCCOLATO</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C104" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>MANDORLA TOSTATA</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C105" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>ZABAIONE GELATO</v>
+      </c>
+      <c r="B106" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C106" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
+      </c>
+      <c r="B107" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C107" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>SEMIFREDDO  TIRAMISU</v>
+      </c>
+      <c r="B108" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C108" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>FICHI</v>
+      </c>
+      <c r="B109" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C109" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>UVA FRAGOLA E ZENZERO</v>
+      </c>
+      <c r="B110" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C110" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
         <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
       </c>
-      <c r="B103" t="str">
-        <v>Da Ordinare</v>
-      </c>
-      <c r="C103" t="str">
+      <c r="B111" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C111" t="str">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C103"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C111"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly SHOCAPP data 2026-04-19
</commit_message>
<xml_diff>
--- a/output/shocapp_da_ordinare.xlsx
+++ b/output/shocapp_da_ordinare.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C110"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,7 +418,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C2" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -429,34 +429,34 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C3" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>GIANDUIA VARIEGATA</v>
+        <v>ANGURIA</v>
       </c>
       <c r="B4" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C4" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>BACIO DEL PRINCIPE</v>
+        <v>ARACHIDI COCCO E CIOCCOLATO</v>
       </c>
       <c r="B5" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C5" t="str">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BAKLAVA</v>
+        <v>BACIO DEL PRINCIPE</v>
       </c>
       <c r="B6" t="str">
         <v>Da Ordinare</v>
@@ -484,7 +484,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C8" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -495,12 +495,12 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C9" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>CAFFE'</v>
       </c>
       <c r="B10" t="str">
         <v>Da Ordinare</v>
@@ -511,106 +511,106 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>CIOCCOLATO AL LATTE gelato</v>
+        <v>CASTAGNA E MIRTO</v>
       </c>
       <c r="B11" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C11" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CIOCCOLATO CRUDO DEL PERU'</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="B12" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C12" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>CIOCCOLATO E ARANCIA</v>
+        <v>CIOCCOLATO AL LATTE gelato</v>
       </c>
       <c r="B13" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C13" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CIOCCOLATO KENTUCKY</v>
+        <v>CIOCCOLATO CRUDO DEL PERU'</v>
       </c>
       <c r="B14" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C14" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CIOCCOLATO VENEZUELA</v>
+        <v>CIOCCOLATO E ARANCIA</v>
       </c>
       <c r="B15" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C15" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CIOCCOLATO ROSEMARY</v>
+        <v>CIOCCOLATO KENTUCKY</v>
       </c>
       <c r="B16" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C16" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>COCCO CREMA</v>
+        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
       </c>
       <c r="B17" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C17" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>CREMA  PASTICCIERA PARISI</v>
+        <v>CIOCCOLATO VENEZUELA</v>
       </c>
       <c r="B18" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C18" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
+        <v>CIOCCOLATO ROSEMARY</v>
       </c>
       <c r="B19" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C19" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CREMA CANNELLA</v>
+        <v>CREMA  PASTICCIERA PARISI</v>
       </c>
       <c r="B20" t="str">
         <v>Da Ordinare</v>
@@ -621,7 +621,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>CREMA FRAGOLE E MANDORLE</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="B21" t="str">
         <v>Da Ordinare</v>
@@ -632,7 +632,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CREMA VANIGLIA</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="B22" t="str">
         <v>Da Ordinare</v>
@@ -643,51 +643,51 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="B23" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C23" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>FIORDILATTE</v>
+        <v>CREMA FRAGOLE E MANDORLE</v>
       </c>
       <c r="B24" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C24" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>FRAGOLA</v>
+        <v>CREMA VANIGLIA</v>
       </c>
       <c r="B25" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C25" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>GIANDUIA</v>
+        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
       </c>
       <c r="B26" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C26" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>ESTASI</v>
       </c>
       <c r="B27" t="str">
         <v>Da Ordinare</v>
@@ -698,18 +698,18 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>LATTE MENTA E CIOCCOLATO</v>
+        <v>FIORDILATTE</v>
       </c>
       <c r="B28" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C28" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>LIMONE</v>
+        <v>FRAGOLA</v>
       </c>
       <c r="B29" t="str">
         <v>Da Ordinare</v>
@@ -720,29 +720,29 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>LIQUIRIZIA</v>
+        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
       </c>
       <c r="B30" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C30" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>GIANDUIA</v>
       </c>
       <c r="B31" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C31" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B32" t="str">
         <v>Da Ordinare</v>
@@ -753,40 +753,40 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>LATTE MENTA E CIOCCOLATO</v>
       </c>
       <c r="B33" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C33" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="B34" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C34" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>MELONE</v>
+        <v>LIMONE</v>
       </c>
       <c r="B35" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C35" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>MIRTILLO</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B36" t="str">
         <v>Da Ordinare</v>
@@ -797,18 +797,18 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>MOJITO ALLA AMARENA</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B37" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C37" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>MORA</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B38" t="str">
         <v>Da Ordinare</v>
@@ -819,29 +819,29 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="B39" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C39" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>NOCCIOLA</v>
+        <v>MANDORLA TOSTATA</v>
       </c>
       <c r="B40" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C40" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>NOCCIOLA AL FRUTTOSIO</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="B41" t="str">
         <v>Da Ordinare</v>
@@ -852,62 +852,62 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>MELA MANDORLA E CANNELLA</v>
       </c>
       <c r="B42" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C42" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>PERA</v>
+        <v>MELONE</v>
       </c>
       <c r="B43" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C43" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>PERE BELLE HELENE</v>
+        <v>MOJITO ALLA AMARENA</v>
       </c>
       <c r="B44" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C44" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>MORA</v>
       </c>
       <c r="B45" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C45" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B46" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C46" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>PUNCH PARADISE</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B47" t="str">
         <v>Da Ordinare</v>
@@ -918,7 +918,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>NOCCIOLA AL FRUTTOSIO</v>
       </c>
       <c r="B48" t="str">
         <v>Da Ordinare</v>
@@ -929,18 +929,18 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
       </c>
       <c r="B49" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C49" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>SEADAS</v>
+        <v>PAPAYA</v>
       </c>
       <c r="B50" t="str">
         <v>Da Ordinare</v>
@@ -951,51 +951,51 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>STRACCIATELLA</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="B51" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C51" t="str">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>TIRAMISU'</v>
+        <v>PERA</v>
       </c>
       <c r="B52" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C52" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>UVA E NOCI</v>
+        <v>PERE BELLE HELENE</v>
       </c>
       <c r="B53" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C53" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="B54" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C54" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>PENSIERO</v>
+        <v>POLLICINA</v>
       </c>
       <c r="B55" t="str">
         <v>Da Ordinare</v>
@@ -1006,18 +1006,18 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>SACRIPANTE</v>
+        <v>PUNCH PARADISE</v>
       </c>
       <c r="B56" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C56" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>BUONGIORNO AMORE</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B57" t="str">
         <v>Da Ordinare</v>
@@ -1028,29 +1028,29 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="B58" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C58" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B59" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C59" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>AVOCADO LIME E VINO BIANCO</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B60" t="str">
         <v>Da Ordinare</v>
@@ -1061,7 +1061,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>MONT BLANC</v>
+        <v>CIOCCOLATO WASABI</v>
       </c>
       <c r="B61" t="str">
         <v>Da Ordinare</v>
@@ -1072,7 +1072,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>COCCO</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
       </c>
       <c r="B62" t="str">
         <v>Da Ordinare</v>
@@ -1083,51 +1083,51 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B63" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C63" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+        <v>BUONGIORNO AMORE</v>
       </c>
       <c r="B64" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C64" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B65" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C65" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>SACHER TORTE</v>
+        <v>CARROT CAKE</v>
       </c>
       <c r="B66" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C66" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>CASTAGNA AL WHISKY</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="B67" t="str">
         <v>Da Ordinare</v>
@@ -1138,18 +1138,18 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+        <v>FIOR DI CIOCCOLATO</v>
       </c>
       <c r="B68" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C68" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+        <v>ROSA KARKADE E ARANCIA</v>
       </c>
       <c r="B69" t="str">
         <v>Da Ordinare</v>
@@ -1160,62 +1160,62 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>ZABAIONE NEW</v>
+        <v>AVOCADO LIME E VINO BIANCO</v>
       </c>
       <c r="B70" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C70" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>ANGURIA</v>
+        <v>MONT BLANC</v>
       </c>
       <c r="B71" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C71" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>ARACHIDI COCCO E CIOCCOLATO</v>
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
       </c>
       <c r="B72" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C72" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>CAFFE'</v>
+        <v>EVERGREEN  BRONTE VEGAN</v>
       </c>
       <c r="B73" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C73" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>CASTAGNA E MIRTO</v>
+        <v>SACHER TORTE</v>
       </c>
       <c r="B74" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C74" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>CIOCCOLATO AL PIMENTO</v>
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
       </c>
       <c r="B75" t="str">
         <v>Da Ordinare</v>
@@ -1226,128 +1226,128 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
+        <v>CREMA MASCARPONE</v>
       </c>
       <c r="B76" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C76" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
       </c>
       <c r="B77" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C77" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>CREMA AGNESE</v>
+        <v>COCONUT RICE CAKE</v>
       </c>
       <c r="B78" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C78" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>ESTASI</v>
+        <v>PISTACCHIO LARNAKA , CIPRO</v>
       </c>
       <c r="B79" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C79" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
+        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
       </c>
       <c r="B80" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C80" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>MANDARINO</v>
+        <v>ZABAIONE NEW</v>
       </c>
       <c r="B81" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C81" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>MELA MANDORLA E CANNELLA</v>
+        <v>BAKLAVA</v>
       </c>
       <c r="B82" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C82" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>PASSION FRUIT</v>
+        <v>CIOCCOLATO AL PIMENTO</v>
       </c>
       <c r="B83" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C83" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>POLLICINA</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="B84" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C84" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>RICOTTA, MIELE E COCCO</v>
+        <v>COCCO CREMA</v>
       </c>
       <c r="B85" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C85" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>CIOCCOLATO WASABI</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="B86" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C86" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>YOGURT</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="B87" t="str">
         <v>Da Ordinare</v>
@@ -1358,7 +1358,7 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>CARROT CAKE</v>
+        <v>SEADAS</v>
       </c>
       <c r="B88" t="str">
         <v>Da Ordinare</v>
@@ -1369,40 +1369,40 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>FIOR DI CIOCCOLATO</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B89" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C89" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>ROSA KARKADE E ARANCIA</v>
+        <v>YOGURT</v>
       </c>
       <c r="B90" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C90" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>PASTIERA NAPOLETANA</v>
+        <v>PENSIERO</v>
       </c>
       <c r="B91" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C91" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
+        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
       </c>
       <c r="B92" t="str">
         <v>Da Ordinare</v>
@@ -1413,18 +1413,18 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>CREMA MASCARPONE</v>
+        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
       </c>
       <c r="B93" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C93" t="str">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>COCONUT RICE CAKE</v>
+        <v>TORTA CAPRESE</v>
       </c>
       <c r="B94" t="str">
         <v>Da Ordinare</v>
@@ -1435,18 +1435,18 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>PISTACCHIO LARNAKA , CIPRO</v>
+        <v>MANDARINO</v>
       </c>
       <c r="B95" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C95" t="str">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>ALBICOCCA</v>
+        <v>RICOTTA, MIELE E COCCO</v>
       </c>
       <c r="B96" t="str">
         <v>Da Ordinare</v>
@@ -1457,40 +1457,40 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>LEMON CURD</v>
+        <v>PASTIERA NAPOLETANA</v>
       </c>
       <c r="B97" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C97" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>PAPAYA</v>
+        <v>ALBICOCCA</v>
       </c>
       <c r="B98" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C98" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>CIOCCOLATA CALDA FONDENTE</v>
+        <v>GIANDUIA VARIEGATA</v>
       </c>
       <c r="B99" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C99" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>ZABAIONE AL SAKE'</v>
+        <v>CIOCCOLATA CALDA FONDENTE</v>
       </c>
       <c r="B100" t="str">
         <v>Da Ordinare</v>
@@ -1501,7 +1501,7 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>TORTA CAPRESE</v>
+        <v>ZABAIONE AL SAKE'</v>
       </c>
       <c r="B101" t="str">
         <v>Da Ordinare</v>
@@ -1512,40 +1512,40 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
+        <v>CACHI</v>
       </c>
       <c r="B102" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C102" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>CACHI</v>
+        <v>CIOCCOLATO</v>
       </c>
       <c r="B103" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C103" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>CIOCCOLATO</v>
+        <v>CASTAGNA AL WHISKY</v>
       </c>
       <c r="B104" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C104" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>MANDORLA TOSTATA</v>
+        <v>ZABAIONE GELATO</v>
       </c>
       <c r="B105" t="str">
         <v>Da Ordinare</v>
@@ -1556,18 +1556,18 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
       </c>
       <c r="B106" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C106" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
+        <v>SEMIFREDDO  TIRAMISU</v>
       </c>
       <c r="B107" t="str">
         <v>Da Ordinare</v>
@@ -1578,7 +1578,7 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>SEMIFREDDO  TIRAMISU</v>
+        <v>FICHI</v>
       </c>
       <c r="B108" t="str">
         <v>Da Ordinare</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>FICHI</v>
+        <v>UVA FRAGOLA E ZENZERO</v>
       </c>
       <c r="B109" t="str">
         <v>Da Ordinare</v>
@@ -1600,29 +1600,18 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>UVA FRAGOLA E ZENZERO</v>
+        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
       </c>
       <c r="B110" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C110" t="str">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="str">
-        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
-      </c>
-      <c r="B111" t="str">
-        <v>Da Ordinare</v>
-      </c>
-      <c r="C111" t="str">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C111"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C110"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly SHOCAPP data 2026-04-26
</commit_message>
<xml_diff>
--- a/output/shocapp_da_ordinare.xlsx
+++ b/output/shocapp_da_ordinare.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C109"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,7 +429,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C3" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -451,7 +451,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C5" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -462,7 +462,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C6" t="str">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -473,7 +473,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C7" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -484,7 +484,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C8" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -495,7 +495,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C9" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -506,7 +506,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C10" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -528,7 +528,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C12" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -539,12 +539,12 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C13" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CIOCCOLATO CRUDO DEL PERU'</v>
+        <v>CIOCCOLATO AL PIMENTO</v>
       </c>
       <c r="B14" t="str">
         <v>Da Ordinare</v>
@@ -555,18 +555,18 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CIOCCOLATO E ARANCIA</v>
+        <v>CIOCCOLATO CRUDO DEL PERU'</v>
       </c>
       <c r="B15" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C15" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CIOCCOLATO KENTUCKY</v>
+        <v>CIOCCOLATO E ARANCIA</v>
       </c>
       <c r="B16" t="str">
         <v>Da Ordinare</v>
@@ -577,7 +577,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
+        <v>CIOCCOLATO KENTUCKY</v>
       </c>
       <c r="B17" t="str">
         <v>Da Ordinare</v>
@@ -588,29 +588,29 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>CIOCCOLATO VENEZUELA</v>
+        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
       </c>
       <c r="B18" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C18" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CIOCCOLATO ROSEMARY</v>
+        <v>CIOCCOLATO VENEZUELA</v>
       </c>
       <c r="B19" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C19" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CREMA  PASTICCIERA PARISI</v>
+        <v>CIOCCOLATO ROSEMARY</v>
       </c>
       <c r="B20" t="str">
         <v>Da Ordinare</v>
@@ -621,35 +621,35 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>CREMA AGNESE</v>
+        <v>COCCO CREMA</v>
       </c>
       <c r="B21" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C21" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
+        <v>CREMA  PASTICCIERA PARISI</v>
       </c>
       <c r="B22" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C22" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>CREMA CANNELLA</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="B23" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C23" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -660,7 +660,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C24" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -682,7 +682,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C26" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -704,7 +704,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C28" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
@@ -715,7 +715,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C29" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -726,56 +726,56 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C30" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>GIANDUIA</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B31" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C31" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>LATTE MENTA E CIOCCOLATO</v>
       </c>
       <c r="B32" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C32" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>LATTE MENTA E CIOCCOLATO</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="B33" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C33" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>LEMON CURD</v>
+        <v>LIMONE</v>
       </c>
       <c r="B34" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C34" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>LIMONE</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B35" t="str">
         <v>Da Ordinare</v>
@@ -786,29 +786,29 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>LIQUIRIZIA</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B36" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C36" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B37" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C37" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="B38" t="str">
         <v>Da Ordinare</v>
@@ -819,18 +819,18 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="B39" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C39" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>MANDORLA TOSTATA</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="B40" t="str">
         <v>Da Ordinare</v>
@@ -841,7 +841,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>MORA</v>
       </c>
       <c r="B41" t="str">
         <v>Da Ordinare</v>
@@ -852,7 +852,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>MELA MANDORLA E CANNELLA</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B42" t="str">
         <v>Da Ordinare</v>
@@ -863,18 +863,18 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>MELONE</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B43" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C43" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>MOJITO ALLA AMARENA</v>
+        <v>NOCCIOLA AL FRUTTOSIO</v>
       </c>
       <c r="B44" t="str">
         <v>Da Ordinare</v>
@@ -885,7 +885,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>MORA</v>
+        <v>PAPAYA</v>
       </c>
       <c r="B45" t="str">
         <v>Da Ordinare</v>
@@ -896,18 +896,18 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>PERA</v>
       </c>
       <c r="B46" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C46" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>NOCCIOLA</v>
+        <v>PERE BELLE HELENE</v>
       </c>
       <c r="B47" t="str">
         <v>Da Ordinare</v>
@@ -918,7 +918,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>NOCCIOLA AL FRUTTOSIO</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="B48" t="str">
         <v>Da Ordinare</v>
@@ -929,7 +929,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="B49" t="str">
         <v>Da Ordinare</v>
@@ -940,18 +940,18 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>PAPAYA</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B50" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C50" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>PASSION FRUIT</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="B51" t="str">
         <v>Da Ordinare</v>
@@ -962,40 +962,40 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>PERA</v>
+        <v>SEADAS</v>
       </c>
       <c r="B52" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C52" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>PERE BELLE HELENE</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B53" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C53" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B54" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C54" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>POLLICINA</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B55" t="str">
         <v>Da Ordinare</v>
@@ -1006,7 +1006,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>PUNCH PARADISE</v>
+        <v>CIOCCOLATO WASABI</v>
       </c>
       <c r="B56" t="str">
         <v>Da Ordinare</v>
@@ -1017,62 +1017,62 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>YOGURT</v>
       </c>
       <c r="B57" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C57" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>PENSIERO</v>
       </c>
       <c r="B58" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C58" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>STRACCIATELLA</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B59" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C59" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>UVA E NOCI</v>
+        <v>BUONGIORNO AMORE</v>
       </c>
       <c r="B60" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C60" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>CIOCCOLATO WASABI</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B61" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C61" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+        <v>CARROT CAKE</v>
       </c>
       <c r="B62" t="str">
         <v>Da Ordinare</v>
@@ -1083,18 +1083,18 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>SACRIPANTE</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="B63" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C63" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>BUONGIORNO AMORE</v>
+        <v>ROSA KARKADE E ARANCIA</v>
       </c>
       <c r="B64" t="str">
         <v>Da Ordinare</v>
@@ -1105,18 +1105,18 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>AVOCADO LIME E VINO BIANCO</v>
       </c>
       <c r="B65" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C65" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>CARROT CAKE</v>
+        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
       </c>
       <c r="B66" t="str">
         <v>Da Ordinare</v>
@@ -1127,7 +1127,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>SACHER TORTE</v>
       </c>
       <c r="B67" t="str">
         <v>Da Ordinare</v>
@@ -1138,29 +1138,29 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>FIOR DI CIOCCOLATO</v>
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
       </c>
       <c r="B68" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C68" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>ROSA KARKADE E ARANCIA</v>
+        <v>CREMA MASCARPONE</v>
       </c>
       <c r="B69" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C69" t="str">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>AVOCADO LIME E VINO BIANCO</v>
+        <v>COCONUT RICE CAKE</v>
       </c>
       <c r="B70" t="str">
         <v>Da Ordinare</v>
@@ -1171,18 +1171,18 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>MONT BLANC</v>
+        <v>PISTACCHIO LARNAKA , CIPRO</v>
       </c>
       <c r="B71" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C71" t="str">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
       </c>
       <c r="B72" t="str">
         <v>Da Ordinare</v>
@@ -1193,18 +1193,18 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
+        <v>ZABAIONE NEW</v>
       </c>
       <c r="B73" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C73" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>SACHER TORTE</v>
+        <v>FASHIONED SPRITZ</v>
       </c>
       <c r="B74" t="str">
         <v>Da Ordinare</v>
@@ -1215,84 +1215,84 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+        <v>GIANDUIA VARIEGATA</v>
       </c>
       <c r="B75" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C75" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>CREMA MASCARPONE</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="B76" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C76" t="str">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="B77" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C77" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>COCONUT RICE CAKE</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="B78" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C78" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>PISTACCHIO LARNAKA , CIPRO</v>
+        <v>GIANDUIA</v>
       </c>
       <c r="B79" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C79" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
+        <v>MANDORLA TOSTATA</v>
       </c>
       <c r="B80" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C80" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>ZABAIONE NEW</v>
+        <v>MELA MANDORLA E CANNELLA</v>
       </c>
       <c r="B81" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C81" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>BAKLAVA</v>
+        <v>MELONE</v>
       </c>
       <c r="B82" t="str">
         <v>Da Ordinare</v>
@@ -1303,40 +1303,40 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>CIOCCOLATO AL PIMENTO</v>
+        <v>MOJITO ALLA AMARENA</v>
       </c>
       <c r="B83" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C83" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
       </c>
       <c r="B84" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C84" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>COCCO CREMA</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="B85" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C85" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>MIRTILLO</v>
+        <v>POLLICINA</v>
       </c>
       <c r="B86" t="str">
         <v>Da Ordinare</v>
@@ -1347,18 +1347,18 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>PUNCH PARADISE</v>
       </c>
       <c r="B87" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C87" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>SEADAS</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
       </c>
       <c r="B88" t="str">
         <v>Da Ordinare</v>
@@ -1369,35 +1369,35 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>TIRAMISU'</v>
+        <v>FIOR DI CIOCCOLATO</v>
       </c>
       <c r="B89" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C89" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>YOGURT</v>
+        <v>MONT BLANC</v>
       </c>
       <c r="B90" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C90" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>PENSIERO</v>
+        <v>COCCO</v>
       </c>
       <c r="B91" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C91" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92">
@@ -1413,29 +1413,29 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
       </c>
       <c r="B93" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C93" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>TORTA CAPRESE</v>
+        <v>EVERGREEN  BRONTE VEGAN</v>
       </c>
       <c r="B94" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C94" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>MANDARINO</v>
+        <v>CASTAGNA AL WHISKY</v>
       </c>
       <c r="B95" t="str">
         <v>Da Ordinare</v>
@@ -1446,29 +1446,29 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>RICOTTA, MIELE E COCCO</v>
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
       </c>
       <c r="B96" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C96" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>PASTIERA NAPOLETANA</v>
+        <v>BAKLAVA</v>
       </c>
       <c r="B97" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C97" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>ALBICOCCA</v>
+        <v>TORTA CAPRESE</v>
       </c>
       <c r="B98" t="str">
         <v>Da Ordinare</v>
@@ -1479,18 +1479,18 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>GIANDUIA VARIEGATA</v>
+        <v>MANDARINO</v>
       </c>
       <c r="B99" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C99" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>CIOCCOLATA CALDA FONDENTE</v>
+        <v>RICOTTA, MIELE E COCCO</v>
       </c>
       <c r="B100" t="str">
         <v>Da Ordinare</v>
@@ -1501,18 +1501,18 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>ZABAIONE AL SAKE'</v>
+        <v>PASTIERA NAPOLETANA</v>
       </c>
       <c r="B101" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C101" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>CACHI</v>
+        <v>ALBICOCCA</v>
       </c>
       <c r="B102" t="str">
         <v>Da Ordinare</v>
@@ -1523,18 +1523,18 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>CIOCCOLATO</v>
+        <v>CIOCCOLATA CALDA FONDENTE</v>
       </c>
       <c r="B103" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C103" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>CASTAGNA AL WHISKY</v>
+        <v>ZABAIONE AL SAKE'</v>
       </c>
       <c r="B104" t="str">
         <v>Da Ordinare</v>
@@ -1545,7 +1545,7 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>CACHI</v>
       </c>
       <c r="B105" t="str">
         <v>Da Ordinare</v>
@@ -1556,18 +1556,18 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
+        <v>CIOCCOLATO</v>
       </c>
       <c r="B106" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C106" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>SEMIFREDDO  TIRAMISU</v>
+        <v>ZABAIONE GELATO</v>
       </c>
       <c r="B107" t="str">
         <v>Da Ordinare</v>
@@ -1578,7 +1578,7 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>FICHI</v>
+        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
       </c>
       <c r="B108" t="str">
         <v>Da Ordinare</v>
@@ -1589,29 +1589,18 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>UVA FRAGOLA E ZENZERO</v>
+        <v>SEMIFREDDO  TIRAMISU</v>
       </c>
       <c r="B109" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C109" t="str">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="str">
-        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
-      </c>
-      <c r="B110" t="str">
-        <v>Da Ordinare</v>
-      </c>
-      <c r="C110" t="str">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C110"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C109"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly SHOCAPP data 2026-05-03
</commit_message>
<xml_diff>
--- a/output/shocapp_da_ordinare.xlsx
+++ b/output/shocapp_da_ordinare.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C112"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,117 +412,117 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>AMARENA</v>
+        <v>ANANAS E ZENZERO</v>
       </c>
       <c r="B2" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C2" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ANANAS E ZENZERO</v>
+        <v>GIANDUIA VARIEGATA</v>
       </c>
       <c r="B3" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C3" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ANGURIA</v>
+        <v>BACIO DEL PRINCIPE</v>
       </c>
       <c r="B4" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C4" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ARACHIDI COCCO E CIOCCOLATO</v>
+        <v>BANANA E LIME</v>
       </c>
       <c r="B5" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C5" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BACIO DEL PRINCIPE</v>
+        <v>BASILICO NOCI E MIELE</v>
       </c>
       <c r="B6" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C6" t="str">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>BANANA E LIME</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="B7" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C7" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>BASILICO NOCI E MIELE</v>
+        <v>CAFFE'</v>
       </c>
       <c r="B8" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C8" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>BIANCANEVE</v>
+        <v>CASTAGNA E MIRTO</v>
       </c>
       <c r="B9" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C9" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>CAFFE'</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="B10" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C10" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>CASTAGNA E MIRTO</v>
+        <v>CIOCCOLATO AL LATTE gelato</v>
       </c>
       <c r="B11" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C11" t="str">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>CIOCCOLATO AL PIMENTO</v>
       </c>
       <c r="B12" t="str">
         <v>Da Ordinare</v>
@@ -533,29 +533,29 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>CIOCCOLATO AL LATTE gelato</v>
+        <v>CIOCCOLATO CRUDO DEL PERU'</v>
       </c>
       <c r="B13" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C13" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CIOCCOLATO AL PIMENTO</v>
+        <v>CIOCCOLATO KENTUCKY</v>
       </c>
       <c r="B14" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C14" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CIOCCOLATO CRUDO DEL PERU'</v>
+        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
       </c>
       <c r="B15" t="str">
         <v>Da Ordinare</v>
@@ -566,29 +566,29 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CIOCCOLATO E ARANCIA</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="B16" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C16" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>CIOCCOLATO KENTUCKY</v>
+        <v>CIOCCOLATO VENEZUELA</v>
       </c>
       <c r="B17" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C17" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
+        <v>COCCO CREMA</v>
       </c>
       <c r="B18" t="str">
         <v>Da Ordinare</v>
@@ -599,18 +599,18 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CIOCCOLATO VENEZUELA</v>
+        <v>CREMA  PASTICCIERA PARISI</v>
       </c>
       <c r="B19" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C19" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CIOCCOLATO ROSEMARY</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="B20" t="str">
         <v>Da Ordinare</v>
@@ -621,73 +621,73 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>COCCO CREMA</v>
+        <v>CREMA FRAGOLE E MANDORLE</v>
       </c>
       <c r="B21" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C21" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CREMA  PASTICCIERA PARISI</v>
+        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
       </c>
       <c r="B22" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C22" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
+        <v>ESTASI</v>
       </c>
       <c r="B23" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C23" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>CREMA FRAGOLE E MANDORLE</v>
+        <v>FIORDILATTE</v>
       </c>
       <c r="B24" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C24" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>CREMA VANIGLIA</v>
+        <v>FRAGOLA</v>
       </c>
       <c r="B25" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C25" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
+        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
       </c>
       <c r="B26" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C26" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ESTASI</v>
+        <v>GIANDUIA</v>
       </c>
       <c r="B27" t="str">
         <v>Da Ordinare</v>
@@ -698,40 +698,40 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>FIORDILATTE</v>
+        <v>LATTE MENTA E CIOCCOLATO</v>
       </c>
       <c r="B28" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C28" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>FRAGOLA</v>
+        <v>LIMONE</v>
       </c>
       <c r="B29" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C29" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B30" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C30" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B31" t="str">
         <v>Da Ordinare</v>
@@ -742,18 +742,18 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>LATTE MENTA E CIOCCOLATO</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B32" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C32" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>LEMON CURD</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="B33" t="str">
         <v>Da Ordinare</v>
@@ -764,73 +764,73 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>LIMONE</v>
+        <v>MELA MANDORLA E CANNELLA</v>
       </c>
       <c r="B34" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C34" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>LIQUIRIZIA</v>
+        <v>MELONE</v>
       </c>
       <c r="B35" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C35" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="B36" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C36" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B37" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C37" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B38" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C38" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>NOCCIOLA AL FRUTTOSIO</v>
       </c>
       <c r="B39" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C39" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>MIRTILLO</v>
+        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
       </c>
       <c r="B40" t="str">
         <v>Da Ordinare</v>
@@ -841,7 +841,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>MORA</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="B41" t="str">
         <v>Da Ordinare</v>
@@ -852,7 +852,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>PERA</v>
       </c>
       <c r="B42" t="str">
         <v>Da Ordinare</v>
@@ -863,18 +863,18 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>NOCCIOLA</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="B43" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C43" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>NOCCIOLA AL FRUTTOSIO</v>
+        <v>POLLICINA</v>
       </c>
       <c r="B44" t="str">
         <v>Da Ordinare</v>
@@ -885,51 +885,51 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>PAPAYA</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B45" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C45" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>PERA</v>
+        <v>RICOTTA, MIELE E COCCO</v>
       </c>
       <c r="B46" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C46" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>PERE BELLE HELENE</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="B47" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C47" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B48" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C48" t="str">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B49" t="str">
         <v>Da Ordinare</v>
@@ -940,7 +940,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>CIOCCOLATO WASABI</v>
       </c>
       <c r="B50" t="str">
         <v>Da Ordinare</v>
@@ -951,73 +951,73 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>YOGURT</v>
       </c>
       <c r="B51" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C51" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>SEADAS</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
       </c>
       <c r="B52" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C52" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>STRACCIATELLA</v>
+        <v>PENSIERO</v>
       </c>
       <c r="B53" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C53" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>TIRAMISU'</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B54" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C54" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>UVA E NOCI</v>
+        <v>BUONGIORNO AMORE</v>
       </c>
       <c r="B55" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C55" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>CIOCCOLATO WASABI</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B56" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C56" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>YOGURT</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="B57" t="str">
         <v>Da Ordinare</v>
@@ -1028,29 +1028,29 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>PENSIERO</v>
+        <v>AVOCADO LIME E VINO BIANCO</v>
       </c>
       <c r="B58" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C58" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>SACRIPANTE</v>
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
       </c>
       <c r="B59" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C59" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>BUONGIORNO AMORE</v>
+        <v>EVERGREEN  BRONTE VEGAN</v>
       </c>
       <c r="B60" t="str">
         <v>Da Ordinare</v>
@@ -1061,7 +1061,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>SACHER TORTE</v>
       </c>
       <c r="B61" t="str">
         <v>Da Ordinare</v>
@@ -1072,7 +1072,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>CARROT CAKE</v>
+        <v>FAVE FRESCHE &amp; PECORINO</v>
       </c>
       <c r="B62" t="str">
         <v>Da Ordinare</v>
@@ -1083,7 +1083,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>LIMONE &amp; BASILICO</v>
       </c>
       <c r="B63" t="str">
         <v>Da Ordinare</v>
@@ -1094,40 +1094,40 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>ROSA KARKADE E ARANCIA</v>
+        <v>CREMA MASCARPONE</v>
       </c>
       <c r="B64" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C64" t="str">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>AVOCADO LIME E VINO BIANCO</v>
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
       </c>
       <c r="B65" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C65" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
+        <v>COCONUT RICE CAKE</v>
       </c>
       <c r="B66" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C66" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>SACHER TORTE</v>
+        <v>PISTACCHIO LARNAKA , CIPRO</v>
       </c>
       <c r="B67" t="str">
         <v>Da Ordinare</v>
@@ -1138,106 +1138,106 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
       </c>
       <c r="B68" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C68" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>CREMA MASCARPONE</v>
+        <v>ZABAIONE NEW</v>
       </c>
       <c r="B69" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C69" t="str">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>COCONUT RICE CAKE</v>
+        <v>STRAWBERRY FIELD FOREVER</v>
       </c>
       <c r="B70" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C70" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>PISTACCHIO LARNAKA , CIPRO</v>
+        <v>AMARENA</v>
       </c>
       <c r="B71" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C71" t="str">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
+        <v>ANGURIA</v>
       </c>
       <c r="B72" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C72" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>ZABAIONE NEW</v>
+        <v>ARACHIDI COCCO E CIOCCOLATO</v>
       </c>
       <c r="B73" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C73" t="str">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>FASHIONED SPRITZ</v>
+        <v>CIOCCOLATO E ARANCIA</v>
       </c>
       <c r="B74" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C74" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>GIANDUIA VARIEGATA</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="B75" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C75" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="B76" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C76" t="str">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>CREMA AGNESE</v>
+        <v>CREMA VANIGLIA</v>
       </c>
       <c r="B77" t="str">
         <v>Da Ordinare</v>
@@ -1248,29 +1248,29 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>CREMA CANNELLA</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B78" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C78" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>GIANDUIA</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="B79" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C79" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>MANDORLA TOSTATA</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="B80" t="str">
         <v>Da Ordinare</v>
@@ -1281,18 +1281,18 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>MELA MANDORLA E CANNELLA</v>
+        <v>MANDORLA TOSTATA</v>
       </c>
       <c r="B81" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C81" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>MELONE</v>
+        <v>MORA</v>
       </c>
       <c r="B82" t="str">
         <v>Da Ordinare</v>
@@ -1303,40 +1303,40 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>MOJITO ALLA AMARENA</v>
+        <v>PAPAYA</v>
       </c>
       <c r="B83" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C83" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>PERE BELLE HELENE</v>
       </c>
       <c r="B84" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C84" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>PASSION FRUIT</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="B85" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C85" t="str">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>POLLICINA</v>
+        <v>PUNCH PARADISE</v>
       </c>
       <c r="B86" t="str">
         <v>Da Ordinare</v>
@@ -1347,7 +1347,7 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>PUNCH PARADISE</v>
+        <v>SEADAS</v>
       </c>
       <c r="B87" t="str">
         <v>Da Ordinare</v>
@@ -1358,7 +1358,7 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B88" t="str">
         <v>Da Ordinare</v>
@@ -1369,7 +1369,7 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>FIOR DI CIOCCOLATO</v>
+        <v>CARROT CAKE</v>
       </c>
       <c r="B89" t="str">
         <v>Da Ordinare</v>
@@ -1380,7 +1380,7 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>MONT BLANC</v>
+        <v>ROSA KARKADE E ARANCIA</v>
       </c>
       <c r="B90" t="str">
         <v>Da Ordinare</v>
@@ -1391,7 +1391,7 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>COCCO</v>
+        <v>SUSHI VEGANO</v>
       </c>
       <c r="B91" t="str">
         <v>Da Ordinare</v>
@@ -1402,7 +1402,7 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
+        <v>CIOCCOLATO AL WHISKY</v>
       </c>
       <c r="B92" t="str">
         <v>Da Ordinare</v>
@@ -1413,18 +1413,18 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+        <v>TORTA CAPRESE</v>
       </c>
       <c r="B93" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C93" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
       </c>
       <c r="B94" t="str">
         <v>Da Ordinare</v>
@@ -1435,40 +1435,40 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>CASTAGNA AL WHISKY</v>
+        <v>MOJITO ALLA AMARENA</v>
       </c>
       <c r="B95" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C95" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+        <v>FIOR DI CIOCCOLATO</v>
       </c>
       <c r="B96" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C96" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>BAKLAVA</v>
+        <v>MONT BLANC</v>
       </c>
       <c r="B97" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C97" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>TORTA CAPRESE</v>
+        <v>COCCO</v>
       </c>
       <c r="B98" t="str">
         <v>Da Ordinare</v>
@@ -1479,7 +1479,7 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>MANDARINO</v>
+        <v>CASTAGNA AL WHISKY</v>
       </c>
       <c r="B99" t="str">
         <v>Da Ordinare</v>
@@ -1490,7 +1490,7 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>RICOTTA, MIELE E COCCO</v>
+        <v>BAKLAVA</v>
       </c>
       <c r="B100" t="str">
         <v>Da Ordinare</v>
@@ -1501,18 +1501,18 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>PASTIERA NAPOLETANA</v>
+        <v>CIOCCOLATO ROSEMARY</v>
       </c>
       <c r="B101" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C101" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>ALBICOCCA</v>
+        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
       </c>
       <c r="B102" t="str">
         <v>Da Ordinare</v>
@@ -1523,7 +1523,7 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>CIOCCOLATA CALDA FONDENTE</v>
+        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
       </c>
       <c r="B103" t="str">
         <v>Da Ordinare</v>
@@ -1534,7 +1534,7 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>ZABAIONE AL SAKE'</v>
+        <v>MANDARINO</v>
       </c>
       <c r="B104" t="str">
         <v>Da Ordinare</v>
@@ -1545,29 +1545,29 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>CACHI</v>
+        <v>PASTIERA NAPOLETANA</v>
       </c>
       <c r="B105" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C105" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>CIOCCOLATO</v>
+        <v>ALBICOCCA</v>
       </c>
       <c r="B106" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C106" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>CIOCCOLATA CALDA FONDENTE</v>
       </c>
       <c r="B107" t="str">
         <v>Da Ordinare</v>
@@ -1578,7 +1578,7 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
+        <v>ZABAIONE AL SAKE'</v>
       </c>
       <c r="B108" t="str">
         <v>Da Ordinare</v>
@@ -1589,18 +1589,51 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>SEMIFREDDO  TIRAMISU</v>
+        <v>CACHI</v>
       </c>
       <c r="B109" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C109" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>CIOCCOLATO</v>
+      </c>
+      <c r="B110" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C110" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>ZABAIONE GELATO</v>
+      </c>
+      <c r="B111" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C111" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
+      </c>
+      <c r="B112" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C112" t="str">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C109"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C112"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly SHOCAPP data 2026-05-10
</commit_message>
<xml_diff>
--- a/output/shocapp_da_ordinare.xlsx
+++ b/output/shocapp_da_ordinare.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,73 +412,73 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ANANAS E ZENZERO</v>
+        <v>AMARENA</v>
       </c>
       <c r="B2" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C2" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>GIANDUIA VARIEGATA</v>
+        <v>ANANAS E ZENZERO</v>
       </c>
       <c r="B3" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C3" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>BACIO DEL PRINCIPE</v>
+        <v>ANGURIA</v>
       </c>
       <c r="B4" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C4" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>BANANA E LIME</v>
+        <v>ARACHIDI COCCO E CIOCCOLATO</v>
       </c>
       <c r="B5" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C5" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BASILICO NOCI E MIELE</v>
+        <v>GIANDUIA VARIEGATA</v>
       </c>
       <c r="B6" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C6" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>BIANCANEVE</v>
+        <v>BACIO DEL PRINCIPE</v>
       </c>
       <c r="B7" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C7" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>CAFFE'</v>
+        <v>BANANA E LIME</v>
       </c>
       <c r="B8" t="str">
         <v>Da Ordinare</v>
@@ -489,24 +489,24 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>CASTAGNA E MIRTO</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="B9" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C9" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>CAFFE'</v>
       </c>
       <c r="B10" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C10" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -517,7 +517,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C11" t="str">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -544,57 +544,57 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CIOCCOLATO KENTUCKY</v>
+        <v>CIOCCOLATO E ARANCIA</v>
       </c>
       <c r="B14" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C14" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
+        <v>CIOCCOLATO KENTUCKY</v>
       </c>
       <c r="B15" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C15" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
       </c>
       <c r="B16" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C16" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>CIOCCOLATO VENEZUELA</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="B17" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C17" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>COCCO CREMA</v>
+        <v>CIOCCOLATO VENEZUELA</v>
       </c>
       <c r="B18" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C18" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
@@ -610,7 +610,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CREMA AGNESE</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="B20" t="str">
         <v>Da Ordinare</v>
@@ -627,29 +627,29 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C21" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
+        <v>CREMA VANIGLIA</v>
       </c>
       <c r="B22" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C22" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ESTASI</v>
+        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
       </c>
       <c r="B23" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C23" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -660,7 +660,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C24" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -671,7 +671,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C25" t="str">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
@@ -682,12 +682,12 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C26" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>GIANDUIA</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B27" t="str">
         <v>Da Ordinare</v>
@@ -698,29 +698,29 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>LATTE MENTA E CIOCCOLATO</v>
+        <v>LIMONE</v>
       </c>
       <c r="B28" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C28" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>LIMONE</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B29" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C29" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>LIQUIRIZIA</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B30" t="str">
         <v>Da Ordinare</v>
@@ -731,7 +731,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B31" t="str">
         <v>Da Ordinare</v>
@@ -742,7 +742,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="B32" t="str">
         <v>Da Ordinare</v>
@@ -753,7 +753,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>MANDORLA TOSTATA</v>
       </c>
       <c r="B33" t="str">
         <v>Da Ordinare</v>
@@ -786,57 +786,57 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>MIRTILLO</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B36" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C36" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B37" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C37" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>NOCCIOLA</v>
+        <v>NOCCIOLA AL FRUTTOSIO</v>
       </c>
       <c r="B38" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C38" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>NOCCIOLA AL FRUTTOSIO</v>
+        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
       </c>
       <c r="B39" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C39" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>PAPAYA</v>
       </c>
       <c r="B40" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C40" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -874,29 +874,29 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>POLLICINA</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="B44" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C44" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>POLLICINA</v>
       </c>
       <c r="B45" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C45" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>RICOTTA, MIELE E COCCO</v>
+        <v>PUNCH PARADISE</v>
       </c>
       <c r="B46" t="str">
         <v>Da Ordinare</v>
@@ -918,29 +918,29 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>STRACCIATELLA</v>
+        <v>SEADAS</v>
       </c>
       <c r="B48" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C48" t="str">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>TIRAMISU'</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B49" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C49" t="str">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>CIOCCOLATO WASABI</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B50" t="str">
         <v>Da Ordinare</v>
@@ -951,18 +951,18 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>YOGURT</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B51" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C51" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+        <v>YOGURT</v>
       </c>
       <c r="B52" t="str">
         <v>Da Ordinare</v>
@@ -973,18 +973,18 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>PENSIERO</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
       </c>
       <c r="B53" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C53" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>SACRIPANTE</v>
+        <v>MELOGRANO WONDERFUL</v>
       </c>
       <c r="B54" t="str">
         <v>Da Ordinare</v>
@@ -995,117 +995,117 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>BUONGIORNO AMORE</v>
+        <v>PENSIERO</v>
       </c>
       <c r="B55" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C55" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B56" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C56" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>BUONGIORNO AMORE</v>
       </c>
       <c r="B57" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C57" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>AVOCADO LIME E VINO BIANCO</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B58" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C58" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+        <v>CARROT CAKE</v>
       </c>
       <c r="B59" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C59" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="B60" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C60" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>SACHER TORTE</v>
+        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
       </c>
       <c r="B61" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C61" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>FAVE FRESCHE &amp; PECORINO</v>
+        <v>ROSA KARKADE E ARANCIA</v>
       </c>
       <c r="B62" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C62" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>LIMONE &amp; BASILICO</v>
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
       </c>
       <c r="B63" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C63" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>CREMA MASCARPONE</v>
+        <v>EVERGREEN  BRONTE VEGAN</v>
       </c>
       <c r="B64" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C64" t="str">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+        <v>CASTAGNA AL WHISKY</v>
       </c>
       <c r="B65" t="str">
         <v>Da Ordinare</v>
@@ -1116,18 +1116,18 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>COCONUT RICE CAKE</v>
+        <v>FAVE FRESCHE &amp; PECORINO</v>
       </c>
       <c r="B66" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C66" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>PISTACCHIO LARNAKA , CIPRO</v>
+        <v>LIMONE &amp; BASILICO</v>
       </c>
       <c r="B67" t="str">
         <v>Da Ordinare</v>
@@ -1138,117 +1138,117 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
+        <v>CREMA MASCARPONE</v>
       </c>
       <c r="B68" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C68" t="str">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>ZABAIONE NEW</v>
+        <v>COCONUT RICE CAKE</v>
       </c>
       <c r="B69" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C69" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>STRAWBERRY FIELD FOREVER</v>
+        <v>PISTACCHIO LARNAKA , CIPRO</v>
       </c>
       <c r="B70" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C70" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>AMARENA</v>
+        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
       </c>
       <c r="B71" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C71" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>ANGURIA</v>
+        <v>BASILICO NOCI E MIELE</v>
       </c>
       <c r="B72" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C72" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>ARACHIDI COCCO E CIOCCOLATO</v>
+        <v>CASTAGNA E MIRTO</v>
       </c>
       <c r="B73" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C73" t="str">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>CIOCCOLATO E ARANCIA</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="B74" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C74" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
+        <v>CIOCCOLATO ROSEMARY</v>
       </c>
       <c r="B75" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C75" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>CREMA CANNELLA</v>
+        <v>COCCO CREMA</v>
       </c>
       <c r="B76" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C76" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>CREMA VANIGLIA</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="B77" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C77" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>ESTASI</v>
       </c>
       <c r="B78" t="str">
         <v>Da Ordinare</v>
@@ -1259,29 +1259,29 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>LEMON CURD</v>
+        <v>GIANDUIA</v>
       </c>
       <c r="B79" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C79" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>LATTE MENTA E CIOCCOLATO</v>
       </c>
       <c r="B80" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C80" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>MANDORLA TOSTATA</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="B81" t="str">
         <v>Da Ordinare</v>
@@ -1292,18 +1292,18 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>MORA</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="B82" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C82" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>PAPAYA</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="B83" t="str">
         <v>Da Ordinare</v>
@@ -1320,45 +1320,45 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C84" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B85" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C85" t="str">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>PUNCH PARADISE</v>
+        <v>RICOTTA, MIELE E COCCO</v>
       </c>
       <c r="B86" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C86" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>SEADAS</v>
+        <v>AVOCADO LIME E VINO BIANCO</v>
       </c>
       <c r="B87" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C87" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>UVA E NOCI</v>
+        <v>MONT BLANC</v>
       </c>
       <c r="B88" t="str">
         <v>Da Ordinare</v>
@@ -1369,18 +1369,18 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>CARROT CAKE</v>
+        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
       </c>
       <c r="B89" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C89" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>ROSA KARKADE E ARANCIA</v>
+        <v>SACHER TORTE</v>
       </c>
       <c r="B90" t="str">
         <v>Da Ordinare</v>
@@ -1391,62 +1391,62 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>SUSHI VEGANO</v>
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
       </c>
       <c r="B91" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C91" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>CIOCCOLATO AL WHISKY</v>
+        <v>ZABAIONE NEW</v>
       </c>
       <c r="B92" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C92" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>TORTA CAPRESE</v>
+        <v>STRAWBERRY FIELD FOREVER</v>
       </c>
       <c r="B93" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C93" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="B94" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C94" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>MOJITO ALLA AMARENA</v>
+        <v>MORA</v>
       </c>
       <c r="B95" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C95" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>FIOR DI CIOCCOLATO</v>
+        <v>SUSHI VEGANO</v>
       </c>
       <c r="B96" t="str">
         <v>Da Ordinare</v>
@@ -1457,18 +1457,18 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>MONT BLANC</v>
+        <v>CIOCCOLATO AL WHISKY</v>
       </c>
       <c r="B97" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C97" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>COCCO</v>
+        <v>TORTA CAPRESE</v>
       </c>
       <c r="B98" t="str">
         <v>Da Ordinare</v>
@@ -1479,18 +1479,18 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>CASTAGNA AL WHISKY</v>
+        <v>MOJITO ALLA AMARENA</v>
       </c>
       <c r="B99" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C99" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>BAKLAVA</v>
+        <v>FIOR DI CIOCCOLATO</v>
       </c>
       <c r="B100" t="str">
         <v>Da Ordinare</v>
@@ -1501,7 +1501,7 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>CIOCCOLATO ROSEMARY</v>
+        <v>COCCO</v>
       </c>
       <c r="B101" t="str">
         <v>Da Ordinare</v>
@@ -1512,18 +1512,18 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
       </c>
       <c r="B102" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C102" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
+        <v>BAKLAVA</v>
       </c>
       <c r="B103" t="str">
         <v>Da Ordinare</v>
@@ -1534,7 +1534,7 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>MANDARINO</v>
+        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
       </c>
       <c r="B104" t="str">
         <v>Da Ordinare</v>
@@ -1545,18 +1545,18 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>PASTIERA NAPOLETANA</v>
+        <v>MANDARINO</v>
       </c>
       <c r="B105" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C105" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>ALBICOCCA</v>
+        <v>CIOCCOLATO WASABI</v>
       </c>
       <c r="B106" t="str">
         <v>Da Ordinare</v>
@@ -1567,18 +1567,18 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>CIOCCOLATA CALDA FONDENTE</v>
+        <v>PASTIERA NAPOLETANA</v>
       </c>
       <c r="B107" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C107" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>ZABAIONE AL SAKE'</v>
+        <v>ALBICOCCA</v>
       </c>
       <c r="B108" t="str">
         <v>Da Ordinare</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>CACHI</v>
+        <v>CIOCCOLATA CALDA FONDENTE</v>
       </c>
       <c r="B109" t="str">
         <v>Da Ordinare</v>
@@ -1600,7 +1600,7 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>CIOCCOLATO</v>
+        <v>ZABAIONE AL SAKE'</v>
       </c>
       <c r="B110" t="str">
         <v>Da Ordinare</v>
@@ -1611,7 +1611,7 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>CACHI</v>
       </c>
       <c r="B111" t="str">
         <v>Da Ordinare</v>
@@ -1622,18 +1622,29 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>FINOCCHIO MIELE LIQUIRIZIA</v>
+        <v>CIOCCOLATO</v>
       </c>
       <c r="B112" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C112" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>ZABAIONE GELATO</v>
+      </c>
+      <c r="B113" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C113" t="str">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C112"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C113"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly SHOCAPP data 2026-05-17
</commit_message>
<xml_diff>
--- a/output/shocapp_da_ordinare.xlsx
+++ b/output/shocapp_da_ordinare.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C116"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,7 +418,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C2" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -451,7 +451,7 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C5" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -473,12 +473,12 @@
         <v>Da Ordinare</v>
       </c>
       <c r="C7" t="str">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>BANANA E LIME</v>
+        <v>BAKLAVA</v>
       </c>
       <c r="B8" t="str">
         <v>Da Ordinare</v>
@@ -489,40 +489,40 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>BIANCANEVE</v>
+        <v>BANANA E LIME</v>
       </c>
       <c r="B9" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C9" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>CAFFE'</v>
+        <v>BASILICO NOCI E MIELE</v>
       </c>
       <c r="B10" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C10" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>CIOCCOLATO AL LATTE gelato</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="B11" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C11" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CIOCCOLATO AL PIMENTO</v>
+        <v>CAFFE'</v>
       </c>
       <c r="B12" t="str">
         <v>Da Ordinare</v>
@@ -533,18 +533,18 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>CIOCCOLATO CRUDO DEL PERU'</v>
+        <v>CASTAGNA E MIRTO</v>
       </c>
       <c r="B13" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C13" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CIOCCOLATO E ARANCIA</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="B14" t="str">
         <v>Da Ordinare</v>
@@ -555,18 +555,18 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CIOCCOLATO KENTUCKY</v>
+        <v>CIOCCOLATO AL LATTE gelato</v>
       </c>
       <c r="B15" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C15" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
+        <v>CIOCCOLATO AL PIMENTO</v>
       </c>
       <c r="B16" t="str">
         <v>Da Ordinare</v>
@@ -577,117 +577,117 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>CIOCCOLATO CRUDO DEL PERU'</v>
       </c>
       <c r="B17" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C17" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>CIOCCOLATO VENEZUELA</v>
+        <v>CIOCCOLATO BIANCO</v>
       </c>
       <c r="B18" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C18" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CREMA  PASTICCIERA PARISI</v>
+        <v>CIOCCOLATO E ARANCIA</v>
       </c>
       <c r="B19" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C19" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CREMA CANNELLA</v>
+        <v>CIOCCOLATO KENTUCKY</v>
       </c>
       <c r="B20" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C20" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>CREMA FRAGOLE E MANDORLE</v>
+        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
       </c>
       <c r="B21" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C21" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CREMA VANIGLIA</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="B22" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C22" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
+        <v>CIOCCOLATO VENEZUELA</v>
       </c>
       <c r="B23" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C23" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>FIORDILATTE</v>
+        <v>COCCO CREMA</v>
       </c>
       <c r="B24" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C24" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>FRAGOLA</v>
+        <v>COCCO AL RUM</v>
       </c>
       <c r="B25" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C25" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
+        <v>CREMA  PASTICCIERA PARISI</v>
       </c>
       <c r="B26" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C26" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="B27" t="str">
         <v>Da Ordinare</v>
@@ -698,40 +698,40 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>LIMONE</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="B28" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C28" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>LIQUIRIZIA</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="B29" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C29" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>CREMA VANIGLIA</v>
       </c>
       <c r="B30" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C30" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
       </c>
       <c r="B31" t="str">
         <v>Da Ordinare</v>
@@ -742,7 +742,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>ESTASI</v>
       </c>
       <c r="B32" t="str">
         <v>Da Ordinare</v>
@@ -753,62 +753,62 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>MANDORLA TOSTATA</v>
+        <v>FIORDILATTE</v>
       </c>
       <c r="B33" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C33" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>MELA MANDORLA E CANNELLA</v>
+        <v>FRAGOLA</v>
       </c>
       <c r="B34" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C34" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>MELONE</v>
+        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
       </c>
       <c r="B35" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C35" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B36" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C36" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>NOCCIOLA</v>
+        <v>LATTE MENTA E CIOCCOLATO</v>
       </c>
       <c r="B37" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C37" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>NOCCIOLA AL FRUTTOSIO</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="B38" t="str">
         <v>Da Ordinare</v>
@@ -819,29 +819,29 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>LIMONE</v>
       </c>
       <c r="B39" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C39" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>PAPAYA</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B40" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C40" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>PASSION FRUIT</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="B41" t="str">
         <v>Da Ordinare</v>
@@ -852,18 +852,18 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>PERA</v>
+        <v>MANDORLA TOSTATA</v>
       </c>
       <c r="B42" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C42" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="B43" t="str">
         <v>Da Ordinare</v>
@@ -874,18 +874,18 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>MELA MANDORLA E CANNELLA</v>
       </c>
       <c r="B44" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C44" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>POLLICINA</v>
+        <v>MELONE</v>
       </c>
       <c r="B45" t="str">
         <v>Da Ordinare</v>
@@ -896,51 +896,51 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>PUNCH PARADISE</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B46" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C46" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B47" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C47" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>SEADAS</v>
+        <v>NOCCIOLA AL FRUTTOSIO</v>
       </c>
       <c r="B48" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C48" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>STRACCIATELLA</v>
+        <v>NOCI  E UVETTA DI CORINTO</v>
       </c>
       <c r="B49" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C49" t="str">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>TIRAMISU'</v>
+        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
       </c>
       <c r="B50" t="str">
         <v>Da Ordinare</v>
@@ -951,7 +951,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>UVA E NOCI</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="B51" t="str">
         <v>Da Ordinare</v>
@@ -962,18 +962,18 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>YOGURT</v>
+        <v>PERA</v>
       </c>
       <c r="B52" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C52" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+        <v>PERA AL GORGONZOLA</v>
       </c>
       <c r="B53" t="str">
         <v>Da Ordinare</v>
@@ -984,7 +984,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>MELOGRANO WONDERFUL</v>
+        <v>PERE BELLE HELENE</v>
       </c>
       <c r="B54" t="str">
         <v>Da Ordinare</v>
@@ -995,7 +995,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>PENSIERO</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="B55" t="str">
         <v>Da Ordinare</v>
@@ -1006,7 +1006,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>SACRIPANTE</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="B56" t="str">
         <v>Da Ordinare</v>
@@ -1017,62 +1017,62 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>BUONGIORNO AMORE</v>
+        <v>POLLICINA</v>
       </c>
       <c r="B57" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C57" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>PUNCH PARADISE</v>
       </c>
       <c r="B58" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C58" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>CARROT CAKE</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B59" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C59" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>RICOTTA, MIELE E COCCO</v>
       </c>
       <c r="B60" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C60" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="B61" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C61" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ROSA KARKADE E ARANCIA</v>
+        <v>SEADAS</v>
       </c>
       <c r="B62" t="str">
         <v>Da Ordinare</v>
@@ -1083,18 +1083,18 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B63" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C63" t="str">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B64" t="str">
         <v>Da Ordinare</v>
@@ -1105,7 +1105,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>CASTAGNA AL WHISKY</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B65" t="str">
         <v>Da Ordinare</v>
@@ -1116,7 +1116,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>FAVE FRESCHE &amp; PECORINO</v>
+        <v>VENERE ROSA</v>
       </c>
       <c r="B66" t="str">
         <v>Da Ordinare</v>
@@ -1127,51 +1127,51 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>LIMONE &amp; BASILICO</v>
+        <v>YOGURT</v>
       </c>
       <c r="B67" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C67" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>CREMA MASCARPONE</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
       </c>
       <c r="B68" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C68" t="str">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>COCONUT RICE CAKE</v>
+        <v>PENSIERO</v>
       </c>
       <c r="B69" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C69" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>PISTACCHIO LARNAKA , CIPRO</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B70" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C70" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
+        <v>CARROT CAKE</v>
       </c>
       <c r="B71" t="str">
         <v>Da Ordinare</v>
@@ -1182,40 +1182,40 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>BASILICO NOCI E MIELE</v>
+        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
       </c>
       <c r="B72" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C72" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>CASTAGNA E MIRTO</v>
+        <v>FIOR DI CIOCCOLATO</v>
       </c>
       <c r="B73" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C73" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>ROSA KARKADE E ARANCIA</v>
       </c>
       <c r="B74" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C74" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>CIOCCOLATO ROSEMARY</v>
+        <v>AVOCADO LIME E VINO BIANCO</v>
       </c>
       <c r="B75" t="str">
         <v>Da Ordinare</v>
@@ -1226,106 +1226,106 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>COCCO CREMA</v>
+        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
       </c>
       <c r="B76" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C76" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>CREMA AGNESE</v>
+        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
       </c>
       <c r="B77" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C77" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>ESTASI</v>
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
       </c>
       <c r="B78" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C78" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>GIANDUIA</v>
+        <v>EVERGREEN  BRONTE VEGAN</v>
       </c>
       <c r="B79" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C79" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>LATTE MENTA E CIOCCOLATO</v>
+        <v>SACHER TORTE</v>
       </c>
       <c r="B80" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C80" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>LEMON CURD</v>
+        <v>FAVE FRESCHE &amp; PECORINO</v>
       </c>
       <c r="B81" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C81" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>CREMA MASCARPONE</v>
       </c>
       <c r="B82" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C82" t="str">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>MIRTILLO</v>
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
       </c>
       <c r="B83" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C83" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>PERE BELLE HELENE</v>
+        <v>COCONUT RICE CAKE</v>
       </c>
       <c r="B84" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C84" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>PISTACCHIO LARNAKA , CIPRO</v>
       </c>
       <c r="B85" t="str">
         <v>Da Ordinare</v>
@@ -1336,29 +1336,29 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>RICOTTA, MIELE E COCCO</v>
+        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
       </c>
       <c r="B86" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C86" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>AVOCADO LIME E VINO BIANCO</v>
+        <v>ZABAIONE NEW</v>
       </c>
       <c r="B87" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C87" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>MONT BLANC</v>
+        <v>CREMA FRAGOLE E MANDORLE</v>
       </c>
       <c r="B88" t="str">
         <v>Da Ordinare</v>
@@ -1369,18 +1369,18 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
+        <v>GIANDUIA</v>
       </c>
       <c r="B89" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C89" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>SACHER TORTE</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B90" t="str">
         <v>Da Ordinare</v>
@@ -1391,139 +1391,139 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="B91" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C91" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>ZABAIONE NEW</v>
+        <v>MORA</v>
       </c>
       <c r="B92" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C92" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>STRAWBERRY FIELD FOREVER</v>
+        <v>PAPAYA</v>
       </c>
       <c r="B93" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C93" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
+        <v>ZABAIONE GELATO</v>
       </c>
       <c r="B94" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C94" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>MORA</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B95" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C95" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>SUSHI VEGANO</v>
+        <v>BUONGIORNO AMORE</v>
       </c>
       <c r="B96" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C96" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>CIOCCOLATO AL WHISKY</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="B97" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C97" t="str">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>TORTA CAPRESE</v>
+        <v>STRAWBERRY FIELD FOREVER</v>
       </c>
       <c r="B98" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C98" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>MOJITO ALLA AMARENA</v>
+        <v>CIOCCOLATO ROSEMARY</v>
       </c>
       <c r="B99" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C99" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>FIOR DI CIOCCOLATO</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B100" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C100" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>COCCO</v>
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
       </c>
       <c r="B101" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C101" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+        <v>SUSHI VEGANO</v>
       </c>
       <c r="B102" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C102" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>BAKLAVA</v>
+        <v>CIOCCOLATO AL WHISKY</v>
       </c>
       <c r="B103" t="str">
         <v>Da Ordinare</v>
@@ -1534,18 +1534,18 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
+        <v>MONT BLANC</v>
       </c>
       <c r="B104" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C104" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>MANDARINO</v>
+        <v>TORTA CAPRESE</v>
       </c>
       <c r="B105" t="str">
         <v>Da Ordinare</v>
@@ -1556,29 +1556,29 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>CIOCCOLATO WASABI</v>
+        <v>MOJITO ALLA AMARENA</v>
       </c>
       <c r="B106" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C106" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>PASTIERA NAPOLETANA</v>
+        <v>COCCO</v>
       </c>
       <c r="B107" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C107" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>ALBICOCCA</v>
+        <v>CASTAGNA AL WHISKY</v>
       </c>
       <c r="B108" t="str">
         <v>Da Ordinare</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>CIOCCOLATA CALDA FONDENTE</v>
+        <v>MANDARINO</v>
       </c>
       <c r="B109" t="str">
         <v>Da Ordinare</v>
@@ -1600,7 +1600,7 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>ZABAIONE AL SAKE'</v>
+        <v>CIOCCOLATO WASABI</v>
       </c>
       <c r="B110" t="str">
         <v>Da Ordinare</v>
@@ -1611,18 +1611,18 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>CACHI</v>
+        <v>PASTIERA NAPOLETANA</v>
       </c>
       <c r="B111" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C111" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>CIOCCOLATO</v>
+        <v>ALBICOCCA</v>
       </c>
       <c r="B112" t="str">
         <v>Da Ordinare</v>
@@ -1633,18 +1633,51 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>CIOCCOLATA CALDA FONDENTE</v>
       </c>
       <c r="B113" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C113" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>ZABAIONE AL SAKE'</v>
+      </c>
+      <c r="B114" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C114" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>CACHI</v>
+      </c>
+      <c r="B115" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C115" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>CIOCCOLATO</v>
+      </c>
+      <c r="B116" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C116" t="str">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C113"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C116"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly SHOCAPP data 2026-05-24
</commit_message>
<xml_diff>
--- a/output/shocapp_da_ordinare.xlsx
+++ b/output/shocapp_da_ordinare.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C118"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,7 +412,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>AMARENA</v>
+        <v>ANANAS E ZENZERO</v>
       </c>
       <c r="B2" t="str">
         <v>Da Ordinare</v>
@@ -423,18 +423,18 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ANANAS E ZENZERO</v>
+        <v>ANGURIA</v>
       </c>
       <c r="B3" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C3" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ANGURIA</v>
+        <v>ARACHIDI COCCO E CIOCCOLATO</v>
       </c>
       <c r="B4" t="str">
         <v>Da Ordinare</v>
@@ -445,40 +445,40 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ARACHIDI COCCO E CIOCCOLATO</v>
+        <v>GIANDUIA VARIEGATA</v>
       </c>
       <c r="B5" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C5" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>GIANDUIA VARIEGATA</v>
+        <v>BACIO DEL PRINCIPE</v>
       </c>
       <c r="B6" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C6" t="str">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>BACIO DEL PRINCIPE</v>
+        <v>BAKLAVA</v>
       </c>
       <c r="B7" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C7" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>BAKLAVA</v>
+        <v>BANANA E LIME</v>
       </c>
       <c r="B8" t="str">
         <v>Da Ordinare</v>
@@ -489,18 +489,18 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>BANANA E LIME</v>
+        <v>BASILICO NOCI E MIELE</v>
       </c>
       <c r="B9" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C9" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>BASILICO NOCI E MIELE</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="B10" t="str">
         <v>Da Ordinare</v>
@@ -511,18 +511,18 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>BIANCANEVE</v>
+        <v>CAFFE'</v>
       </c>
       <c r="B11" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C11" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CAFFE'</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="B12" t="str">
         <v>Da Ordinare</v>
@@ -533,18 +533,18 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>CASTAGNA E MIRTO</v>
+        <v>CIOCCOLATO AL LATTE gelato</v>
       </c>
       <c r="B13" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C13" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>CIOCCOLATO AL PIMENTO</v>
       </c>
       <c r="B14" t="str">
         <v>Da Ordinare</v>
@@ -555,29 +555,29 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CIOCCOLATO AL LATTE gelato</v>
+        <v>CIOCCOLATO BIANCO</v>
       </c>
       <c r="B15" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C15" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CIOCCOLATO AL PIMENTO</v>
+        <v>CIOCCOLATO E ARANCIA</v>
       </c>
       <c r="B16" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C16" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>CIOCCOLATO CRUDO DEL PERU'</v>
+        <v>CIOCCOLATO KENTUCKY</v>
       </c>
       <c r="B17" t="str">
         <v>Da Ordinare</v>
@@ -588,7 +588,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>CIOCCOLATO BIANCO</v>
+        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
       </c>
       <c r="B18" t="str">
         <v>Da Ordinare</v>
@@ -599,18 +599,18 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CIOCCOLATO E ARANCIA</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="B19" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C19" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CIOCCOLATO KENTUCKY</v>
+        <v>CIOCCOLATO VENEZUELA</v>
       </c>
       <c r="B20" t="str">
         <v>Da Ordinare</v>
@@ -621,7 +621,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
+        <v>COCCO AL RUM</v>
       </c>
       <c r="B21" t="str">
         <v>Da Ordinare</v>
@@ -632,18 +632,18 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>CREMA  PASTICCIERA PARISI</v>
       </c>
       <c r="B22" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C22" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>CIOCCOLATO VENEZUELA</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="B23" t="str">
         <v>Da Ordinare</v>
@@ -654,7 +654,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>COCCO CREMA</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="B24" t="str">
         <v>Da Ordinare</v>
@@ -665,7 +665,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>COCCO AL RUM</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="B25" t="str">
         <v>Da Ordinare</v>
@@ -676,18 +676,18 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>CREMA  PASTICCIERA PARISI</v>
+        <v>CREMA FRAGOLE E MANDORLE</v>
       </c>
       <c r="B26" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C26" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>CREMA AGNESE</v>
+        <v>CREMA VANIGLIA</v>
       </c>
       <c r="B27" t="str">
         <v>Da Ordinare</v>
@@ -698,7 +698,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
+        <v>ESTASI</v>
       </c>
       <c r="B28" t="str">
         <v>Da Ordinare</v>
@@ -709,95 +709,95 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>CREMA CANNELLA</v>
+        <v>FIORDILATTE</v>
       </c>
       <c r="B29" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C29" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>CREMA VANIGLIA</v>
+        <v>FRAGOLA</v>
       </c>
       <c r="B30" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C30" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
+        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
       </c>
       <c r="B31" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C31" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ESTASI</v>
+        <v>GIANDUIA</v>
       </c>
       <c r="B32" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C32" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>FIORDILATTE</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B33" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C33" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>FRAGOLA</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="B34" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C34" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
+        <v>LIMONE</v>
       </c>
       <c r="B35" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C35" t="str">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B36" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C36" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>LATTE MENTA E CIOCCOLATO</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B37" t="str">
         <v>Da Ordinare</v>
@@ -808,7 +808,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>LEMON CURD</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B38" t="str">
         <v>Da Ordinare</v>
@@ -819,29 +819,29 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>LIMONE</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="B39" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C39" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>MANDORLA TOSTATA</v>
       </c>
       <c r="B40" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C40" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>MELA MANDORLA E CANNELLA</v>
       </c>
       <c r="B41" t="str">
         <v>Da Ordinare</v>
@@ -852,7 +852,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>MANDORLA TOSTATA</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="B42" t="str">
         <v>Da Ordinare</v>
@@ -863,7 +863,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>MORA</v>
       </c>
       <c r="B43" t="str">
         <v>Da Ordinare</v>
@@ -874,7 +874,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>MELA MANDORLA E CANNELLA</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B44" t="str">
         <v>Da Ordinare</v>
@@ -885,40 +885,40 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>MELONE</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B45" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C45" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>NOCCIOLA AL FRUTTOSIO</v>
       </c>
       <c r="B46" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C46" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>NOCCIOLA</v>
+        <v>NOCI  E UVETTA DI CORINTO</v>
       </c>
       <c r="B47" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C47" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>NOCCIOLA AL FRUTTOSIO</v>
+        <v>PERA</v>
       </c>
       <c r="B48" t="str">
         <v>Da Ordinare</v>
@@ -929,7 +929,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>NOCI  E UVETTA DI CORINTO</v>
+        <v>PERA AL GORGONZOLA</v>
       </c>
       <c r="B49" t="str">
         <v>Da Ordinare</v>
@@ -940,7 +940,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>PERE BELLE HELENE</v>
       </c>
       <c r="B50" t="str">
         <v>Da Ordinare</v>
@@ -951,29 +951,29 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>PASSION FRUIT</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="B51" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C51" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>PERA</v>
+        <v>POLLICINA</v>
       </c>
       <c r="B52" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C52" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>PERA AL GORGONZOLA</v>
+        <v>PUNCH PARADISE</v>
       </c>
       <c r="B53" t="str">
         <v>Da Ordinare</v>
@@ -984,128 +984,128 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>PERE BELLE HELENE</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B54" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C54" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="B55" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C55" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>SEADAS</v>
       </c>
       <c r="B56" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C56" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>POLLICINA</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B57" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C57" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>PUNCH PARADISE</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B58" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C58" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B59" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C59" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>RICOTTA, MIELE E COCCO</v>
+        <v>YOGURT</v>
       </c>
       <c r="B60" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C60" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>MELOGRANO WONDERFUL</v>
       </c>
       <c r="B61" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C61" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>SEADAS</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B62" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C62" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>STRACCIATELLA</v>
+        <v>BUONGIORNO AMORE</v>
       </c>
       <c r="B63" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C63" t="str">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>TIRAMISU'</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B64" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C64" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>UVA E NOCI</v>
+        <v>CARROT CAKE</v>
       </c>
       <c r="B65" t="str">
         <v>Da Ordinare</v>
@@ -1116,84 +1116,84 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>VENERE ROSA</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="B66" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C66" t="str">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>YOGURT</v>
+        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
       </c>
       <c r="B67" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C67" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+        <v>ROSA KARKADE E ARANCIA</v>
       </c>
       <c r="B68" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C68" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>PENSIERO</v>
+        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
       </c>
       <c r="B69" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C69" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>LATTE DI FICO (PAMPANELLA)</v>
       </c>
       <c r="B70" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C70" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>CARROT CAKE</v>
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
       </c>
       <c r="B71" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C71" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
+        <v>SACHER TORTE</v>
       </c>
       <c r="B72" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C72" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>FIOR DI CIOCCOLATO</v>
+        <v>FRAGOLE DI TERRACINA &amp; CHAMPAGNE</v>
       </c>
       <c r="B73" t="str">
         <v>Da Ordinare</v>
@@ -1204,29 +1204,29 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>ROSA KARKADE E ARANCIA</v>
+        <v>CREMA MASCARPONE</v>
       </c>
       <c r="B74" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C74" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>AVOCADO LIME E VINO BIANCO</v>
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
       </c>
       <c r="B75" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C75" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
+        <v>COCONUT RICE CAKE</v>
       </c>
       <c r="B76" t="str">
         <v>Da Ordinare</v>
@@ -1237,128 +1237,128 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
+        <v>PISTACCHIO LARNAKA , CIPRO</v>
       </c>
       <c r="B77" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C77" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
       </c>
       <c r="B78" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C78" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
+        <v>AMARENA</v>
       </c>
       <c r="B79" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C79" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>SACHER TORTE</v>
+        <v>CIOCCOLATO CRUDO DEL PERU'</v>
       </c>
       <c r="B80" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C80" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>FAVE FRESCHE &amp; PECORINO</v>
+        <v>COCCO CREMA</v>
       </c>
       <c r="B81" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C81" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>CREMA MASCARPONE</v>
+        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
       </c>
       <c r="B82" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C82" t="str">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+        <v>LATTE MENTA E CIOCCOLATO</v>
       </c>
       <c r="B83" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C83" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>COCONUT RICE CAKE</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="B84" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C84" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>PISTACCHIO LARNAKA , CIPRO</v>
+        <v>MELONE</v>
       </c>
       <c r="B85" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C85" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
+        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
       </c>
       <c r="B86" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C86" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>ZABAIONE NEW</v>
+        <v>PAPAYA</v>
       </c>
       <c r="B87" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C87" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>CREMA FRAGOLE E MANDORLE</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="B88" t="str">
         <v>Da Ordinare</v>
@@ -1369,18 +1369,18 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>GIANDUIA</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="B89" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C89" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>RICOTTA, MIELE E COCCO</v>
       </c>
       <c r="B90" t="str">
         <v>Da Ordinare</v>
@@ -1391,29 +1391,29 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>MIRTILLO</v>
+        <v>VENERE ROSA</v>
       </c>
       <c r="B91" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C91" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>MORA</v>
+        <v>CIOCCOLATO WASABI</v>
       </c>
       <c r="B92" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C92" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>PAPAYA</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
       </c>
       <c r="B93" t="str">
         <v>Da Ordinare</v>
@@ -1424,51 +1424,51 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>PENSIERO</v>
       </c>
       <c r="B94" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C94" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>SACRIPANTE</v>
+        <v>FIOR DI CIOCCOLATO</v>
       </c>
       <c r="B95" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C95" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>BUONGIORNO AMORE</v>
+        <v>AVOCADO LIME E VINO BIANCO</v>
       </c>
       <c r="B96" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C96" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
       </c>
       <c r="B97" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C97" t="str">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>STRAWBERRY FIELD FOREVER</v>
+        <v>EVERGREEN  BRONTE VEGAN</v>
       </c>
       <c r="B98" t="str">
         <v>Da Ordinare</v>
@@ -1479,7 +1479,7 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>CIOCCOLATO ROSEMARY</v>
+        <v>CASTAGNA AL WHISKY</v>
       </c>
       <c r="B99" t="str">
         <v>Da Ordinare</v>
@@ -1490,51 +1490,51 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>LIQUIRIZIA</v>
+        <v>FAVE FRESCHE &amp; PECORINO</v>
       </c>
       <c r="B100" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C100" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+        <v>LIMONE &amp; BASILICO</v>
       </c>
       <c r="B101" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C101" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>SUSHI VEGANO</v>
+        <v>ZABAIONE NEW</v>
       </c>
       <c r="B102" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C102" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>CIOCCOLATO AL WHISKY</v>
+        <v>STRAWBERRY FIELD FOREVER</v>
       </c>
       <c r="B103" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C103" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>MONT BLANC</v>
+        <v>CASTAGNA E MIRTO</v>
       </c>
       <c r="B104" t="str">
         <v>Da Ordinare</v>
@@ -1545,7 +1545,7 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>TORTA CAPRESE</v>
+        <v>ZABAIONE GELATO</v>
       </c>
       <c r="B105" t="str">
         <v>Da Ordinare</v>
@@ -1556,29 +1556,29 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>MOJITO ALLA AMARENA</v>
+        <v>CIOCCOLATO ROSEMARY</v>
       </c>
       <c r="B106" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C106" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>COCCO</v>
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
       </c>
       <c r="B107" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C107" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>CASTAGNA AL WHISKY</v>
+        <v>SUSHI VEGANO</v>
       </c>
       <c r="B108" t="str">
         <v>Da Ordinare</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>MANDARINO</v>
+        <v>CIOCCOLATO AL WHISKY</v>
       </c>
       <c r="B109" t="str">
         <v>Da Ordinare</v>
@@ -1600,7 +1600,7 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>CIOCCOLATO WASABI</v>
+        <v>MONT BLANC</v>
       </c>
       <c r="B110" t="str">
         <v>Da Ordinare</v>
@@ -1611,29 +1611,29 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>PASTIERA NAPOLETANA</v>
+        <v>TORTA CAPRESE</v>
       </c>
       <c r="B111" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C111" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>ALBICOCCA</v>
+        <v>MOJITO ALLA AMARENA</v>
       </c>
       <c r="B112" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C112" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>CIOCCOLATA CALDA FONDENTE</v>
+        <v>COCCO</v>
       </c>
       <c r="B113" t="str">
         <v>Da Ordinare</v>
@@ -1644,7 +1644,7 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>ZABAIONE AL SAKE'</v>
+        <v>MANDARINO</v>
       </c>
       <c r="B114" t="str">
         <v>Da Ordinare</v>
@@ -1655,29 +1655,51 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>CACHI</v>
+        <v>PASTIERA NAPOLETANA</v>
       </c>
       <c r="B115" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C115" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>CIOCCOLATO</v>
+        <v>ALBICOCCA</v>
       </c>
       <c r="B116" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C116" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>CIOCCOLATA CALDA FONDENTE</v>
+      </c>
+      <c r="B117" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C117" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>ZABAIONE AL SAKE'</v>
+      </c>
+      <c r="B118" t="str">
+        <v>Da Ordinare</v>
+      </c>
+      <c r="C118" t="str">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C116"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C118"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly SHOCAPP data 2026-05-31
</commit_message>
<xml_diff>
--- a/output/shocapp_da_ordinare.xlsx
+++ b/output/shocapp_da_ordinare.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C114"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,18 +412,18 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ANANAS E ZENZERO</v>
+        <v>AMARENA</v>
       </c>
       <c r="B2" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C2" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ANGURIA</v>
+        <v>ANANAS E ZENZERO</v>
       </c>
       <c r="B3" t="str">
         <v>Da Ordinare</v>
@@ -434,7 +434,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ARACHIDI COCCO E CIOCCOLATO</v>
+        <v>BACIO DEL PRINCIPE</v>
       </c>
       <c r="B4" t="str">
         <v>Da Ordinare</v>
@@ -445,7 +445,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>GIANDUIA VARIEGATA</v>
+        <v>BAKLAVA</v>
       </c>
       <c r="B5" t="str">
         <v>Da Ordinare</v>
@@ -456,40 +456,40 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BACIO DEL PRINCIPE</v>
+        <v>BANANA E LIME</v>
       </c>
       <c r="B6" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C6" t="str">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>BAKLAVA</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="B7" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C7" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>BANANA E LIME</v>
+        <v>CIOCCOLATO AL LATTE gelato</v>
       </c>
       <c r="B8" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C8" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>BASILICO NOCI E MIELE</v>
+        <v>CIOCCOLATO AL PIMENTO</v>
       </c>
       <c r="B9" t="str">
         <v>Da Ordinare</v>
@@ -500,7 +500,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>BIANCANEVE</v>
+        <v>CIOCCOLATO BIANCO</v>
       </c>
       <c r="B10" t="str">
         <v>Da Ordinare</v>
@@ -511,40 +511,40 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>CAFFE'</v>
+        <v>CIOCCOLATO E ARANCIA</v>
       </c>
       <c r="B11" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C11" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>CIOCCOLATO KENTUCKY</v>
       </c>
       <c r="B12" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C12" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>CIOCCOLATO AL LATTE gelato</v>
+        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
       </c>
       <c r="B13" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C13" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CIOCCOLATO AL PIMENTO</v>
+        <v>CIOCCOLATO MADAGASCAR</v>
       </c>
       <c r="B14" t="str">
         <v>Da Ordinare</v>
@@ -555,40 +555,40 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CIOCCOLATO BIANCO</v>
+        <v>CIOCCOLATO VENEZUELA</v>
       </c>
       <c r="B15" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C15" t="str">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CIOCCOLATO E ARANCIA</v>
+        <v>COCCO CREMA</v>
       </c>
       <c r="B16" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C16" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>CIOCCOLATO KENTUCKY</v>
+        <v>CREMA  PASTICCIERA PARISI</v>
       </c>
       <c r="B17" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C17" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>CIOCCOLATO LAPSANG SOUCHOUNG</v>
+        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
       </c>
       <c r="B18" t="str">
         <v>Da Ordinare</v>
@@ -599,7 +599,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CIOCCOLATO MADAGASCAR</v>
+        <v>CREMA CANNELLA</v>
       </c>
       <c r="B19" t="str">
         <v>Da Ordinare</v>
@@ -610,18 +610,18 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CIOCCOLATO VENEZUELA</v>
+        <v>CREMA FRAGOLE E MANDORLE</v>
       </c>
       <c r="B20" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C20" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>COCCO AL RUM</v>
+        <v>CREMA VANIGLIA</v>
       </c>
       <c r="B21" t="str">
         <v>Da Ordinare</v>
@@ -632,7 +632,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CREMA  PASTICCIERA PARISI</v>
+        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
       </c>
       <c r="B22" t="str">
         <v>Da Ordinare</v>
@@ -643,51 +643,51 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>CREMA AGNESE</v>
+        <v>FIORDILATTE</v>
       </c>
       <c r="B23" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C23" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>CREMA BANANA CON CROCCANTINO CIOCCOLATO &amp; SESAMO</v>
+        <v>FRAGOLA</v>
       </c>
       <c r="B24" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C24" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>CREMA CANNELLA</v>
+        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
       </c>
       <c r="B25" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C25" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>CREMA FRAGOLE E MANDORLE</v>
+        <v>GIANDUIA</v>
       </c>
       <c r="B26" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C26" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>CREMA VANIGLIA</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B27" t="str">
         <v>Da Ordinare</v>
@@ -698,7 +698,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ESTASI</v>
+        <v>LATTE MENTA E CIOCCOLATO</v>
       </c>
       <c r="B28" t="str">
         <v>Da Ordinare</v>
@@ -709,40 +709,40 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>FIORDILATTE</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="B29" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C29" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>FRAGOLA</v>
+        <v>LIMONE</v>
       </c>
       <c r="B30" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C30" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>FRUTTI DI BOSCO(LAMPONE,RIBES,MORA,MIRTILLO)</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B31" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C31" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>GIANDUIA</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B32" t="str">
         <v>Da Ordinare</v>
@@ -753,18 +753,18 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="B33" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C33" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>LEMON CURD</v>
+        <v>MANDORLA TOSTATA</v>
       </c>
       <c r="B34" t="str">
         <v>Da Ordinare</v>
@@ -775,62 +775,62 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>LIMONE</v>
+        <v>MANGO SOLE DI SICILIA</v>
       </c>
       <c r="B35" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C35" t="str">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>LIQUIRIZIA</v>
+        <v>MELA MANDORLA E CANNELLA</v>
       </c>
       <c r="B36" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C36" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>MELONE</v>
       </c>
       <c r="B37" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C37" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="B38" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C38" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B39" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C39" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>MANDORLA TOSTATA</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B40" t="str">
         <v>Da Ordinare</v>
@@ -841,29 +841,29 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>MELA MANDORLA E CANNELLA</v>
+        <v>NOCCIOLA AL FRUTTOSIO</v>
       </c>
       <c r="B41" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C41" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>MIRTILLO</v>
+        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
       </c>
       <c r="B42" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C42" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>MORA</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="B43" t="str">
         <v>Da Ordinare</v>
@@ -874,62 +874,62 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>PERA</v>
       </c>
       <c r="B44" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C44" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>NOCCIOLA</v>
+        <v>PERE BELLE HELENE</v>
       </c>
       <c r="B45" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C45" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>NOCCIOLA AL FRUTTOSIO</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="B46" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C46" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>NOCI  E UVETTA DI CORINTO</v>
+        <v>PISTACCHIO DI BRONTE</v>
       </c>
       <c r="B47" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C47" t="str">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>PERA</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B48" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C48" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>PERA AL GORGONZOLA</v>
+        <v>RICOTTA, MIELE E COCCO</v>
       </c>
       <c r="B49" t="str">
         <v>Da Ordinare</v>
@@ -940,106 +940,106 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>PERE BELLE HELENE</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="B50" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C50" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>PISTACCHIO DI BRONTE</v>
+        <v>SEADAS</v>
       </c>
       <c r="B51" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C51" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>POLLICINA</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B52" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C52" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>PUNCH PARADISE</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B53" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C53" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B54" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C54" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>CIOCCOLATO WASABI</v>
       </c>
       <c r="B55" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C55" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>SEADAS</v>
+        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
       </c>
       <c r="B56" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C56" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>STRACCIATELLA</v>
+        <v>PENSIERO</v>
       </c>
       <c r="B57" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C57" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>TIRAMISU'</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B58" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C58" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>UVA E NOCI</v>
+        <v>CARROT CAKE</v>
       </c>
       <c r="B59" t="str">
         <v>Da Ordinare</v>
@@ -1050,18 +1050,18 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>YOGURT</v>
+        <v>PISTACCHIO SIRIANO</v>
       </c>
       <c r="B60" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C60" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>MELOGRANO WONDERFUL</v>
+        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
       </c>
       <c r="B61" t="str">
         <v>Da Ordinare</v>
@@ -1072,40 +1072,40 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>SACRIPANTE</v>
+        <v>ROSA KARKADE E ARANCIA</v>
       </c>
       <c r="B62" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C62" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>BUONGIORNO AMORE</v>
+        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
       </c>
       <c r="B63" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C63" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
       </c>
       <c r="B64" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C64" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>CARROT CAKE</v>
+        <v>LATTE DI FICO (PAMPANELLA)</v>
       </c>
       <c r="B65" t="str">
         <v>Da Ordinare</v>
@@ -1116,29 +1116,29 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>PISTACCHIO SIRIANO</v>
+        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
       </c>
       <c r="B66" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C66" t="str">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>STRACCHINO CON SALSA DI PERE AL MARSALA &amp; NOCI LARA</v>
+        <v>EVERGREEN  BRONTE VEGAN</v>
       </c>
       <c r="B67" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C67" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>ROSA KARKADE E ARANCIA</v>
+        <v>SACHER TORTE</v>
       </c>
       <c r="B68" t="str">
         <v>Da Ordinare</v>
@@ -1149,51 +1149,51 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>NOCCIOLA, BURRO &amp; FIORI DI SALVIA</v>
+        <v>CREMA MASCARPONE</v>
       </c>
       <c r="B69" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C69" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>LATTE DI FICO (PAMPANELLA)</v>
+        <v>COCONUT RICE CAKE</v>
       </c>
       <c r="B70" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C70" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>RICOTTA ROMANA, CACAO CRUDO &amp; PERA (LA-LA-LAND)</v>
+        <v>PISTACCHIO LARNAKA , CIPRO</v>
       </c>
       <c r="B71" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C71" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>SACHER TORTE</v>
+        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
       </c>
       <c r="B72" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C72" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>FRAGOLE DI TERRACINA &amp; CHAMPAGNE</v>
+        <v>FIORDILATTE NEW</v>
       </c>
       <c r="B73" t="str">
         <v>Da Ordinare</v>
@@ -1204,18 +1204,18 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>CREMA MASCARPONE</v>
+        <v>ZABAIONE NEW</v>
       </c>
       <c r="B74" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C74" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
+        <v>FASHIONED SPRITZ</v>
       </c>
       <c r="B75" t="str">
         <v>Da Ordinare</v>
@@ -1226,40 +1226,40 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>COCONUT RICE CAKE</v>
+        <v>ANGURIA</v>
       </c>
       <c r="B76" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C76" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>PISTACCHIO LARNAKA , CIPRO</v>
+        <v>ARACHIDI COCCO E CIOCCOLATO</v>
       </c>
       <c r="B77" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C77" t="str">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>CIOCCOLATO  UGANDA PERLA D'AFRICA</v>
+        <v>GIANDUIA VARIEGATA</v>
       </c>
       <c r="B78" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C78" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>AMARENA</v>
+        <v>BASILICO NOCI E MIELE</v>
       </c>
       <c r="B79" t="str">
         <v>Da Ordinare</v>
@@ -1270,29 +1270,29 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>CIOCCOLATO CRUDO DEL PERU'</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="B80" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C80" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>COCCO CREMA</v>
+        <v>CAFFE'</v>
       </c>
       <c r="B81" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C81" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>CREMA ZENZERO MIELE DI CASTAGNO E LIMONE</v>
+        <v>CASTAGNA E MIRTO</v>
       </c>
       <c r="B82" t="str">
         <v>Da Ordinare</v>
@@ -1303,40 +1303,40 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>LATTE MENTA E CIOCCOLATO</v>
+        <v>CIOCCOLATO CRUDO DEL PERU'</v>
       </c>
       <c r="B83" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C83" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>MANGO SOLE DI SICILIA</v>
+        <v>CREMA AGNESE</v>
       </c>
       <c r="B84" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C84" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>MELONE</v>
+        <v>ESTASI</v>
       </c>
       <c r="B85" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C85" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>PANACEA (Latte di mandorla Menta &amp; Ginseng)</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B86" t="str">
         <v>Da Ordinare</v>
@@ -1347,7 +1347,7 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>PAPAYA</v>
+        <v>MORA</v>
       </c>
       <c r="B87" t="str">
         <v>Da Ordinare</v>
@@ -1358,29 +1358,29 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>PASSION FRUIT</v>
+        <v>POLLICINA</v>
       </c>
       <c r="B88" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C88" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>PUNCH PARADISE</v>
       </c>
       <c r="B89" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C89" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>RICOTTA, MIELE E COCCO</v>
+        <v>VENERE ROSA</v>
       </c>
       <c r="B90" t="str">
         <v>Da Ordinare</v>
@@ -1391,40 +1391,40 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>VENERE ROSA</v>
+        <v>YOGURT</v>
       </c>
       <c r="B91" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C91" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>CIOCCOLATO WASABI</v>
+        <v>MELOGRANO WONDERFUL</v>
       </c>
       <c r="B92" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C92" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>FIORI DI LAVANDA E FRAGOLINE DI NEMI</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B93" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C93" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>PENSIERO</v>
+        <v>BUONGIORNO AMORE</v>
       </c>
       <c r="B94" t="str">
         <v>Da Ordinare</v>
@@ -1435,40 +1435,40 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>FIOR DI CIOCCOLATO</v>
+        <v>AVOCADO LIME E VINO BIANCO</v>
       </c>
       <c r="B95" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C95" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>AVOCADO LIME E VINO BIANCO</v>
+        <v>FRAGOLE DI TERRACINA &amp; CHAMPAGNE</v>
       </c>
       <c r="B96" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C96" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>DRACARYS (dragon fruit ,fragole &amp; peperoncino)</v>
+        <v>LIMONE &amp; BASILICO</v>
       </c>
       <c r="B97" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C97" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>EVERGREEN  BRONTE VEGAN</v>
+        <v>BANACHI, BANANA ARACHIDI &amp; CARAMELLO</v>
       </c>
       <c r="B98" t="str">
         <v>Da Ordinare</v>
@@ -1479,18 +1479,18 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>CASTAGNA AL WHISKY</v>
+        <v>PAPAYA</v>
       </c>
       <c r="B99" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C99" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>FAVE FRESCHE &amp; PECORINO</v>
+        <v>FIOR DI CIOCCOLATO</v>
       </c>
       <c r="B100" t="str">
         <v>Da Ordinare</v>
@@ -1501,7 +1501,7 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>LIMONE &amp; BASILICO</v>
+        <v>CASTAGNA AL WHISKY</v>
       </c>
       <c r="B101" t="str">
         <v>Da Ordinare</v>
@@ -1512,13 +1512,13 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>ZABAIONE NEW</v>
+        <v>FAVE FRESCHE &amp; PECORINO</v>
       </c>
       <c r="B102" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C102" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103">
@@ -1534,18 +1534,18 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>CASTAGNA E MIRTO</v>
+        <v>ZABAIONE GELATO</v>
       </c>
       <c r="B104" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C104" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>CIOCCOLATO ROSEMARY</v>
       </c>
       <c r="B105" t="str">
         <v>Da Ordinare</v>
@@ -1556,29 +1556,29 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>CIOCCOLATO ROSEMARY</v>
+        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
       </c>
       <c r="B106" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C106" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>STRACCHINO, ALBICOCCHE AL ROSMARINO &amp; BRICIOLE DI CROSTATA</v>
+        <v>SUSHI VEGANO</v>
       </c>
       <c r="B107" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C107" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>SUSHI VEGANO</v>
+        <v>CIOCCOLATO AL WHISKY</v>
       </c>
       <c r="B108" t="str">
         <v>Da Ordinare</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>CIOCCOLATO AL WHISKY</v>
+        <v>MONT BLANC</v>
       </c>
       <c r="B109" t="str">
         <v>Da Ordinare</v>
@@ -1600,7 +1600,7 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>MONT BLANC</v>
+        <v>TORTA CAPRESE</v>
       </c>
       <c r="B110" t="str">
         <v>Da Ordinare</v>
@@ -1611,29 +1611,29 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>TORTA CAPRESE</v>
+        <v>MOJITO ALLA AMARENA</v>
       </c>
       <c r="B111" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C111" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>MOJITO ALLA AMARENA</v>
+        <v>COCCO</v>
       </c>
       <c r="B112" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C112" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>COCCO</v>
+        <v>MANDARINO</v>
       </c>
       <c r="B113" t="str">
         <v>Da Ordinare</v>
@@ -1644,62 +1644,18 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>MANDARINO</v>
+        <v>PASTIERA NAPOLETANA</v>
       </c>
       <c r="B114" t="str">
         <v>Da Ordinare</v>
       </c>
       <c r="C114" t="str">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="str">
-        <v>PASTIERA NAPOLETANA</v>
-      </c>
-      <c r="B115" t="str">
-        <v>Da Ordinare</v>
-      </c>
-      <c r="C115" t="str">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="str">
-        <v>ALBICOCCA</v>
-      </c>
-      <c r="B116" t="str">
-        <v>Da Ordinare</v>
-      </c>
-      <c r="C116" t="str">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="str">
-        <v>CIOCCOLATA CALDA FONDENTE</v>
-      </c>
-      <c r="B117" t="str">
-        <v>Da Ordinare</v>
-      </c>
-      <c r="C117" t="str">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="str">
-        <v>ZABAIONE AL SAKE'</v>
-      </c>
-      <c r="B118" t="str">
-        <v>Da Ordinare</v>
-      </c>
-      <c r="C118" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C118"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C114"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add mobile app, server, GitHub Actions workflow
</commit_message>
<xml_diff>
--- a/output/shocapp_da_ordinare.xlsx
+++ b/output/shocapp_da_ordinare.xlsx
@@ -433,310 +433,310 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>P.BRONTE</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E2">
-        <v>766</v>
+        <v>454</v>
       </c>
       <c r="F2" t="str">
-        <v>1.20</v>
+        <v>1.06</v>
       </c>
       <c r="G2" t="str">
         <v>↑↑</v>
       </c>
       <c r="H2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J2" t="str">
-        <v>forecast 9 (7d:10 30d:26 trend:↑↑) +safety 3 -scorta 1</v>
+        <v>forecast 8 (7d:9 30d:22 trend:↑↑) +safety 3 -scorta 3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>STRACCIATELLA</v>
+        <v>C. AL LATTE GELATO</v>
       </c>
       <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>15</v>
+      </c>
+      <c r="E3">
+        <v>364</v>
+      </c>
+      <c r="F3" t="str">
+        <v>0.63</v>
+      </c>
+      <c r="G3" t="str">
+        <v>↑↑</v>
+      </c>
+      <c r="H3">
         <v>7</v>
       </c>
-      <c r="C3">
-        <v>11</v>
-      </c>
-      <c r="D3">
-        <v>45</v>
-      </c>
-      <c r="E3">
-        <v>806</v>
-      </c>
-      <c r="F3" t="str">
-        <v>1.54</v>
-      </c>
-      <c r="G3" t="str">
-        <v>→</v>
-      </c>
-      <c r="H3">
-        <v>15</v>
-      </c>
       <c r="I3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J3" t="str">
-        <v>forecast 11 (7d:11 30d:45 trend:→) +safety 4 -scorta 7</v>
+        <v>forecast 5 (7d:5 30d:15 trend:↑↑) +safety 2 -scorta 0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>C. VENEZUELA</v>
+        <v>P.BRONTE</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E4">
-        <v>265</v>
+        <v>768</v>
       </c>
       <c r="F4" t="str">
-        <v>0.73</v>
+        <v>1.09</v>
       </c>
       <c r="G4" t="str">
         <v>↑↑</v>
       </c>
       <c r="H4">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I4">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J4" t="str">
-        <v>forecast 6 (7d:6 30d:16 trend:↑↑) +safety 2 -scorta 0</v>
+        <v>forecast 8 (7d:9 30d:24 trend:↑↑) +safety 3 -scorta 6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>FIORDILATTE</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D5">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="E5">
-        <v>350</v>
+        <v>810</v>
       </c>
       <c r="F5" t="str">
-        <v>0.78</v>
+        <v>1.53</v>
       </c>
       <c r="G5" t="str">
-        <v>↑</v>
+        <v>→</v>
       </c>
       <c r="H5">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="I5">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J5" t="str">
-        <v>forecast 6 (7d:6 30d:20 trend:↑) +safety 2 -scorta 1</v>
+        <v>forecast 11 (7d:11 30d:44 trend:→) +safety 4 -scorta 11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ARACHIDI</v>
+        <v>BACIO</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C6">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D6">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="E6">
-        <v>288</v>
+        <v>809</v>
       </c>
       <c r="F6" t="str">
-        <v>0.59</v>
+        <v>1.39</v>
       </c>
       <c r="G6" t="str">
-        <v>↑↑</v>
+        <v>→</v>
       </c>
       <c r="H6">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="I6">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J6" t="str">
-        <v>forecast 5 (7d:5 30d:12 trend:↑↑) +safety 2 -scorta 0</v>
+        <v>forecast 10 (7d:10 30d:40 trend:→) +safety 3 -scorta 9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>PISTACCHIO LARNAKA</v>
+        <v>FIORDILATTE</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D7">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>352</v>
       </c>
       <c r="F7" t="str">
-        <v>0.72</v>
+        <v>0.78</v>
       </c>
       <c r="G7" t="str">
-        <v>↓↓</v>
+        <v>↑</v>
       </c>
       <c r="H7">
         <v>8</v>
       </c>
       <c r="I7">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J7" t="str">
-        <v>forecast 6 (7d:4 30d:28 trend:↓↓) +safety 2 -scorta 1</v>
+        <v>forecast 6 (7d:6 30d:20 trend:↑) +safety 2 -scorta 4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>FRAGOLA</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B8">
         <v>3</v>
       </c>
       <c r="C8">
+        <v>6</v>
+      </c>
+      <c r="D8">
         <v>7</v>
       </c>
-      <c r="D8">
-        <v>26</v>
-      </c>
       <c r="E8">
-        <v>513</v>
+        <v>176</v>
       </c>
       <c r="F8" t="str">
-        <v>0.95</v>
+        <v>0.61</v>
       </c>
       <c r="G8" t="str">
-        <v>↑</v>
+        <v>↑↑</v>
       </c>
       <c r="H8">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I8">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J8" t="str">
-        <v>forecast 7 (7d:7 30d:26 trend:↑) +safety 2 -scorta 3</v>
+        <v>forecast 5 (7d:6 30d:7 trend:↑↑) +safety 2 -scorta 3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>C. AL LATTE GELATO</v>
+        <v>C. VENEZUELA</v>
       </c>
       <c r="B9">
         <v>2</v>
       </c>
       <c r="C9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E9">
-        <v>362</v>
+        <v>266</v>
       </c>
       <c r="F9" t="str">
-        <v>0.63</v>
+        <v>0.57</v>
       </c>
       <c r="G9" t="str">
-        <v>↑↑</v>
+        <v>→</v>
       </c>
       <c r="H9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J9" t="str">
-        <v>forecast 5 (7d:5 30d:15 trend:↑↑) +safety 2 -scorta 2</v>
+        <v>forecast 4 (7d:4 30d:17 trend:→) +safety 2 -scorta 2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>CAFFE'</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="B10">
         <v>0</v>
       </c>
       <c r="C10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E10">
-        <v>240</v>
+        <v>39</v>
       </c>
       <c r="F10" t="str">
-        <v>0.48</v>
+        <v>0.34</v>
       </c>
       <c r="G10" t="str">
         <v>↑↑</v>
       </c>
       <c r="H10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J10" t="str">
-        <v>forecast 4 (7d:4 30d:10 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 3 (7d:3 30d:6 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>MELOGRANO</v>
+        <v>PUNCH PARADISE</v>
       </c>
       <c r="B11">
         <v>0</v>
       </c>
       <c r="C11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E11">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="F11" t="str">
-        <v>0.41</v>
+        <v>0.30</v>
       </c>
       <c r="G11" t="str">
         <v>↑↑</v>
@@ -748,12 +748,12 @@
         <v>4</v>
       </c>
       <c r="J11" t="str">
-        <v>forecast 3 (7d:4 30d:5 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 3 (7d:3 30d:3 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ANGURIA</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -762,13 +762,13 @@
         <v>3</v>
       </c>
       <c r="D12">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E12">
         <v>98</v>
       </c>
       <c r="F12" t="str">
-        <v>0.31</v>
+        <v>0.35</v>
       </c>
       <c r="G12" t="str">
         <v>↑↑</v>
@@ -780,187 +780,187 @@
         <v>4</v>
       </c>
       <c r="J12" t="str">
-        <v>forecast 3 (7d:3 30d:4 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 3 (7d:3 30d:7 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>BASILICO</v>
+        <v>PISTACCHIO LARNAKA</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C13">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D13">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="E13">
-        <v>233</v>
+        <v>0</v>
       </c>
       <c r="F13" t="str">
-        <v>0.35</v>
+        <v>0.90</v>
       </c>
       <c r="G13" t="str">
-        <v>↑↑</v>
+        <v>↓</v>
       </c>
       <c r="H13">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J13" t="str">
-        <v>forecast 3 (7d:3 30d:7 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 7 (7d:6 30d:29 trend:↓) +safety 2 -scorta 6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>BIANCANEVE</v>
+        <v>MENTA E C.</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D14">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E14">
-        <v>236</v>
+        <v>298</v>
       </c>
       <c r="F14" t="str">
-        <v>0.36</v>
+        <v>0.49</v>
       </c>
       <c r="G14" t="str">
         <v>↑↑</v>
       </c>
       <c r="H14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J14" t="str">
-        <v>forecast 3 (7d:3 30d:8 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 4 (7d:4 30d:11 trend:↑↑) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>MANGO</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D15">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E15">
-        <v>231</v>
+        <v>286</v>
       </c>
       <c r="F15" t="str">
-        <v>0.35</v>
+        <v>0.53</v>
       </c>
       <c r="G15" t="str">
-        <v>↑↑</v>
+        <v>↑</v>
       </c>
       <c r="H15">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I15">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J15" t="str">
-        <v>forecast 3 (7d:3 30d:7 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 4 (7d:4 30d:14 trend:↑) +safety 2 -scorta 3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>C. AGNESE</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E16">
-        <v>177</v>
+        <v>261</v>
       </c>
       <c r="F16" t="str">
-        <v>0.35</v>
+        <v>0.49</v>
       </c>
       <c r="G16" t="str">
         <v>↑↑</v>
       </c>
       <c r="H16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J16" t="str">
-        <v>forecast 3 (7d:3 30d:7 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 4 (7d:4 30d:11 trend:↑↑) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ESTASI</v>
+        <v>ARACHIDI</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17">
         <v>3</v>
       </c>
       <c r="D17">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E17">
-        <v>138</v>
+        <v>288</v>
       </c>
       <c r="F17" t="str">
-        <v>0.34</v>
+        <v>0.39</v>
       </c>
       <c r="G17" t="str">
-        <v>↑↑</v>
+        <v>↑</v>
       </c>
       <c r="H17">
         <v>4</v>
       </c>
       <c r="I17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J17" t="str">
-        <v>forecast 3 (7d:3 30d:6 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 3 (7d:3 30d:10 trend:↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C18">
         <v>3</v>
       </c>
       <c r="D18">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E18">
-        <v>38</v>
+        <v>285</v>
       </c>
       <c r="F18" t="str">
-        <v>0.34</v>
+        <v>0.38</v>
       </c>
       <c r="G18" t="str">
         <v>↑↑</v>
@@ -969,30 +969,30 @@
         <v>4</v>
       </c>
       <c r="I18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J18" t="str">
-        <v>forecast 3 (7d:3 30d:6 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 3 (7d:3 30d:9 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>MELA M.C.</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E19">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="F19" t="str">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="G19" t="str">
         <v>↑↑</v>
@@ -1001,30 +1001,30 @@
         <v>4</v>
       </c>
       <c r="I19">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J19" t="str">
-        <v>forecast 3 (7d:3 30d:4 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 3 (7d:3 30d:5 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SACRIPANTE</v>
+        <v>BUONGIORNO AMORE</v>
       </c>
       <c r="B20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C20">
         <v>3</v>
       </c>
       <c r="D20">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E20">
-        <v>97</v>
+        <v>153</v>
       </c>
       <c r="F20" t="str">
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="G20" t="str">
         <v>↑↑</v>
@@ -1033,15 +1033,15 @@
         <v>4</v>
       </c>
       <c r="I20">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J20" t="str">
-        <v>forecast 3 (7d:3 30d:6 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 3 (7d:3 30d:8 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>YOGURT</v>
+        <v>V. GIANDUIA VARIEGATA</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -1050,176 +1050,176 @@
         <v>2</v>
       </c>
       <c r="D21">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E21">
-        <v>110</v>
+        <v>72</v>
       </c>
       <c r="F21" t="str">
-        <v>0.29</v>
+        <v>0.20</v>
       </c>
       <c r="G21" t="str">
-        <v>→</v>
+        <v>↑↑</v>
       </c>
       <c r="H21">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I21">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J21" t="str">
-        <v>forecast 3 (7d:2 30d:9 trend:→) +safety 1 -scorta 0</v>
+        <v>forecast 2 (7d:2 30d:2 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>BACIO</v>
+        <v>BASILICO</v>
       </c>
       <c r="B22">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C22">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D22">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="E22">
-        <v>804</v>
+        <v>233</v>
       </c>
       <c r="F22" t="str">
-        <v>1.15</v>
+        <v>0.24</v>
       </c>
       <c r="G22" t="str">
-        <v>↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H22">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="I22">
         <v>3</v>
       </c>
       <c r="J22" t="str">
-        <v>forecast 9 (7d:7 30d:41 trend:↓) +safety 3 -scorta 9</v>
+        <v>forecast 2 (7d:2 30d:5 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>NOCCIOLA</v>
+        <v>MANDORLA TOSTATA</v>
       </c>
       <c r="B23">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C23">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D23">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E23">
-        <v>449</v>
+        <v>26</v>
       </c>
       <c r="F23" t="str">
-        <v>0.70</v>
+        <v>0.22</v>
       </c>
       <c r="G23" t="str">
-        <v>→</v>
+        <v>↑↑</v>
       </c>
       <c r="H23">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I23">
         <v>3</v>
       </c>
       <c r="J23" t="str">
-        <v>forecast 5 (7d:5 30d:20 trend:→) +safety 2 -scorta 4</v>
+        <v>forecast 2 (7d:2 30d:4 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>BANANA E LIME</v>
+        <v>PERA</v>
       </c>
       <c r="B24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C24">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D24">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E24">
-        <v>140</v>
+        <v>39</v>
       </c>
       <c r="F24" t="str">
-        <v>0.39</v>
+        <v>0.28</v>
       </c>
       <c r="G24" t="str">
-        <v>↑</v>
+        <v>→</v>
       </c>
       <c r="H24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I24">
         <v>3</v>
       </c>
       <c r="J24" t="str">
-        <v>forecast 3 (7d:3 30d:10 trend:↑) +safety 1 -scorta 1</v>
+        <v>forecast 2 (7d:2 30d:8 trend:→) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>C. PASTICCIERA PARISI</v>
+        <v>POLLICINA</v>
       </c>
       <c r="B25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D25">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E25">
-        <v>246</v>
+        <v>147</v>
       </c>
       <c r="F25" t="str">
-        <v>0.38</v>
+        <v>0.24</v>
       </c>
       <c r="G25" t="str">
         <v>↑↑</v>
       </c>
       <c r="H25">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I25">
         <v>3</v>
       </c>
       <c r="J25" t="str">
-        <v>forecast 3 (7d:3 30d:9 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 2 (7d:2 30d:5 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>V. GIANDUIA VARIEGATA</v>
+        <v>PENSIERO</v>
       </c>
       <c r="B26">
         <v>0</v>
       </c>
       <c r="C26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E26">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F26" t="str">
-        <v>0.20</v>
+        <v>0.15</v>
       </c>
       <c r="G26" t="str">
-        <v>↑↑</v>
+        <v>↓</v>
       </c>
       <c r="H26">
         <v>3</v>
@@ -1228,30 +1228,30 @@
         <v>3</v>
       </c>
       <c r="J26" t="str">
-        <v>forecast 2 (7d:2 30d:2 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 2 (7d:1 30d:5 trend:↓) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>ROSA E ARANCIA</v>
       </c>
       <c r="B27">
         <v>0</v>
       </c>
       <c r="C27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27">
         <v>5</v>
       </c>
       <c r="E27">
-        <v>102</v>
+        <v>0</v>
       </c>
       <c r="F27" t="str">
-        <v>0.24</v>
+        <v>0.15</v>
       </c>
       <c r="G27" t="str">
-        <v>↑↑</v>
+        <v>↓</v>
       </c>
       <c r="H27">
         <v>3</v>
@@ -1260,123 +1260,123 @@
         <v>3</v>
       </c>
       <c r="J27" t="str">
-        <v>forecast 2 (7d:2 30d:5 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 2 (7d:1 30d:5 trend:↓) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>MELONE</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="B28">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C28">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D28">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E28">
-        <v>121</v>
+        <v>232</v>
       </c>
       <c r="F28" t="str">
-        <v>0.22</v>
+        <v>0.42</v>
       </c>
       <c r="G28" t="str">
         <v>↑↑</v>
       </c>
       <c r="H28">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I28">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J28" t="str">
-        <v>forecast 2 (7d:2 30d:4 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 3 (7d:4 30d:6 trend:↑↑) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>POLLICINA</v>
+        <v>C. E ARANCIA</v>
       </c>
       <c r="B29">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D29">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E29">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="F29" t="str">
-        <v>0.22</v>
+        <v>0.35</v>
       </c>
       <c r="G29" t="str">
         <v>↑↑</v>
       </c>
       <c r="H29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J29" t="str">
-        <v>forecast 2 (7d:2 30d:4 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 3 (7d:3 30d:7 trend:↑↑) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>PUNCH PARADISE</v>
+        <v>CAFFE'</v>
       </c>
       <c r="B30">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C30">
         <v>2</v>
       </c>
       <c r="D30">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E30">
-        <v>45</v>
+        <v>240</v>
       </c>
       <c r="F30" t="str">
-        <v>0.21</v>
+        <v>0.29</v>
       </c>
       <c r="G30" t="str">
-        <v>↑↑</v>
+        <v>→</v>
       </c>
       <c r="H30">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J30" t="str">
-        <v>forecast 2 (7d:2 30d:3 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 3 (7d:2 30d:9 trend:→) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>PENSIERO</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C31">
         <v>2</v>
       </c>
       <c r="D31">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E31">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="F31" t="str">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="G31" t="str">
         <v>↑↑</v>
@@ -1385,18 +1385,18 @@
         <v>3</v>
       </c>
       <c r="I31">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J31" t="str">
-        <v>forecast 2 (7d:2 30d:5 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 2 (7d:2 30d:6 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>BUONGIORNO AMORE</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="B32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C32">
         <v>2</v>
@@ -1405,7 +1405,7 @@
         <v>8</v>
       </c>
       <c r="E32">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F32" t="str">
         <v>0.28</v>
@@ -1417,431 +1417,431 @@
         <v>3</v>
       </c>
       <c r="I32">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J32" t="str">
-        <v>forecast 2 (7d:2 30d:8 trend:→) +safety 1 -scorta 0</v>
+        <v>forecast 2 (7d:2 30d:8 trend:→) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ROSA E ARANCIA</v>
+        <v>YOGURT</v>
       </c>
       <c r="B33">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C33">
         <v>2</v>
       </c>
       <c r="D33">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>111</v>
       </c>
       <c r="F33" t="str">
-        <v>0.25</v>
+        <v>0.29</v>
       </c>
       <c r="G33" t="str">
-        <v>↑↑</v>
+        <v>→</v>
       </c>
       <c r="H33">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I33">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J33" t="str">
-        <v>forecast 2 (7d:2 30d:6 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 3 (7d:2 30d:9 trend:→) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>AVOCADO</v>
+        <v>V. BANACHI</v>
       </c>
       <c r="B34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D34">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E34">
         <v>0</v>
       </c>
       <c r="F34" t="str">
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="G34" t="str">
-        <v>↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H34">
         <v>3</v>
       </c>
       <c r="I34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J34" t="str">
-        <v>forecast 2 (7d:1 30d:5 trend:↓) +safety 1 -scorta 0</v>
+        <v>forecast 2 (7d:2 30d:3 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>LIMONE</v>
+        <v>ESTASI</v>
       </c>
       <c r="B35">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C35">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D35">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="E35">
-        <v>447</v>
+        <v>138</v>
       </c>
       <c r="F35" t="str">
-        <v>0.51</v>
+        <v>0.17</v>
       </c>
       <c r="G35" t="str">
-        <v>↓↓</v>
+        <v>↓</v>
       </c>
       <c r="H35">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I35">
         <v>2</v>
       </c>
       <c r="J35" t="str">
-        <v>forecast 4 (7d:3 30d:19 trend:↓↓) +safety 2 -scorta 4</v>
+        <v>forecast 2 (7d:1 30d:6 trend:↓) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C36">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D36">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E36">
-        <v>284</v>
+        <v>54</v>
       </c>
       <c r="F36" t="str">
-        <v>0.39</v>
+        <v>0.18</v>
       </c>
       <c r="G36" t="str">
-        <v>↑</v>
+        <v>↓↓</v>
       </c>
       <c r="H36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I36">
         <v>2</v>
       </c>
       <c r="J36" t="str">
-        <v>forecast 3 (7d:3 30d:10 trend:↑) +safety 1 -scorta 2</v>
+        <v>forecast 2 (7d:1 30d:7 trend:↓↓) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>TIRAMISU'</v>
+        <v>C. KENTUCKY</v>
       </c>
       <c r="B37">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C37">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D37">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E37">
-        <v>259</v>
+        <v>86</v>
       </c>
       <c r="F37" t="str">
-        <v>0.38</v>
+        <v>0.14</v>
       </c>
       <c r="G37" t="str">
-        <v>↑↑</v>
+        <v>→</v>
       </c>
       <c r="H37">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I37">
         <v>2</v>
       </c>
       <c r="J37" t="str">
-        <v>forecast 3 (7d:3 30d:9 trend:↑↑) +safety 1 -scorta 2</v>
+        <v>forecast 1 (7d:1 30d:4 trend:→) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>C. FRAGOLE E MANDORLE</v>
+        <v>PANACEA</v>
       </c>
       <c r="B38">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C38">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E38">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="F38" t="str">
-        <v>0.26</v>
+        <v>0.13</v>
       </c>
       <c r="G38" t="str">
-        <v>↑</v>
+        <v>↑↑</v>
       </c>
       <c r="H38">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I38">
         <v>2</v>
       </c>
       <c r="J38" t="str">
-        <v>forecast 2 (7d:2 30d:7 trend:↑) +safety 1 -scorta 1</v>
+        <v>forecast 1 (7d:1 30d:3 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>AVOCADO</v>
       </c>
       <c r="B39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C39">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D39">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E39">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="F39" t="str">
-        <v>0.25</v>
+        <v>0.14</v>
       </c>
       <c r="G39" t="str">
-        <v>↑↑</v>
+        <v>→</v>
       </c>
       <c r="H39">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I39">
         <v>2</v>
       </c>
       <c r="J39" t="str">
-        <v>forecast 2 (7d:2 30d:6 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 1 (7d:1 30d:4 trend:→) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>PERA</v>
+        <v>C. PASTICCIERA PARISI</v>
       </c>
       <c r="B40">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C40">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D40">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E40">
-        <v>38</v>
+        <v>248</v>
       </c>
       <c r="F40" t="str">
-        <v>0.28</v>
+        <v>0.49</v>
       </c>
       <c r="G40" t="str">
-        <v>→</v>
+        <v>↑↑</v>
       </c>
       <c r="H40">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J40" t="str">
-        <v>forecast 2 (7d:2 30d:8 trend:→) +safety 1 -scorta 1</v>
+        <v>forecast 4 (7d:4 30d:11 trend:↑↑) +safety 1 -scorta 4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>V. CASTAGNA E MIRTO</v>
+        <v>MELONE</v>
       </c>
       <c r="B41">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C41">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D41">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E41">
-        <v>34</v>
+        <v>122</v>
       </c>
       <c r="F41" t="str">
-        <v>0.13</v>
+        <v>0.32</v>
       </c>
       <c r="G41" t="str">
         <v>↑↑</v>
       </c>
       <c r="H41">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J41" t="str">
-        <v>forecast 1 (7d:1 30d:3 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 3 (7d:3 30d:5 trend:↑↑) +safety 1 -scorta 3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>MORA</v>
+        <v>C. CANNELLA</v>
       </c>
       <c r="B42">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D42">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E42">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="F42" t="str">
-        <v>0.11</v>
+        <v>0.22</v>
       </c>
       <c r="G42" t="str">
         <v>↑↑</v>
       </c>
       <c r="H42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I42">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J42" t="str">
-        <v>forecast 1 (7d:1 30d:2 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 2 (7d:2 30d:4 trend:↑↑) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>V. BANACHI</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B43">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D43">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E43">
-        <v>0</v>
+        <v>103</v>
       </c>
       <c r="F43" t="str">
-        <v>0.11</v>
+        <v>0.24</v>
       </c>
       <c r="G43" t="str">
         <v>↑↑</v>
       </c>
       <c r="H43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J43" t="str">
-        <v>forecast 1 (7d:1 30d:2 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 2 (7d:2 30d:5 trend:↑↑) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B44">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C44">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D44">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E44">
-        <v>174</v>
+        <v>55</v>
       </c>
       <c r="F44" t="str">
-        <v>0.52</v>
+        <v>0.14</v>
       </c>
       <c r="G44" t="str">
-        <v>↑↑</v>
+        <v>→</v>
       </c>
       <c r="H44">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I44">
         <v>1</v>
       </c>
       <c r="J44" t="str">
-        <v>forecast 4 (7d:5 30d:7 trend:↑↑) +safety 2 -scorta 5</v>
+        <v>forecast 1 (7d:1 30d:4 trend:→) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>MORA</v>
       </c>
       <c r="B45">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C45">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D45">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E45">
-        <v>139</v>
+        <v>11</v>
       </c>
       <c r="F45" t="str">
-        <v>0.28</v>
+        <v>0.11</v>
       </c>
       <c r="G45" t="str">
-        <v>→</v>
+        <v>↑↑</v>
       </c>
       <c r="H45">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I45">
         <v>1</v>
       </c>
       <c r="J45" t="str">
-        <v>forecast 2 (7d:2 30d:8 trend:→) +safety 1 -scorta 2</v>
+        <v>forecast 1 (7d:1 30d:2 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>C. KENTUCKY</v>
+        <v>V. NOCCIOLA F.</v>
       </c>
       <c r="B46">
         <v>1</v>
@@ -1853,7 +1853,7 @@
         <v>3</v>
       </c>
       <c r="E46">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="F46" t="str">
         <v>0.13</v>
@@ -1873,7 +1873,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>MANDORLA TOSTATA</v>
+        <v>PEREBH</v>
       </c>
       <c r="B47">
         <v>1</v>
@@ -1882,13 +1882,13 @@
         <v>1</v>
       </c>
       <c r="D47">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E47">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="F47" t="str">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="G47" t="str">
         <v>↑↑</v>
@@ -1900,12 +1900,12 @@
         <v>1</v>
       </c>
       <c r="J47" t="str">
-        <v>forecast 1 (7d:1 30d:3 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 1 (7d:1 30d:2 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>V. NOCCIOLA F.</v>
+        <v>STRACCHINO PERA</v>
       </c>
       <c r="B48">
         <v>1</v>
@@ -1914,16 +1914,16 @@
         <v>1</v>
       </c>
       <c r="D48">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E48">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="F48" t="str">
-        <v>0.14</v>
+        <v>0.11</v>
       </c>
       <c r="G48" t="str">
-        <v>→</v>
+        <v>↑↑</v>
       </c>
       <c r="H48">
         <v>2</v>
@@ -1932,12 +1932,12 @@
         <v>1</v>
       </c>
       <c r="J48" t="str">
-        <v>forecast 1 (7d:1 30d:4 trend:→) +safety 1 -scorta 1</v>
+        <v>forecast 1 (7d:1 30d:2 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>PANACEA</v>
+        <v>NOCCIOLA BURRO</v>
       </c>
       <c r="B49">
         <v>1</v>
@@ -1946,13 +1946,13 @@
         <v>1</v>
       </c>
       <c r="D49">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E49">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="F49" t="str">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="G49" t="str">
         <v>↑↑</v>
@@ -1964,12 +1964,12 @@
         <v>1</v>
       </c>
       <c r="J49" t="str">
-        <v>forecast 1 (7d:1 30d:2 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 1 (7d:1 30d:3 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>PASSION FRUIT</v>
+        <v>COCONUT RICE CAKE</v>
       </c>
       <c r="B50">
         <v>1</v>
@@ -1978,16 +1978,16 @@
         <v>1</v>
       </c>
       <c r="D50">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E50">
-        <v>169</v>
+        <v>0</v>
       </c>
       <c r="F50" t="str">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="G50" t="str">
-        <v>↑↑</v>
+        <v>→</v>
       </c>
       <c r="H50">
         <v>2</v>
@@ -1996,62 +1996,62 @@
         <v>1</v>
       </c>
       <c r="J50" t="str">
-        <v>forecast 1 (7d:1 30d:3 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 1 (7d:1 30d:4 trend:→) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>V. CASTAGNA E MIRTO</v>
       </c>
       <c r="B51">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C51">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D51">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E51">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="F51" t="str">
-        <v>0.18</v>
+        <v>0.04</v>
       </c>
       <c r="G51" t="str">
         <v>↓↓</v>
       </c>
       <c r="H51">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I51">
         <v>1</v>
       </c>
       <c r="J51" t="str">
-        <v>forecast 2 (7d:1 30d:7 trend:↓↓) +safety 1 -scorta 2</v>
+        <v>venduto nel mese (3 vasche), assente questa settimana — ordine minimo</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>VENERE ROSA</v>
+        <v>C. CRUDO DEL PERU'</v>
       </c>
       <c r="B52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D52">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E52">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="F52" t="str">
-        <v>0.11</v>
+        <v>0.07</v>
       </c>
       <c r="G52" t="str">
-        <v>↑↑</v>
+        <v>↓↓</v>
       </c>
       <c r="H52">
         <v>2</v>
@@ -2060,30 +2060,30 @@
         <v>1</v>
       </c>
       <c r="J52" t="str">
-        <v>forecast 1 (7d:1 30d:2 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>venduto nel mese (5 vasche), assente questa settimana — ordine minimo</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>COCONUT RICE CAKE</v>
+        <v>C. ROSEMARY</v>
       </c>
       <c r="B53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D53">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E53">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F53" t="str">
-        <v>0.14</v>
+        <v>0.01</v>
       </c>
       <c r="G53" t="str">
-        <v>→</v>
+        <v>↓↓</v>
       </c>
       <c r="H53">
         <v>2</v>
@@ -2092,44 +2092,44 @@
         <v>1</v>
       </c>
       <c r="J53" t="str">
-        <v>forecast 1 (7d:1 30d:4 trend:→) +safety 1 -scorta 1</v>
+        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ZABAIONE GELATO</v>
+        <v>C. WASABI</v>
       </c>
       <c r="B54">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C54">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D54">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E54">
-        <v>127</v>
+        <v>5</v>
       </c>
       <c r="F54" t="str">
-        <v>0.17</v>
+        <v>0.01</v>
       </c>
       <c r="G54" t="str">
-        <v>↓</v>
+        <v>↓↓</v>
       </c>
       <c r="H54">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I54">
         <v>1</v>
       </c>
       <c r="J54" t="str">
-        <v>forecast 2 (7d:1 30d:6 trend:↓) +safety 1 -scorta 2</v>
+        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>C. CRUDO DEL PERU'</v>
+        <v>V. FIOR DI CIOCCOLATO</v>
       </c>
       <c r="B55">
         <v>0</v>
@@ -2138,13 +2138,13 @@
         <v>0</v>
       </c>
       <c r="D55">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E55">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="F55" t="str">
-        <v>0.07</v>
+        <v>0.01</v>
       </c>
       <c r="G55" t="str">
         <v>↓↓</v>
@@ -2156,12 +2156,12 @@
         <v>1</v>
       </c>
       <c r="J55" t="str">
-        <v>venduto nel mese (5 vasche), assente questa settimana — ordine minimo</v>
+        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>C. ROSEMARY</v>
+        <v>V. CASTAGNA AL WHISKY</v>
       </c>
       <c r="B56">
         <v>0</v>
@@ -2173,7 +2173,7 @@
         <v>1</v>
       </c>
       <c r="E56">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F56" t="str">
         <v>0.01</v>
@@ -2193,7 +2193,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>PAPAYA</v>
+        <v>STRACCHINO ALBICOCCHA</v>
       </c>
       <c r="B57">
         <v>0</v>
@@ -2202,13 +2202,13 @@
         <v>0</v>
       </c>
       <c r="D57">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E57">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="F57" t="str">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="G57" t="str">
         <v>↓↓</v>
@@ -2220,126 +2220,126 @@
         <v>1</v>
       </c>
       <c r="J57" t="str">
-        <v>venduto nel mese (2 vasche), assente questa settimana — ordine minimo</v>
+        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>V. FIOR DI CIOCCOLATO</v>
+        <v>FRAGOLA</v>
       </c>
       <c r="B58">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C58">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D58">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="E58">
-        <v>0</v>
+        <v>516</v>
       </c>
       <c r="F58" t="str">
-        <v>0.01</v>
+        <v>0.95</v>
       </c>
       <c r="G58" t="str">
-        <v>↓↓</v>
+        <v>↑</v>
       </c>
       <c r="H58">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I58">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J58" t="str">
-        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
+        <v>scorta (9) copre forecast 7+safety 2 [trend ↑]</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>V. CASTAGNA AL WHISKY</v>
+        <v>BANANA E LIME</v>
       </c>
       <c r="B59">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C59">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D59">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E59">
-        <v>0</v>
+        <v>141</v>
       </c>
       <c r="F59" t="str">
-        <v>0.01</v>
+        <v>0.38</v>
       </c>
       <c r="G59" t="str">
-        <v>↓↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H59">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I59">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J59" t="str">
-        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
+        <v>scorta (4) copre forecast 3+safety 1 [trend ↑↑]</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>STRACCHINO ALBICOCCHA</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="B60">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C60">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D60">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E60">
-        <v>0</v>
+        <v>237</v>
       </c>
       <c r="F60" t="str">
-        <v>0.01</v>
+        <v>0.36</v>
       </c>
       <c r="G60" t="str">
-        <v>↓↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H60">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I60">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J60" t="str">
-        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
+        <v>scorta (4) copre forecast 3+safety 1 [trend ↑↑]</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>FRUTTI DI BOSCO</v>
+        <v>C. AGNESE</v>
       </c>
       <c r="B61">
         <v>4</v>
       </c>
       <c r="C61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D61">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E61">
-        <v>125</v>
+        <v>178</v>
       </c>
       <c r="F61" t="str">
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="G61" t="str">
-        <v>↓↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H61">
         <v>4</v>
@@ -2348,94 +2348,94 @@
         <v>0</v>
       </c>
       <c r="J61" t="str">
-        <v>scorta (4) copre forecast 3+safety 1 [trend ↓↓]</v>
+        <v>scorta (4) copre forecast 3+safety 1 [trend ↑↑]</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>C. UGANDA</v>
+        <v>LIMONE</v>
       </c>
       <c r="B62">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D62">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E62">
-        <v>0</v>
+        <v>449</v>
       </c>
       <c r="F62" t="str">
-        <v>0.20</v>
+        <v>0.51</v>
       </c>
       <c r="G62" t="str">
-        <v>↑↑</v>
+        <v>↓↓</v>
       </c>
       <c r="H62">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I62">
         <v>0</v>
       </c>
       <c r="J62" t="str">
-        <v>scorta (5) copre forecast 2+safety 1 [trend ↑↑]</v>
+        <v>scorta (6) copre forecast 4+safety 2 [trend ↓↓]</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>ANANAS</v>
+        <v>MELA M.C.</v>
       </c>
       <c r="B63">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C63">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D63">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E63">
-        <v>134</v>
+        <v>166</v>
       </c>
       <c r="F63" t="str">
-        <v>0.18</v>
+        <v>0.32</v>
       </c>
       <c r="G63" t="str">
-        <v>↓↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H63">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I63">
         <v>0</v>
       </c>
       <c r="J63" t="str">
-        <v>scorta (3) copre forecast 2+safety 1 [trend ↓↓]</v>
+        <v>scorta (4) copre forecast 3+safety 1 [trend ↑↑]</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>C. E ARANCIA</v>
+        <v>ANGURIA</v>
       </c>
       <c r="B64">
         <v>4</v>
       </c>
       <c r="C64">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D64">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E64">
-        <v>154</v>
+        <v>98</v>
       </c>
       <c r="F64" t="str">
-        <v>0.17</v>
+        <v>0.21</v>
       </c>
       <c r="G64" t="str">
-        <v>↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H64">
         <v>3</v>
@@ -2444,94 +2444,94 @@
         <v>0</v>
       </c>
       <c r="J64" t="str">
-        <v>scorta (4) copre forecast 2+safety 1 [trend ↓]</v>
+        <v>scorta (4) copre forecast 2+safety 1 [trend ↑↑]</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>C. LAPSANG SOUCHOUNG</v>
+        <v>C. MADAGASCAR</v>
       </c>
       <c r="B65">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C65">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D65">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E65">
-        <v>5</v>
+        <v>303</v>
       </c>
       <c r="F65" t="str">
-        <v>0.10</v>
+        <v>0.26</v>
       </c>
       <c r="G65" t="str">
-        <v>↑↑</v>
+        <v>↑</v>
       </c>
       <c r="H65">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I65">
         <v>0</v>
       </c>
       <c r="J65" t="str">
-        <v>scorta (2) copre forecast 1+safety 1 [trend ↑↑]</v>
+        <v>scorta (3) copre forecast 2+safety 1 [trend ↑]</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>C. CANNELLA</v>
+        <v>COCCO C.</v>
       </c>
       <c r="B66">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C66">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D66">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E66">
-        <v>32</v>
+        <v>253</v>
       </c>
       <c r="F66" t="str">
-        <v>0.13</v>
+        <v>0.30</v>
       </c>
       <c r="G66" t="str">
-        <v>↑↑</v>
+        <v>↓</v>
       </c>
       <c r="H66">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I66">
         <v>0</v>
       </c>
       <c r="J66" t="str">
-        <v>scorta (2) copre forecast 1+safety 1 [trend ↑↑]</v>
+        <v>scorta (4) copre forecast 3+safety 1 [trend ↓]</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>MENTA E C.</v>
+        <v>C. FRAGOLE E MANDORLE</v>
       </c>
       <c r="B67">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C67">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D67">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E67">
-        <v>295</v>
+        <v>155</v>
       </c>
       <c r="F67" t="str">
-        <v>0.21</v>
+        <v>0.26</v>
       </c>
       <c r="G67" t="str">
-        <v>↓↓</v>
+        <v>↑</v>
       </c>
       <c r="H67">
         <v>3</v>
@@ -2540,30 +2540,30 @@
         <v>0</v>
       </c>
       <c r="J67" t="str">
-        <v>scorta (4) copre forecast 2+safety 1 [trend ↓↓]</v>
+        <v>scorta (3) copre forecast 2+safety 1 [trend ↑]</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>MELOGRANO</v>
       </c>
       <c r="B68">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C68">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D68">
         <v>5</v>
       </c>
       <c r="E68">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="F68" t="str">
-        <v>0.15</v>
+        <v>0.24</v>
       </c>
       <c r="G68" t="str">
-        <v>↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H68">
         <v>3</v>
@@ -2572,44 +2572,44 @@
         <v>0</v>
       </c>
       <c r="J68" t="str">
-        <v>scorta (3) copre forecast 2+safety 1 [trend ↓]</v>
+        <v>scorta (4) copre forecast 2+safety 1 [trend ↑↑]</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>SEADAS</v>
+        <v>C. UGANDA</v>
       </c>
       <c r="B69">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C69">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D69">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E69">
-        <v>102</v>
+        <v>0</v>
       </c>
       <c r="F69" t="str">
-        <v>0.14</v>
+        <v>0.21</v>
       </c>
       <c r="G69" t="str">
-        <v>→</v>
+        <v>↑↑</v>
       </c>
       <c r="H69">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I69">
         <v>0</v>
       </c>
       <c r="J69" t="str">
-        <v>scorta (2) copre forecast 1+safety 1 [trend →]</v>
+        <v>scorta (4) copre forecast 2+safety 1 [trend ↑↑]</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>UVA E NOCI</v>
+        <v>C. LAPSANG SOUCHOUNG</v>
       </c>
       <c r="B70">
         <v>2</v>
@@ -2618,13 +2618,13 @@
         <v>1</v>
       </c>
       <c r="D70">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E70">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="F70" t="str">
-        <v>0.11</v>
+        <v>0.10</v>
       </c>
       <c r="G70" t="str">
         <v>↑↑</v>
@@ -2641,57 +2641,57 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>SEADAS</v>
       </c>
       <c r="B71">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C71">
         <v>1</v>
       </c>
       <c r="D71">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E71">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="F71" t="str">
-        <v>0.19</v>
+        <v>0.13</v>
       </c>
       <c r="G71" t="str">
-        <v>↓↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H71">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I71">
         <v>0</v>
       </c>
       <c r="J71" t="str">
-        <v>scorta (3) copre forecast 2+safety 1 [trend ↓↓]</v>
+        <v>scorta (2) copre forecast 1+safety 1 [trend ↑↑]</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>AMARENA</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B72">
         <v>2</v>
       </c>
       <c r="C72">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D72">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E72">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F72" t="str">
-        <v>0.08</v>
+        <v>0.10</v>
       </c>
       <c r="G72" t="str">
-        <v>↓↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H72">
         <v>2</v>
@@ -2700,91 +2700,91 @@
         <v>0</v>
       </c>
       <c r="J72" t="str">
-        <v>nessuna vendita 7gg (30gg: 6, scorta: 2)</v>
+        <v>scorta (2) copre forecast 1+safety 1 [trend ↑↑]</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>C. AL PIMENTO</v>
+        <v>VENERE ROSA</v>
       </c>
       <c r="B73">
         <v>2</v>
       </c>
       <c r="C73">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D73">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E73">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F73" t="str">
-        <v>0.00</v>
+        <v>0.11</v>
       </c>
       <c r="G73" t="str">
-        <v>→</v>
+        <v>↑↑</v>
       </c>
       <c r="H73">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I73">
         <v>0</v>
       </c>
       <c r="J73" t="str">
-        <v>nessuna vendita 30gg</v>
+        <v>scorta (2) copre forecast 1+safety 1 [trend ↑↑]</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>C. BIANCO</v>
+        <v>AMARENA</v>
       </c>
       <c r="B74">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C74">
         <v>0</v>
       </c>
       <c r="D74">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E74">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="F74" t="str">
-        <v>0.00</v>
+        <v>0.08</v>
       </c>
       <c r="G74" t="str">
-        <v>→</v>
+        <v>↓↓</v>
       </c>
       <c r="H74">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I74">
         <v>0</v>
       </c>
       <c r="J74" t="str">
-        <v>nessuna vendita 30gg</v>
+        <v>nessuna vendita 7gg (30gg: 6, scorta: 2)</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>C. MADAGASCAR</v>
+        <v>ANANAS</v>
       </c>
       <c r="B75">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C75">
         <v>0</v>
       </c>
       <c r="D75">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E75">
-        <v>301</v>
+        <v>134</v>
       </c>
       <c r="F75" t="str">
-        <v>0.11</v>
+        <v>0.08</v>
       </c>
       <c r="G75" t="str">
         <v>↓↓</v>
@@ -2796,111 +2796,111 @@
         <v>0</v>
       </c>
       <c r="J75" t="str">
-        <v>nessuna vendita 7gg (30gg: 8, scorta: 5)</v>
+        <v>nessuna vendita 7gg (30gg: 6, scorta: 2)</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>COCCO C.</v>
+        <v>C. AL PIMENTO</v>
       </c>
       <c r="B76">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C76">
         <v>0</v>
       </c>
       <c r="D76">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E76">
-        <v>251</v>
+        <v>3</v>
       </c>
       <c r="F76" t="str">
-        <v>0.11</v>
+        <v>0.00</v>
       </c>
       <c r="G76" t="str">
-        <v>↓↓</v>
+        <v>→</v>
       </c>
       <c r="H76">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I76">
         <v>0</v>
       </c>
       <c r="J76" t="str">
-        <v>nessuna vendita 7gg (30gg: 8, scorta: 5)</v>
+        <v>nessuna vendita 30gg</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>C. VANIGLIA</v>
+        <v>C. BIANCO</v>
       </c>
       <c r="B77">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C77">
         <v>0</v>
       </c>
       <c r="D77">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E77">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="F77" t="str">
-        <v>0.01</v>
+        <v>0.00</v>
       </c>
       <c r="G77" t="str">
-        <v>↓↓</v>
+        <v>→</v>
       </c>
       <c r="H77">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I77">
         <v>0</v>
       </c>
       <c r="J77" t="str">
-        <v>nessuna vendita 7gg (30gg: 1, scorta: 2)</v>
+        <v>nessuna vendita 30gg</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>C. ZENZERO</v>
+        <v>C. VANIGLIA</v>
       </c>
       <c r="B78">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C78">
         <v>0</v>
       </c>
       <c r="D78">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E78">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F78" t="str">
-        <v>0.04</v>
+        <v>0.00</v>
       </c>
       <c r="G78" t="str">
-        <v>↓↓</v>
+        <v>→</v>
       </c>
       <c r="H78">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I78">
         <v>0</v>
       </c>
       <c r="J78" t="str">
-        <v>nessuna vendita 7gg (30gg: 3, scorta: 3)</v>
+        <v>nessuna vendita 30gg</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>GIANDUIA</v>
+        <v>C. ZENZERO</v>
       </c>
       <c r="B79">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C79">
         <v>0</v>
@@ -2909,7 +2909,7 @@
         <v>3</v>
       </c>
       <c r="E79">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="F79" t="str">
         <v>0.04</v>
@@ -2924,47 +2924,47 @@
         <v>0</v>
       </c>
       <c r="J79" t="str">
-        <v>nessuna vendita 7gg (30gg: 3, scorta: 1)</v>
+        <v>nessuna vendita 7gg (30gg: 3, scorta: 3)</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>LEMON CURD</v>
+        <v>FRUTTI DI BOSCO</v>
       </c>
       <c r="B80">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C80">
         <v>0</v>
       </c>
       <c r="D80">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E80">
-        <v>26</v>
+        <v>125</v>
       </c>
       <c r="F80" t="str">
-        <v>0.04</v>
+        <v>0.16</v>
       </c>
       <c r="G80" t="str">
         <v>↓↓</v>
       </c>
       <c r="H80">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I80">
         <v>0</v>
       </c>
       <c r="J80" t="str">
-        <v>nessuna vendita 7gg (30gg: 3, scorta: 1)</v>
+        <v>nessuna vendita 7gg (30gg: 12, scorta: 6)</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>LIQUIRIZIA</v>
+        <v>GIANDUIA</v>
       </c>
       <c r="B81">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C81">
         <v>0</v>
@@ -2973,7 +2973,7 @@
         <v>3</v>
       </c>
       <c r="E81">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="F81" t="str">
         <v>0.04</v>
@@ -2988,39 +2988,39 @@
         <v>0</v>
       </c>
       <c r="J81" t="str">
-        <v>nessuna vendita 7gg (30gg: 3, scorta: 2)</v>
+        <v>nessuna vendita 7gg (30gg: 3, scorta: 1)</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>MANGO</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="B82">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C82">
         <v>0</v>
       </c>
       <c r="D82">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E82">
-        <v>282</v>
+        <v>26</v>
       </c>
       <c r="F82" t="str">
-        <v>0.16</v>
+        <v>0.03</v>
       </c>
       <c r="G82" t="str">
         <v>↓↓</v>
       </c>
       <c r="H82">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I82">
         <v>0</v>
       </c>
       <c r="J82" t="str">
-        <v>nessuna vendita 7gg (30gg: 12, scorta: 6)</v>
+        <v>nessuna vendita 7gg (30gg: 2, scorta: 1)</v>
       </c>
     </row>
     <row r="83">
@@ -3057,10 +3057,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>PEREBH</v>
+        <v>PAPAYA</v>
       </c>
       <c r="B84">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C84">
         <v>0</v>
@@ -3069,7 +3069,7 @@
         <v>2</v>
       </c>
       <c r="E84">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="F84" t="str">
         <v>0.03</v>
@@ -3084,27 +3084,27 @@
         <v>0</v>
       </c>
       <c r="J84" t="str">
-        <v>nessuna vendita 7gg (30gg: 2, scorta: 2)</v>
+        <v>nessuna vendita 7gg (30gg: 2, scorta: 1)</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>RICOTTA E COCCO</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="B85">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C85">
         <v>0</v>
       </c>
       <c r="D85">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E85">
-        <v>17</v>
+        <v>83</v>
       </c>
       <c r="F85" t="str">
-        <v>0.04</v>
+        <v>0.07</v>
       </c>
       <c r="G85" t="str">
         <v>↓↓</v>
@@ -3116,27 +3116,27 @@
         <v>0</v>
       </c>
       <c r="J85" t="str">
-        <v>nessuna vendita 7gg (30gg: 3, scorta: 2)</v>
+        <v>nessuna vendita 7gg (30gg: 5, scorta: 3)</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>C. WASABI</v>
+        <v>RICOTTA E COCCO</v>
       </c>
       <c r="B86">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C86">
         <v>0</v>
       </c>
       <c r="D86">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E86">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="F86" t="str">
-        <v>0.01</v>
+        <v>0.04</v>
       </c>
       <c r="G86" t="str">
         <v>↓↓</v>
@@ -3148,7 +3148,7 @@
         <v>0</v>
       </c>
       <c r="J86" t="str">
-        <v>nessuna vendita 7gg (30gg: 1, scorta: 1)</v>
+        <v>nessuna vendita 7gg (30gg: 3, scorta: 2)</v>
       </c>
     </row>
     <row r="87">
@@ -3185,22 +3185,22 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>CARROT CAKE</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B88">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C88">
         <v>0</v>
       </c>
       <c r="D88">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E88">
         <v>0</v>
       </c>
       <c r="F88" t="str">
-        <v>0.01</v>
+        <v>0.08</v>
       </c>
       <c r="G88" t="str">
         <v>↓↓</v>
@@ -3212,59 +3212,59 @@
         <v>0</v>
       </c>
       <c r="J88" t="str">
-        <v>nessuna vendita 7gg (30gg: 1, scorta: 2)</v>
+        <v>nessuna vendita 7gg (30gg: 6, scorta: 3)</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>STRACCHINO PERA</v>
+        <v>CARROT CAKE</v>
       </c>
       <c r="B89">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C89">
         <v>0</v>
       </c>
       <c r="D89">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E89">
         <v>0</v>
       </c>
       <c r="F89" t="str">
-        <v>0.01</v>
+        <v>0.00</v>
       </c>
       <c r="G89" t="str">
-        <v>↓↓</v>
+        <v>→</v>
       </c>
       <c r="H89">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I89">
         <v>0</v>
       </c>
       <c r="J89" t="str">
-        <v>nessuna vendita 7gg (30gg: 1, scorta: 3)</v>
+        <v>nessuna vendita 30gg</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>NOCCIOLA BURRO</v>
+        <v>RICOTTA E PERA</v>
       </c>
       <c r="B90">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C90">
         <v>0</v>
       </c>
       <c r="D90">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E90">
         <v>0</v>
       </c>
       <c r="F90" t="str">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="G90" t="str">
         <v>↓↓</v>
@@ -3276,12 +3276,12 @@
         <v>0</v>
       </c>
       <c r="J90" t="str">
-        <v>nessuna vendita 7gg (30gg: 2, scorta: 2)</v>
+        <v>nessuna vendita 7gg (30gg: 3, scorta: 1)</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>RICOTTA E PERA</v>
+        <v>V.BRONTE GREEN</v>
       </c>
       <c r="B91">
         <v>1</v>
@@ -3290,13 +3290,13 @@
         <v>0</v>
       </c>
       <c r="D91">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E91">
         <v>0</v>
       </c>
       <c r="F91" t="str">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="G91" t="str">
         <v>↓↓</v>
@@ -3308,15 +3308,15 @@
         <v>0</v>
       </c>
       <c r="J91" t="str">
-        <v>nessuna vendita 7gg (30gg: 3, scorta: 1)</v>
+        <v>nessuna vendita 7gg (30gg: 2, scorta: 1)</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>V.BRONTE GREEN</v>
+        <v>SACHER TORTE</v>
       </c>
       <c r="B92">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C92">
         <v>0</v>
@@ -3340,27 +3340,27 @@
         <v>0</v>
       </c>
       <c r="J92" t="str">
-        <v>nessuna vendita 7gg (30gg: 2, scorta: 1)</v>
+        <v>nessuna vendita 7gg (30gg: 2, scorta: 2)</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>SACHER TORTE</v>
+        <v>ZABAIONE GELATO</v>
       </c>
       <c r="B93">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C93">
         <v>0</v>
       </c>
       <c r="D93">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E93">
-        <v>0</v>
+        <v>127</v>
       </c>
       <c r="F93" t="str">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="G93" t="str">
         <v>↓↓</v>
@@ -3372,7 +3372,7 @@
         <v>0</v>
       </c>
       <c r="J93" t="str">
-        <v>nessuna vendita 7gg (30gg: 3, scorta: 1)</v>
+        <v>nessuna vendita 7gg (30gg: 4, scorta: 3)</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update output artifacts and add logo
Regenerated order PDF and Excel files reflecting latest ordering logic
fixes (missing flavors, lean safety stock). Added logo.png for the app.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/shocapp_da_ordinare.xlsx
+++ b/output/shocapp_da_ordinare.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J93"/>
+  <dimension ref="A1:J99"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -433,199 +433,199 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>NOCCIOLA</v>
+        <v>STRACCIATELLA</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D2">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="E2">
-        <v>454</v>
+        <v>812</v>
       </c>
       <c r="F2" t="str">
-        <v>1.06</v>
+        <v>1.54</v>
       </c>
       <c r="G2" t="str">
-        <v>↑↑</v>
+        <v>→</v>
       </c>
       <c r="H2">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J2" t="str">
-        <v>forecast 8 (7d:9 30d:22 trend:↑↑) +safety 3 -scorta 3</v>
+        <v>forecast 11 (7d:11 30d:45 trend:→) +safety 4 -scorta 9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>C. AL LATTE GELATO</v>
+        <v>NOCCIOLA</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D3">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E3">
-        <v>364</v>
+        <v>454</v>
       </c>
       <c r="F3" t="str">
-        <v>0.63</v>
+        <v>0.98</v>
       </c>
       <c r="G3" t="str">
         <v>↑↑</v>
       </c>
       <c r="H3">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J3" t="str">
-        <v>forecast 5 (7d:5 30d:15 trend:↑↑) +safety 2 -scorta 0</v>
+        <v>forecast 7 (7d:8 30d:22 trend:↑↑) +safety 2 -scorta 3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>P.BRONTE</v>
+        <v>C. AL LATTE GELATO</v>
       </c>
       <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4">
+        <v>14</v>
+      </c>
+      <c r="E4">
+        <v>364</v>
+      </c>
+      <c r="F4" t="str">
+        <v>0.53</v>
+      </c>
+      <c r="G4" t="str">
+        <v>↑</v>
+      </c>
+      <c r="H4">
         <v>6</v>
       </c>
-      <c r="C4">
-        <v>9</v>
-      </c>
-      <c r="D4">
-        <v>24</v>
-      </c>
-      <c r="E4">
-        <v>768</v>
-      </c>
-      <c r="F4" t="str">
-        <v>1.09</v>
-      </c>
-      <c r="G4" t="str">
-        <v>↑↑</v>
-      </c>
-      <c r="H4">
-        <v>11</v>
-      </c>
       <c r="I4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J4" t="str">
-        <v>forecast 8 (7d:9 30d:24 trend:↑↑) +safety 3 -scorta 6</v>
+        <v>forecast 4 (7d:4 30d:14 trend:↑) +safety 2 -scorta 0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>STRACCIATELLA</v>
+        <v>BACIO</v>
       </c>
       <c r="B5">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C5">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D5">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E5">
         <v>810</v>
       </c>
       <c r="F5" t="str">
-        <v>1.53</v>
+        <v>1.39</v>
       </c>
       <c r="G5" t="str">
         <v>→</v>
       </c>
       <c r="H5">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J5" t="str">
-        <v>forecast 11 (7d:11 30d:44 trend:→) +safety 4 -scorta 11</v>
+        <v>forecast 10 (7d:10 30d:40 trend:→) +safety 3 -scorta 8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BACIO</v>
+        <v>P.BRONTE</v>
       </c>
       <c r="B6">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D6">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="E6">
-        <v>809</v>
+        <v>768</v>
       </c>
       <c r="F6" t="str">
-        <v>1.39</v>
+        <v>1.01</v>
       </c>
       <c r="G6" t="str">
-        <v>→</v>
+        <v>↑↑</v>
       </c>
       <c r="H6">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J6" t="str">
-        <v>forecast 10 (7d:10 30d:40 trend:→) +safety 3 -scorta 9</v>
+        <v>forecast 8 (7d:8 30d:24 trend:↑↑) +safety 3 -scorta 6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>FIORDILATTE</v>
+        <v>LAMPONI SORBETTO</v>
       </c>
       <c r="B7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="E7">
-        <v>352</v>
+        <v>177</v>
       </c>
       <c r="F7" t="str">
-        <v>0.78</v>
+        <v>0.71</v>
       </c>
       <c r="G7" t="str">
-        <v>↑</v>
+        <v>↑↑</v>
       </c>
       <c r="H7">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J7" t="str">
-        <v>forecast 6 (7d:6 30d:20 trend:↑) +safety 2 -scorta 4</v>
+        <v>forecast 5 (7d:7 30d:8 trend:↑↑) +safety 2 -scorta 2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>LAMPONI SORBETTO</v>
+        <v>FIORDILATTE</v>
       </c>
       <c r="B8">
         <v>3</v>
@@ -634,190 +634,190 @@
         <v>6</v>
       </c>
       <c r="D8">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="E8">
-        <v>176</v>
+        <v>352</v>
       </c>
       <c r="F8" t="str">
-        <v>0.61</v>
+        <v>0.79</v>
       </c>
       <c r="G8" t="str">
-        <v>↑↑</v>
+        <v>↑</v>
       </c>
       <c r="H8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J8" t="str">
-        <v>forecast 5 (7d:6 30d:7 trend:↑↑) +safety 2 -scorta 3</v>
+        <v>forecast 6 (7d:6 30d:21 trend:↑) +safety 2 -scorta 3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>C. VENEZUELA</v>
+        <v>MANGO</v>
       </c>
       <c r="B9">
         <v>2</v>
       </c>
       <c r="C9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D9">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E9">
-        <v>266</v>
+        <v>287</v>
       </c>
       <c r="F9" t="str">
-        <v>0.57</v>
+        <v>0.63</v>
       </c>
       <c r="G9" t="str">
-        <v>→</v>
+        <v>↑↑</v>
       </c>
       <c r="H9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J9" t="str">
-        <v>forecast 4 (7d:4 30d:17 trend:→) +safety 2 -scorta 2</v>
+        <v>forecast 5 (7d:5 30d:15 trend:↑↑) +safety 2 -scorta 2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MANDORLA E ARANCIA</v>
+        <v>MOU LATTE SALATO</v>
       </c>
       <c r="B10">
         <v>0</v>
       </c>
       <c r="C10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E10">
-        <v>39</v>
+        <v>286</v>
       </c>
       <c r="F10" t="str">
-        <v>0.34</v>
+        <v>0.48</v>
       </c>
       <c r="G10" t="str">
         <v>↑↑</v>
       </c>
       <c r="H10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J10" t="str">
-        <v>forecast 3 (7d:3 30d:6 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 4 (7d:4 30d:10 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>PUNCH PARADISE</v>
+        <v>SACRIPANTE</v>
       </c>
       <c r="B11">
         <v>0</v>
       </c>
       <c r="C11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D11">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E11">
-        <v>46</v>
+        <v>98</v>
       </c>
       <c r="F11" t="str">
-        <v>0.30</v>
+        <v>0.46</v>
       </c>
       <c r="G11" t="str">
         <v>↑↑</v>
       </c>
       <c r="H11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J11" t="str">
-        <v>forecast 3 (7d:3 30d:3 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 4 (7d:4 30d:9 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>SACRIPANTE</v>
+        <v>PISTACCHIO LARNAKA</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C12">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D12">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="E12">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="F12" t="str">
-        <v>0.35</v>
+        <v>0.90</v>
       </c>
       <c r="G12" t="str">
-        <v>↑↑</v>
+        <v>↓</v>
       </c>
       <c r="H12">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I12">
         <v>4</v>
       </c>
       <c r="J12" t="str">
-        <v>forecast 3 (7d:3 30d:7 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 7 (7d:6 30d:29 trend:↓) +safety 2 -scorta 5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>PISTACCHIO LARNAKA</v>
+        <v>CHEESECAKE MIRTILLI</v>
       </c>
       <c r="B13">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C13">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D13">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>233</v>
       </c>
       <c r="F13" t="str">
-        <v>0.90</v>
+        <v>0.44</v>
       </c>
       <c r="G13" t="str">
-        <v>↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H13">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J13" t="str">
-        <v>forecast 7 (7d:6 30d:29 trend:↓) +safety 2 -scorta 6</v>
+        <v>forecast 4 (7d:4 30d:7 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MENTA E C.</v>
+        <v>C. VENEZUELA</v>
       </c>
       <c r="B14">
         <v>2</v>
@@ -826,254 +826,254 @@
         <v>4</v>
       </c>
       <c r="D14">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E14">
-        <v>298</v>
+        <v>266</v>
       </c>
       <c r="F14" t="str">
-        <v>0.49</v>
+        <v>0.57</v>
       </c>
       <c r="G14" t="str">
-        <v>↑↑</v>
+        <v>→</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J14" t="str">
-        <v>forecast 4 (7d:4 30d:11 trend:↑↑) +safety 1 -scorta 2</v>
+        <v>forecast 4 (7d:4 30d:17 trend:→) +safety 2 -scorta 2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>MANGO</v>
+        <v>PASSION FRUIT</v>
       </c>
       <c r="B15">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C15">
         <v>4</v>
       </c>
       <c r="D15">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E15">
-        <v>286</v>
+        <v>172</v>
       </c>
       <c r="F15" t="str">
-        <v>0.53</v>
+        <v>0.42</v>
       </c>
       <c r="G15" t="str">
-        <v>↑</v>
+        <v>↑↑</v>
       </c>
       <c r="H15">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J15" t="str">
-        <v>forecast 4 (7d:4 30d:14 trend:↑) +safety 2 -scorta 3</v>
+        <v>forecast 3 (7d:4 30d:6 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>TIRAMISU'</v>
+        <v>V. BANACHI</v>
       </c>
       <c r="B16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E16">
-        <v>261</v>
+        <v>0</v>
       </c>
       <c r="F16" t="str">
-        <v>0.49</v>
+        <v>0.31</v>
       </c>
       <c r="G16" t="str">
         <v>↑↑</v>
       </c>
       <c r="H16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J16" t="str">
-        <v>forecast 4 (7d:4 30d:11 trend:↑↑) +safety 1 -scorta 2</v>
+        <v>forecast 3 (7d:3 30d:4 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ARACHIDI</v>
+        <v>FRAGOLA</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C17">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D17">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="E17">
-        <v>288</v>
+        <v>517</v>
       </c>
       <c r="F17" t="str">
-        <v>0.39</v>
+        <v>1.05</v>
       </c>
       <c r="G17" t="str">
         <v>↑</v>
       </c>
       <c r="H17">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I17">
         <v>3</v>
       </c>
       <c r="J17" t="str">
-        <v>forecast 3 (7d:3 30d:10 trend:↑) +safety 1 -scorta 1</v>
+        <v>forecast 8 (7d:8 30d:27 trend:↑) +safety 3 -scorta 8</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>MOU LATTE SALATO</v>
+        <v>MENTA E C.</v>
       </c>
       <c r="B18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D18">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E18">
-        <v>285</v>
+        <v>298</v>
       </c>
       <c r="F18" t="str">
-        <v>0.38</v>
+        <v>0.49</v>
       </c>
       <c r="G18" t="str">
         <v>↑↑</v>
       </c>
       <c r="H18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I18">
         <v>3</v>
       </c>
       <c r="J18" t="str">
-        <v>forecast 3 (7d:3 30d:9 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 4 (7d:4 30d:11 trend:↑↑) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>PASSION FRUIT</v>
+        <v>LIMONE</v>
       </c>
       <c r="B19">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C19">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D19">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E19">
-        <v>171</v>
+        <v>450</v>
       </c>
       <c r="F19" t="str">
-        <v>0.32</v>
+        <v>0.61</v>
       </c>
       <c r="G19" t="str">
-        <v>↑↑</v>
+        <v>↓</v>
       </c>
       <c r="H19">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I19">
         <v>3</v>
       </c>
       <c r="J19" t="str">
-        <v>forecast 3 (7d:3 30d:5 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 5 (7d:4 30d:20 trend:↓) +safety 2 -scorta 4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>BUONGIORNO AMORE</v>
+        <v>TIRAMISU'</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D20">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E20">
-        <v>153</v>
+        <v>261</v>
       </c>
       <c r="F20" t="str">
-        <v>0.36</v>
+        <v>0.49</v>
       </c>
       <c r="G20" t="str">
         <v>↑↑</v>
       </c>
       <c r="H20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I20">
         <v>3</v>
       </c>
       <c r="J20" t="str">
-        <v>forecast 3 (7d:3 30d:8 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 4 (7d:4 30d:11 trend:↑↑) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>V. GIANDUIA VARIEGATA</v>
+        <v>ARACHIDI</v>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C21">
         <v>2</v>
       </c>
       <c r="D21">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E21">
-        <v>72</v>
+        <v>288</v>
       </c>
       <c r="F21" t="str">
-        <v>0.20</v>
+        <v>0.30</v>
       </c>
       <c r="G21" t="str">
-        <v>↑↑</v>
+        <v>↓</v>
       </c>
       <c r="H21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I21">
         <v>3</v>
       </c>
       <c r="J21" t="str">
-        <v>forecast 2 (7d:2 30d:2 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 3 (7d:2 30d:10 trend:↓) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>BASILICO</v>
+        <v>MANDORLA E ARANCIA</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -1082,13 +1082,13 @@
         <v>2</v>
       </c>
       <c r="D22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E22">
-        <v>233</v>
+        <v>39</v>
       </c>
       <c r="F22" t="str">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="G22" t="str">
         <v>↑↑</v>
@@ -1100,7 +1100,7 @@
         <v>3</v>
       </c>
       <c r="J22" t="str">
-        <v>forecast 2 (7d:2 30d:5 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 2 (7d:2 30d:6 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="23">
@@ -1201,25 +1201,25 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>PENSIERO</v>
+        <v>PUNCH PARADISE</v>
       </c>
       <c r="B26">
         <v>0</v>
       </c>
       <c r="C26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E26">
-        <v>77</v>
+        <v>46</v>
       </c>
       <c r="F26" t="str">
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="G26" t="str">
-        <v>↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H26">
         <v>3</v>
@@ -1228,30 +1228,30 @@
         <v>3</v>
       </c>
       <c r="J26" t="str">
-        <v>forecast 2 (7d:1 30d:5 trend:↓) +safety 1 -scorta 0</v>
+        <v>forecast 2 (7d:2 30d:3 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ROSA E ARANCIA</v>
+        <v>COCONUT RICE CAKE</v>
       </c>
       <c r="B27">
         <v>0</v>
       </c>
       <c r="C27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E27">
         <v>0</v>
       </c>
       <c r="F27" t="str">
-        <v>0.15</v>
+        <v>0.22</v>
       </c>
       <c r="G27" t="str">
-        <v>↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H27">
         <v>3</v>
@@ -1260,190 +1260,190 @@
         <v>3</v>
       </c>
       <c r="J27" t="str">
-        <v>forecast 2 (7d:1 30d:5 trend:↓) +safety 1 -scorta 0</v>
+        <v>forecast 2 (7d:2 30d:4 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>CHEESECAKE MIRTILLI</v>
+        <v>BASILICO</v>
       </c>
       <c r="B28">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C28">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D28">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E28">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F28" t="str">
-        <v>0.42</v>
+        <v>0.15</v>
       </c>
       <c r="G28" t="str">
-        <v>↑↑</v>
+        <v>↓</v>
       </c>
       <c r="H28">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J28" t="str">
-        <v>forecast 3 (7d:4 30d:6 trend:↑↑) +safety 1 -scorta 2</v>
+        <v>forecast 2 (7d:1 30d:5 trend:↓) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>C. E ARANCIA</v>
+        <v>ROSA E ARANCIA</v>
       </c>
       <c r="B29">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C29">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D29">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E29">
-        <v>156</v>
+        <v>0</v>
       </c>
       <c r="F29" t="str">
-        <v>0.35</v>
+        <v>0.15</v>
       </c>
       <c r="G29" t="str">
-        <v>↑↑</v>
+        <v>↓</v>
       </c>
       <c r="H29">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J29" t="str">
-        <v>forecast 3 (7d:3 30d:7 trend:↑↑) +safety 1 -scorta 2</v>
+        <v>forecast 2 (7d:1 30d:5 trend:↓) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>CAFFE'</v>
+        <v>MELA M.C.</v>
       </c>
       <c r="B30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C30">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D30">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E30">
-        <v>240</v>
+        <v>168</v>
       </c>
       <c r="F30" t="str">
-        <v>0.29</v>
+        <v>0.44</v>
       </c>
       <c r="G30" t="str">
-        <v>→</v>
+        <v>↑↑</v>
       </c>
       <c r="H30">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I30">
         <v>2</v>
       </c>
       <c r="J30" t="str">
-        <v>forecast 3 (7d:2 30d:9 trend:→) +safety 1 -scorta 2</v>
+        <v>forecast 4 (7d:4 30d:7 trend:↑↑) +safety 1 -scorta 3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>MANDORLA AL CARDAMOMO</v>
+        <v>C. E ARANCIA</v>
       </c>
       <c r="B31">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D31">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E31">
-        <v>62</v>
+        <v>156</v>
       </c>
       <c r="F31" t="str">
-        <v>0.25</v>
+        <v>0.35</v>
       </c>
       <c r="G31" t="str">
         <v>↑↑</v>
       </c>
       <c r="H31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I31">
         <v>2</v>
       </c>
       <c r="J31" t="str">
-        <v>forecast 2 (7d:2 30d:6 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 3 (7d:3 30d:7 trend:↑↑) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>RISO E VANIGLIA</v>
+        <v>C. MADAGASCAR</v>
       </c>
       <c r="B32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C32">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D32">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E32">
-        <v>140</v>
+        <v>304</v>
       </c>
       <c r="F32" t="str">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="G32" t="str">
-        <v>→</v>
+        <v>↑↑</v>
       </c>
       <c r="H32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I32">
         <v>2</v>
       </c>
       <c r="J32" t="str">
-        <v>forecast 2 (7d:2 30d:8 trend:→) +safety 1 -scorta 1</v>
+        <v>forecast 3 (7d:3 30d:7 trend:↑↑) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>YOGURT</v>
+        <v>COCCO C.</v>
       </c>
       <c r="B33">
         <v>2</v>
       </c>
       <c r="C33">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D33">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E33">
-        <v>111</v>
+        <v>254</v>
       </c>
       <c r="F33" t="str">
-        <v>0.29</v>
+        <v>0.39</v>
       </c>
       <c r="G33" t="str">
-        <v>→</v>
+        <v>↑</v>
       </c>
       <c r="H33">
         <v>4</v>
@@ -1452,12 +1452,12 @@
         <v>2</v>
       </c>
       <c r="J33" t="str">
-        <v>forecast 3 (7d:2 30d:9 trend:→) +safety 1 -scorta 2</v>
+        <v>forecast 3 (7d:3 30d:10 trend:↑) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>V. BANACHI</v>
+        <v>CAFFE'</v>
       </c>
       <c r="B34">
         <v>1</v>
@@ -1466,16 +1466,16 @@
         <v>2</v>
       </c>
       <c r="D34">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E34">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="F34" t="str">
-        <v>0.21</v>
+        <v>0.28</v>
       </c>
       <c r="G34" t="str">
-        <v>↑↑</v>
+        <v>→</v>
       </c>
       <c r="H34">
         <v>3</v>
@@ -1484,30 +1484,30 @@
         <v>2</v>
       </c>
       <c r="J34" t="str">
-        <v>forecast 2 (7d:2 30d:3 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 2 (7d:2 30d:8 trend:→) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ESTASI</v>
+        <v>MANDORLA AL CARDAMOMO</v>
       </c>
       <c r="B35">
         <v>1</v>
       </c>
       <c r="C35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35">
         <v>6</v>
       </c>
       <c r="E35">
-        <v>138</v>
+        <v>62</v>
       </c>
       <c r="F35" t="str">
-        <v>0.17</v>
+        <v>0.25</v>
       </c>
       <c r="G35" t="str">
-        <v>↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H35">
         <v>3</v>
@@ -1516,30 +1516,30 @@
         <v>2</v>
       </c>
       <c r="J35" t="str">
-        <v>forecast 2 (7d:1 30d:6 trend:↓) +safety 1 -scorta 1</v>
+        <v>forecast 2 (7d:2 30d:6 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>RICOTTA E AGRUMI</v>
+        <v>RISO E VANIGLIA</v>
       </c>
       <c r="B36">
         <v>1</v>
       </c>
       <c r="C36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E36">
-        <v>54</v>
+        <v>140</v>
       </c>
       <c r="F36" t="str">
-        <v>0.18</v>
+        <v>0.28</v>
       </c>
       <c r="G36" t="str">
-        <v>↓↓</v>
+        <v>→</v>
       </c>
       <c r="H36">
         <v>3</v>
@@ -1548,478 +1548,478 @@
         <v>2</v>
       </c>
       <c r="J36" t="str">
-        <v>forecast 2 (7d:1 30d:7 trend:↓↓) +safety 1 -scorta 1</v>
+        <v>forecast 2 (7d:2 30d:8 trend:→) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>C. KENTUCKY</v>
+        <v>YOGURT</v>
       </c>
       <c r="B37">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E37">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="F37" t="str">
-        <v>0.14</v>
+        <v>0.29</v>
       </c>
       <c r="G37" t="str">
         <v>→</v>
       </c>
       <c r="H37">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I37">
         <v>2</v>
       </c>
       <c r="J37" t="str">
-        <v>forecast 1 (7d:1 30d:4 trend:→) +safety 1 -scorta 0</v>
+        <v>forecast 3 (7d:2 30d:9 trend:→) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>PANACEA</v>
+        <v>BUONGIORNO AMORE</v>
       </c>
       <c r="B38">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E38">
-        <v>56</v>
+        <v>153</v>
       </c>
       <c r="F38" t="str">
-        <v>0.13</v>
+        <v>0.26</v>
       </c>
       <c r="G38" t="str">
-        <v>↑↑</v>
+        <v>↑</v>
       </c>
       <c r="H38">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I38">
         <v>2</v>
       </c>
       <c r="J38" t="str">
-        <v>forecast 1 (7d:1 30d:3 trend:↑↑) +safety 1 -scorta 0</v>
+        <v>forecast 2 (7d:2 30d:7 trend:↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>AVOCADO</v>
+        <v>ESTASI</v>
       </c>
       <c r="B39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C39">
         <v>1</v>
       </c>
       <c r="D39">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E39">
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="F39" t="str">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="G39" t="str">
-        <v>→</v>
+        <v>↓</v>
       </c>
       <c r="H39">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I39">
         <v>2</v>
       </c>
       <c r="J39" t="str">
-        <v>forecast 1 (7d:1 30d:4 trend:→) +safety 1 -scorta 0</v>
+        <v>forecast 2 (7d:1 30d:5 trend:↓) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>C. PASTICCIERA PARISI</v>
+        <v>RICOTTA E AGRUMI</v>
       </c>
       <c r="B40">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C40">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D40">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E40">
-        <v>248</v>
+        <v>54</v>
       </c>
       <c r="F40" t="str">
-        <v>0.49</v>
+        <v>0.18</v>
       </c>
       <c r="G40" t="str">
-        <v>↑↑</v>
+        <v>↓↓</v>
       </c>
       <c r="H40">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I40">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J40" t="str">
-        <v>forecast 4 (7d:4 30d:11 trend:↑↑) +safety 1 -scorta 4</v>
+        <v>forecast 2 (7d:1 30d:7 trend:↓↓) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>MELONE</v>
+        <v>V. GIANDUIA VARIEGATA</v>
       </c>
       <c r="B41">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C41">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D41">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E41">
-        <v>122</v>
+        <v>72</v>
       </c>
       <c r="F41" t="str">
-        <v>0.32</v>
+        <v>0.11</v>
       </c>
       <c r="G41" t="str">
         <v>↑↑</v>
       </c>
       <c r="H41">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J41" t="str">
-        <v>forecast 3 (7d:3 30d:5 trend:↑↑) +safety 1 -scorta 3</v>
+        <v>forecast 1 (7d:1 30d:2 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>C. CANNELLA</v>
+        <v>C. KENTUCKY</v>
       </c>
       <c r="B42">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C42">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D42">
         <v>4</v>
       </c>
       <c r="E42">
-        <v>33</v>
+        <v>86</v>
       </c>
       <c r="F42" t="str">
-        <v>0.22</v>
+        <v>0.14</v>
       </c>
       <c r="G42" t="str">
-        <v>↑↑</v>
+        <v>→</v>
       </c>
       <c r="H42">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J42" t="str">
-        <v>forecast 2 (7d:2 30d:4 trend:↑↑) +safety 1 -scorta 2</v>
+        <v>forecast 1 (7d:1 30d:4 trend:→) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>MANDORLA BIANCA</v>
+        <v>NOCI UVETTA</v>
       </c>
       <c r="B43">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D43">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E43">
-        <v>103</v>
+        <v>14</v>
       </c>
       <c r="F43" t="str">
-        <v>0.24</v>
+        <v>0.10</v>
       </c>
       <c r="G43" t="str">
         <v>↑↑</v>
       </c>
       <c r="H43">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J43" t="str">
-        <v>forecast 2 (7d:2 30d:5 trend:↑↑) +safety 1 -scorta 2</v>
+        <v>forecast 1 (7d:1 30d:1 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>LIQUIRIZIA</v>
+        <v>PANACEA</v>
       </c>
       <c r="B44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C44">
         <v>1</v>
       </c>
       <c r="D44">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E44">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F44" t="str">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="G44" t="str">
-        <v>→</v>
+        <v>↑↑</v>
       </c>
       <c r="H44">
         <v>2</v>
       </c>
       <c r="I44">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J44" t="str">
-        <v>forecast 1 (7d:1 30d:4 trend:→) +safety 1 -scorta 1</v>
+        <v>forecast 1 (7d:1 30d:3 trend:↑↑) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>MORA</v>
+        <v>PENSIERO</v>
       </c>
       <c r="B45">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C45">
         <v>1</v>
       </c>
       <c r="D45">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E45">
-        <v>11</v>
+        <v>77</v>
       </c>
       <c r="F45" t="str">
-        <v>0.11</v>
+        <v>0.14</v>
       </c>
       <c r="G45" t="str">
-        <v>↑↑</v>
+        <v>→</v>
       </c>
       <c r="H45">
         <v>2</v>
       </c>
       <c r="I45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J45" t="str">
-        <v>forecast 1 (7d:1 30d:2 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 1 (7d:1 30d:4 trend:→) +safety 1 -scorta 0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>V. NOCCIOLA F.</v>
+        <v>C. PASTICCIERA PARISI</v>
       </c>
       <c r="B46">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C46">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D46">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E46">
-        <v>68</v>
+        <v>248</v>
       </c>
       <c r="F46" t="str">
-        <v>0.13</v>
+        <v>0.39</v>
       </c>
       <c r="G46" t="str">
-        <v>↑↑</v>
+        <v>↑</v>
       </c>
       <c r="H46">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I46">
         <v>1</v>
       </c>
       <c r="J46" t="str">
-        <v>forecast 1 (7d:1 30d:3 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 3 (7d:3 30d:10 trend:↑) +safety 1 -scorta 3</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>PEREBH</v>
+        <v>MELONE</v>
       </c>
       <c r="B47">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C47">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D47">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E47">
-        <v>72</v>
+        <v>122</v>
       </c>
       <c r="F47" t="str">
-        <v>0.11</v>
+        <v>0.32</v>
       </c>
       <c r="G47" t="str">
         <v>↑↑</v>
       </c>
       <c r="H47">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I47">
         <v>1</v>
       </c>
       <c r="J47" t="str">
-        <v>forecast 1 (7d:1 30d:2 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 3 (7d:3 30d:5 trend:↑↑) +safety 1 -scorta 3</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>STRACCHINO PERA</v>
+        <v>C. UGANDA</v>
       </c>
       <c r="B48">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C48">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D48">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E48">
-        <v>0</v>
+        <v>254</v>
       </c>
       <c r="F48" t="str">
-        <v>0.11</v>
+        <v>0.31</v>
       </c>
       <c r="G48" t="str">
         <v>↑↑</v>
       </c>
       <c r="H48">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I48">
         <v>1</v>
       </c>
       <c r="J48" t="str">
-        <v>forecast 1 (7d:1 30d:2 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 3 (7d:3 30d:4 trend:↑↑) +safety 1 -scorta 3</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>NOCCIOLA BURRO</v>
+        <v>C. FRAGOLE E MANDORLE</v>
       </c>
       <c r="B49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D49">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E49">
-        <v>0</v>
+        <v>156</v>
       </c>
       <c r="F49" t="str">
-        <v>0.13</v>
+        <v>0.26</v>
       </c>
       <c r="G49" t="str">
-        <v>↑↑</v>
+        <v>↑</v>
       </c>
       <c r="H49">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I49">
         <v>1</v>
       </c>
       <c r="J49" t="str">
-        <v>forecast 1 (7d:1 30d:3 trend:↑↑) +safety 1 -scorta 1</v>
+        <v>forecast 2 (7d:2 30d:7 trend:↑) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>COCONUT RICE CAKE</v>
+        <v>MANDORLA BIANCA</v>
       </c>
       <c r="B50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D50">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E50">
-        <v>0</v>
+        <v>103</v>
       </c>
       <c r="F50" t="str">
-        <v>0.14</v>
+        <v>0.24</v>
       </c>
       <c r="G50" t="str">
-        <v>→</v>
+        <v>↑↑</v>
       </c>
       <c r="H50">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I50">
         <v>1</v>
       </c>
       <c r="J50" t="str">
-        <v>forecast 1 (7d:1 30d:4 trend:→) +safety 1 -scorta 1</v>
+        <v>forecast 2 (7d:2 30d:5 trend:↑↑) +safety 1 -scorta 2</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>V. CASTAGNA E MIRTO</v>
+        <v>C. VANIGLIA</v>
       </c>
       <c r="B51">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C51">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D51">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E51">
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="F51" t="str">
-        <v>0.04</v>
+        <v>0.10</v>
       </c>
       <c r="G51" t="str">
-        <v>↓↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H51">
         <v>2</v>
@@ -2028,30 +2028,30 @@
         <v>1</v>
       </c>
       <c r="J51" t="str">
-        <v>venduto nel mese (3 vasche), assente questa settimana — ordine minimo</v>
+        <v>forecast 1 (7d:1 30d:1 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>C. CRUDO DEL PERU'</v>
+        <v>LIQUIRIZIA</v>
       </c>
       <c r="B52">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C52">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D52">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E52">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="F52" t="str">
-        <v>0.07</v>
+        <v>0.14</v>
       </c>
       <c r="G52" t="str">
-        <v>↓↓</v>
+        <v>→</v>
       </c>
       <c r="H52">
         <v>2</v>
@@ -2060,30 +2060,30 @@
         <v>1</v>
       </c>
       <c r="J52" t="str">
-        <v>venduto nel mese (5 vasche), assente questa settimana — ordine minimo</v>
+        <v>forecast 1 (7d:1 30d:4 trend:→) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>C. ROSEMARY</v>
+        <v>MORA</v>
       </c>
       <c r="B53">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C53">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D53">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E53">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F53" t="str">
-        <v>0.01</v>
+        <v>0.11</v>
       </c>
       <c r="G53" t="str">
-        <v>↓↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H53">
         <v>2</v>
@@ -2092,30 +2092,30 @@
         <v>1</v>
       </c>
       <c r="J53" t="str">
-        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
+        <v>forecast 1 (7d:1 30d:2 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>C. WASABI</v>
+        <v>V. NOCCIOLA F.</v>
       </c>
       <c r="B54">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C54">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D54">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E54">
-        <v>5</v>
+        <v>68</v>
       </c>
       <c r="F54" t="str">
-        <v>0.01</v>
+        <v>0.13</v>
       </c>
       <c r="G54" t="str">
-        <v>↓↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H54">
         <v>2</v>
@@ -2124,30 +2124,30 @@
         <v>1</v>
       </c>
       <c r="J54" t="str">
-        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
+        <v>forecast 1 (7d:1 30d:3 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>V. FIOR DI CIOCCOLATO</v>
+        <v>PEREBH</v>
       </c>
       <c r="B55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D55">
         <v>1</v>
       </c>
       <c r="E55">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="F55" t="str">
-        <v>0.01</v>
+        <v>0.10</v>
       </c>
       <c r="G55" t="str">
-        <v>↓↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H55">
         <v>2</v>
@@ -2156,30 +2156,30 @@
         <v>1</v>
       </c>
       <c r="J55" t="str">
-        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
+        <v>forecast 1 (7d:1 30d:1 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>V. CASTAGNA AL WHISKY</v>
+        <v>SEADAS</v>
       </c>
       <c r="B56">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C56">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D56">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E56">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="F56" t="str">
-        <v>0.01</v>
+        <v>0.13</v>
       </c>
       <c r="G56" t="str">
-        <v>↓↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H56">
         <v>2</v>
@@ -2188,30 +2188,30 @@
         <v>1</v>
       </c>
       <c r="J56" t="str">
-        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
+        <v>forecast 1 (7d:1 30d:3 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>STRACCHINO ALBICOCCHA</v>
+        <v>STRACCHINO PERA</v>
       </c>
       <c r="B57">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C57">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E57">
         <v>0</v>
       </c>
       <c r="F57" t="str">
-        <v>0.01</v>
+        <v>0.11</v>
       </c>
       <c r="G57" t="str">
-        <v>↓↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H57">
         <v>2</v>
@@ -2220,286 +2220,286 @@
         <v>1</v>
       </c>
       <c r="J57" t="str">
-        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
+        <v>forecast 1 (7d:1 30d:2 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>FRAGOLA</v>
+        <v>NOCCIOLA BURRO</v>
       </c>
       <c r="B58">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C58">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D58">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="E58">
-        <v>516</v>
+        <v>0</v>
       </c>
       <c r="F58" t="str">
-        <v>0.95</v>
+        <v>0.13</v>
       </c>
       <c r="G58" t="str">
-        <v>↑</v>
+        <v>↑↑</v>
       </c>
       <c r="H58">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I58">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J58" t="str">
-        <v>scorta (9) copre forecast 7+safety 2 [trend ↑]</v>
+        <v>forecast 1 (7d:1 30d:3 trend:↑↑) +safety 1 -scorta 1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>BANANA E LIME</v>
+        <v>V. CASTAGNA E MIRTO</v>
       </c>
       <c r="B59">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C59">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D59">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E59">
-        <v>141</v>
+        <v>34</v>
       </c>
       <c r="F59" t="str">
-        <v>0.38</v>
+        <v>0.03</v>
       </c>
       <c r="G59" t="str">
-        <v>↑↑</v>
+        <v>↓↓</v>
       </c>
       <c r="H59">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I59">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J59" t="str">
-        <v>scorta (4) copre forecast 3+safety 1 [trend ↑↑]</v>
+        <v>venduto nel mese (2 vasche), assente questa settimana — ordine minimo</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>BIANCANEVE</v>
+        <v>C. CRUDO DEL PERU'</v>
       </c>
       <c r="B60">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C60">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D60">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E60">
-        <v>237</v>
+        <v>37</v>
       </c>
       <c r="F60" t="str">
-        <v>0.36</v>
+        <v>0.07</v>
       </c>
       <c r="G60" t="str">
-        <v>↑↑</v>
+        <v>↓↓</v>
       </c>
       <c r="H60">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I60">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J60" t="str">
-        <v>scorta (4) copre forecast 3+safety 1 [trend ↑↑]</v>
+        <v>venduto nel mese (5 vasche), assente questa settimana — ordine minimo</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>C. AGNESE</v>
+        <v>C. ROSEMARY</v>
       </c>
       <c r="B61">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C61">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D61">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E61">
-        <v>178</v>
+        <v>6</v>
       </c>
       <c r="F61" t="str">
-        <v>0.36</v>
+        <v>0.01</v>
       </c>
       <c r="G61" t="str">
-        <v>↑↑</v>
+        <v>↓↓</v>
       </c>
       <c r="H61">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J61" t="str">
-        <v>scorta (4) copre forecast 3+safety 1 [trend ↑↑]</v>
+        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>LIMONE</v>
+        <v>C. WASABI</v>
       </c>
       <c r="B62">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C62">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D62">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E62">
-        <v>449</v>
+        <v>5</v>
       </c>
       <c r="F62" t="str">
-        <v>0.51</v>
+        <v>0.01</v>
       </c>
       <c r="G62" t="str">
         <v>↓↓</v>
       </c>
       <c r="H62">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I62">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J62" t="str">
-        <v>scorta (6) copre forecast 4+safety 2 [trend ↓↓]</v>
+        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>MELA M.C.</v>
+        <v>V. FIOR DI CIOCCOLATO</v>
       </c>
       <c r="B63">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C63">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D63">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E63">
-        <v>166</v>
+        <v>0</v>
       </c>
       <c r="F63" t="str">
-        <v>0.32</v>
+        <v>0.01</v>
       </c>
       <c r="G63" t="str">
-        <v>↑↑</v>
+        <v>↓↓</v>
       </c>
       <c r="H63">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I63">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J63" t="str">
-        <v>scorta (4) copre forecast 3+safety 1 [trend ↑↑]</v>
+        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>ANGURIA</v>
+        <v>AVOCADO</v>
       </c>
       <c r="B64">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C64">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D64">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E64">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="F64" t="str">
-        <v>0.21</v>
+        <v>0.05</v>
       </c>
       <c r="G64" t="str">
-        <v>↑↑</v>
+        <v>↓↓</v>
       </c>
       <c r="H64">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I64">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J64" t="str">
-        <v>scorta (4) copre forecast 2+safety 1 [trend ↑↑]</v>
+        <v>venduto nel mese (4 vasche), assente questa settimana — ordine minimo</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>C. MADAGASCAR</v>
+        <v>V. CASTAGNA AL WHISKY</v>
       </c>
       <c r="B65">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C65">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D65">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E65">
-        <v>303</v>
+        <v>0</v>
       </c>
       <c r="F65" t="str">
-        <v>0.26</v>
+        <v>0.01</v>
       </c>
       <c r="G65" t="str">
-        <v>↑</v>
+        <v>↓↓</v>
       </c>
       <c r="H65">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I65">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J65" t="str">
-        <v>scorta (3) copre forecast 2+safety 1 [trend ↑]</v>
+        <v>venduto nel mese (1 vasche), assente questa settimana — ordine minimo</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>COCCO C.</v>
+        <v>BANANA E LIME</v>
       </c>
       <c r="B66">
         <v>4</v>
       </c>
       <c r="C66">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D66">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E66">
-        <v>253</v>
+        <v>141</v>
       </c>
       <c r="F66" t="str">
-        <v>0.30</v>
+        <v>0.38</v>
       </c>
       <c r="G66" t="str">
-        <v>↓</v>
+        <v>↑↑</v>
       </c>
       <c r="H66">
         <v>4</v>
@@ -2508,30 +2508,30 @@
         <v>0</v>
       </c>
       <c r="J66" t="str">
-        <v>scorta (4) copre forecast 3+safety 1 [trend ↓]</v>
+        <v>scorta (4) copre forecast 3+safety 1 [trend ↑↑]</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>C. FRAGOLE E MANDORLE</v>
+        <v>BIANCANEVE</v>
       </c>
       <c r="B67">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C67">
         <v>2</v>
       </c>
       <c r="D67">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E67">
-        <v>155</v>
+        <v>237</v>
       </c>
       <c r="F67" t="str">
-        <v>0.26</v>
+        <v>0.28</v>
       </c>
       <c r="G67" t="str">
-        <v>↑</v>
+        <v>→</v>
       </c>
       <c r="H67">
         <v>3</v>
@@ -2540,12 +2540,12 @@
         <v>0</v>
       </c>
       <c r="J67" t="str">
-        <v>scorta (3) copre forecast 2+safety 1 [trend ↑]</v>
+        <v>scorta (4) copre forecast 2+safety 1 [trend →]</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>MELOGRANO</v>
+        <v>C. AGNESE</v>
       </c>
       <c r="B68">
         <v>4</v>
@@ -2554,16 +2554,16 @@
         <v>2</v>
       </c>
       <c r="D68">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E68">
-        <v>30</v>
+        <v>178</v>
       </c>
       <c r="F68" t="str">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="G68" t="str">
-        <v>↑↑</v>
+        <v>↑</v>
       </c>
       <c r="H68">
         <v>3</v>
@@ -2572,12 +2572,12 @@
         <v>0</v>
       </c>
       <c r="J68" t="str">
-        <v>scorta (4) copre forecast 2+safety 1 [trend ↑↑]</v>
+        <v>scorta (4) copre forecast 2+safety 1 [trend ↑]</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>C. UGANDA</v>
+        <v>MELOGRANO</v>
       </c>
       <c r="B69">
         <v>4</v>
@@ -2586,13 +2586,13 @@
         <v>2</v>
       </c>
       <c r="D69">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E69">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F69" t="str">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="G69" t="str">
         <v>↑↑</v>
@@ -2609,22 +2609,22 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>C. LAPSANG SOUCHOUNG</v>
+        <v>ANGURIA</v>
       </c>
       <c r="B70">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C70">
         <v>1</v>
       </c>
       <c r="D70">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E70">
-        <v>5</v>
+        <v>98</v>
       </c>
       <c r="F70" t="str">
-        <v>0.10</v>
+        <v>0.13</v>
       </c>
       <c r="G70" t="str">
         <v>↑↑</v>
@@ -2636,12 +2636,12 @@
         <v>0</v>
       </c>
       <c r="J70" t="str">
-        <v>scorta (2) copre forecast 1+safety 1 [trend ↑↑]</v>
+        <v>scorta (4) copre forecast 1+safety 1 [trend ↑↑]</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>SEADAS</v>
+        <v>C. LAPSANG SOUCHOUNG</v>
       </c>
       <c r="B71">
         <v>2</v>
@@ -2650,13 +2650,13 @@
         <v>1</v>
       </c>
       <c r="D71">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E71">
-        <v>102</v>
+        <v>5</v>
       </c>
       <c r="F71" t="str">
-        <v>0.13</v>
+        <v>0.10</v>
       </c>
       <c r="G71" t="str">
         <v>↑↑</v>
@@ -2673,7 +2673,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>UVA E NOCI</v>
+        <v>C. CANNELLA</v>
       </c>
       <c r="B72">
         <v>2</v>
@@ -2682,16 +2682,16 @@
         <v>1</v>
       </c>
       <c r="D72">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E72">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F72" t="str">
-        <v>0.10</v>
+        <v>0.14</v>
       </c>
       <c r="G72" t="str">
-        <v>↑↑</v>
+        <v>→</v>
       </c>
       <c r="H72">
         <v>2</v>
@@ -2700,12 +2700,12 @@
         <v>0</v>
       </c>
       <c r="J72" t="str">
-        <v>scorta (2) copre forecast 1+safety 1 [trend ↑↑]</v>
+        <v>scorta (2) copre forecast 1+safety 1 [trend →]</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>VENERE ROSA</v>
+        <v>UVA E NOCI</v>
       </c>
       <c r="B73">
         <v>2</v>
@@ -2714,13 +2714,13 @@
         <v>1</v>
       </c>
       <c r="D73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E73">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="F73" t="str">
-        <v>0.11</v>
+        <v>0.10</v>
       </c>
       <c r="G73" t="str">
         <v>↑↑</v>
@@ -2801,7 +2801,7 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>C. AL PIMENTO</v>
+        <v>BAKLAVA</v>
       </c>
       <c r="B76">
         <v>2</v>
@@ -2813,7 +2813,7 @@
         <v>0</v>
       </c>
       <c r="E76">
-        <v>3</v>
+        <v>133</v>
       </c>
       <c r="F76" t="str">
         <v>0.00</v>
@@ -2833,10 +2833,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>C. BIANCO</v>
+        <v>C. AL PIMENTO</v>
       </c>
       <c r="B77">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C77">
         <v>0</v>
@@ -2845,7 +2845,7 @@
         <v>0</v>
       </c>
       <c r="E77">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="F77" t="str">
         <v>0.00</v>
@@ -2865,10 +2865,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>C. VANIGLIA</v>
+        <v>C. BIANCO</v>
       </c>
       <c r="B78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C78">
         <v>0</v>
@@ -2877,7 +2877,7 @@
         <v>0</v>
       </c>
       <c r="E78">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="F78" t="str">
         <v>0.00</v>
@@ -2897,103 +2897,103 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>C. ZENZERO</v>
+        <v>C. BANANA</v>
       </c>
       <c r="B79">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C79">
         <v>0</v>
       </c>
       <c r="D79">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E79">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="F79" t="str">
-        <v>0.04</v>
+        <v>0.00</v>
       </c>
       <c r="G79" t="str">
-        <v>↓↓</v>
+        <v>→</v>
       </c>
       <c r="H79">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I79">
         <v>0</v>
       </c>
       <c r="J79" t="str">
-        <v>nessuna vendita 7gg (30gg: 3, scorta: 3)</v>
+        <v>nessuna vendita 30gg</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>FRUTTI DI BOSCO</v>
+        <v>C. ZENZERO</v>
       </c>
       <c r="B80">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C80">
         <v>0</v>
       </c>
       <c r="D80">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E80">
-        <v>125</v>
+        <v>67</v>
       </c>
       <c r="F80" t="str">
-        <v>0.16</v>
+        <v>0.04</v>
       </c>
       <c r="G80" t="str">
         <v>↓↓</v>
       </c>
       <c r="H80">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I80">
         <v>0</v>
       </c>
       <c r="J80" t="str">
-        <v>nessuna vendita 7gg (30gg: 12, scorta: 6)</v>
+        <v>nessuna vendita 7gg (30gg: 3, scorta: 3)</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>GIANDUIA</v>
+        <v>FRUTTI DI BOSCO</v>
       </c>
       <c r="B81">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C81">
         <v>0</v>
       </c>
       <c r="D81">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E81">
-        <v>77</v>
+        <v>125</v>
       </c>
       <c r="F81" t="str">
-        <v>0.04</v>
+        <v>0.16</v>
       </c>
       <c r="G81" t="str">
         <v>↓↓</v>
       </c>
       <c r="H81">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I81">
         <v>0</v>
       </c>
       <c r="J81" t="str">
-        <v>nessuna vendita 7gg (30gg: 3, scorta: 1)</v>
+        <v>nessuna vendita 7gg (30gg: 12, scorta: 6)</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>LEMON CURD</v>
+        <v>GIANDUIA</v>
       </c>
       <c r="B82">
         <v>1</v>
@@ -3002,13 +3002,13 @@
         <v>0</v>
       </c>
       <c r="D82">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E82">
-        <v>26</v>
+        <v>77</v>
       </c>
       <c r="F82" t="str">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="G82" t="str">
         <v>↓↓</v>
@@ -3020,27 +3020,27 @@
         <v>0</v>
       </c>
       <c r="J82" t="str">
-        <v>nessuna vendita 7gg (30gg: 2, scorta: 1)</v>
+        <v>nessuna vendita 7gg (30gg: 3, scorta: 1)</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>MIRTILLO</v>
+        <v>LEMON CURD</v>
       </c>
       <c r="B83">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C83">
         <v>0</v>
       </c>
       <c r="D83">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E83">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="F83" t="str">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="G83" t="str">
         <v>↓↓</v>
@@ -3052,27 +3052,27 @@
         <v>0</v>
       </c>
       <c r="J83" t="str">
-        <v>nessuna vendita 7gg (30gg: 3, scorta: 2)</v>
+        <v>nessuna vendita 7gg (30gg: 2, scorta: 1)</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>PAPAYA</v>
+        <v>MIRTILLO</v>
       </c>
       <c r="B84">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C84">
         <v>0</v>
       </c>
       <c r="D84">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E84">
-        <v>21</v>
+        <v>76</v>
       </c>
       <c r="F84" t="str">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="G84" t="str">
         <v>↓↓</v>
@@ -3084,27 +3084,27 @@
         <v>0</v>
       </c>
       <c r="J84" t="str">
-        <v>nessuna vendita 7gg (30gg: 2, scorta: 1)</v>
+        <v>nessuna vendita 7gg (30gg: 3, scorta: 2)</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>PESCHE AL VINO</v>
+        <v>PAPAYA</v>
       </c>
       <c r="B85">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C85">
         <v>0</v>
       </c>
       <c r="D85">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E85">
-        <v>83</v>
+        <v>21</v>
       </c>
       <c r="F85" t="str">
-        <v>0.07</v>
+        <v>0.03</v>
       </c>
       <c r="G85" t="str">
         <v>↓↓</v>
@@ -3116,27 +3116,27 @@
         <v>0</v>
       </c>
       <c r="J85" t="str">
-        <v>nessuna vendita 7gg (30gg: 5, scorta: 3)</v>
+        <v>nessuna vendita 7gg (30gg: 2, scorta: 1)</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>RICOTTA E COCCO</v>
+        <v>PESCHE AL VINO</v>
       </c>
       <c r="B86">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C86">
         <v>0</v>
       </c>
       <c r="D86">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E86">
-        <v>17</v>
+        <v>83</v>
       </c>
       <c r="F86" t="str">
-        <v>0.04</v>
+        <v>0.07</v>
       </c>
       <c r="G86" t="str">
         <v>↓↓</v>
@@ -3148,12 +3148,12 @@
         <v>0</v>
       </c>
       <c r="J86" t="str">
-        <v>nessuna vendita 7gg (30gg: 3, scorta: 2)</v>
+        <v>nessuna vendita 7gg (30gg: 5, scorta: 3)</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>LAVANDA</v>
+        <v>RICOTTA E COCCO</v>
       </c>
       <c r="B87">
         <v>2</v>
@@ -3162,13 +3162,13 @@
         <v>0</v>
       </c>
       <c r="D87">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E87">
-        <v>106</v>
+        <v>17</v>
       </c>
       <c r="F87" t="str">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="G87" t="str">
         <v>↓↓</v>
@@ -3180,27 +3180,27 @@
         <v>0</v>
       </c>
       <c r="J87" t="str">
-        <v>nessuna vendita 7gg (30gg: 2, scorta: 2)</v>
+        <v>nessuna vendita 7gg (30gg: 3, scorta: 2)</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>TE VERDE MATCHA</v>
+        <v>VENERE ROSA</v>
       </c>
       <c r="B88">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C88">
         <v>0</v>
       </c>
       <c r="D88">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E88">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F88" t="str">
-        <v>0.08</v>
+        <v>0.03</v>
       </c>
       <c r="G88" t="str">
         <v>↓↓</v>
@@ -3212,12 +3212,12 @@
         <v>0</v>
       </c>
       <c r="J88" t="str">
-        <v>nessuna vendita 7gg (30gg: 6, scorta: 3)</v>
+        <v>nessuna vendita 7gg (30gg: 2, scorta: 2)</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>CARROT CAKE</v>
+        <v>LAVANDA</v>
       </c>
       <c r="B89">
         <v>2</v>
@@ -3226,45 +3226,45 @@
         <v>0</v>
       </c>
       <c r="D89">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E89">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="F89" t="str">
-        <v>0.00</v>
+        <v>0.03</v>
       </c>
       <c r="G89" t="str">
-        <v>→</v>
+        <v>↓↓</v>
       </c>
       <c r="H89">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I89">
         <v>0</v>
       </c>
       <c r="J89" t="str">
-        <v>nessuna vendita 30gg</v>
+        <v>nessuna vendita 7gg (30gg: 2, scorta: 2)</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>RICOTTA E PERA</v>
+        <v>TE VERDE MATCHA</v>
       </c>
       <c r="B90">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C90">
         <v>0</v>
       </c>
       <c r="D90">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E90">
         <v>0</v>
       </c>
       <c r="F90" t="str">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="G90" t="str">
         <v>↓↓</v>
@@ -3276,59 +3276,59 @@
         <v>0</v>
       </c>
       <c r="J90" t="str">
-        <v>nessuna vendita 7gg (30gg: 3, scorta: 1)</v>
+        <v>nessuna vendita 7gg (30gg: 6, scorta: 2)</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>V.BRONTE GREEN</v>
+        <v>CARROT CAKE</v>
       </c>
       <c r="B91">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C91">
         <v>0</v>
       </c>
       <c r="D91">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E91">
         <v>0</v>
       </c>
       <c r="F91" t="str">
-        <v>0.03</v>
+        <v>0.00</v>
       </c>
       <c r="G91" t="str">
-        <v>↓↓</v>
+        <v>→</v>
       </c>
       <c r="H91">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I91">
         <v>0</v>
       </c>
       <c r="J91" t="str">
-        <v>nessuna vendita 7gg (30gg: 2, scorta: 1)</v>
+        <v>nessuna vendita 30gg</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>SACHER TORTE</v>
+        <v>DRACARYS</v>
       </c>
       <c r="B92">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C92">
         <v>0</v>
       </c>
       <c r="D92">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E92">
         <v>0</v>
       </c>
       <c r="F92" t="str">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="G92" t="str">
         <v>↓↓</v>
@@ -3340,44 +3340,236 @@
         <v>0</v>
       </c>
       <c r="J92" t="str">
-        <v>nessuna vendita 7gg (30gg: 2, scorta: 2)</v>
+        <v>nessuna vendita 7gg (30gg: 1, scorta: 1)</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
+        <v>PAMPANELLA</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93">
+        <v>0</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93">
+        <v>0</v>
+      </c>
+      <c r="F93" t="str">
+        <v>0.00</v>
+      </c>
+      <c r="G93" t="str">
+        <v>→</v>
+      </c>
+      <c r="H93">
+        <v>0</v>
+      </c>
+      <c r="I93">
+        <v>0</v>
+      </c>
+      <c r="J93" t="str">
+        <v>nessuna vendita 30gg</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>RICOTTA E PERA</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94">
+        <v>0</v>
+      </c>
+      <c r="D94">
+        <v>3</v>
+      </c>
+      <c r="E94">
+        <v>0</v>
+      </c>
+      <c r="F94" t="str">
+        <v>0.04</v>
+      </c>
+      <c r="G94" t="str">
+        <v>↓↓</v>
+      </c>
+      <c r="H94">
+        <v>2</v>
+      </c>
+      <c r="I94">
+        <v>0</v>
+      </c>
+      <c r="J94" t="str">
+        <v>nessuna vendita 7gg (30gg: 3, scorta: 1)</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>V.BRONTE GREEN</v>
+      </c>
+      <c r="B95">
+        <v>1</v>
+      </c>
+      <c r="C95">
+        <v>0</v>
+      </c>
+      <c r="D95">
+        <v>2</v>
+      </c>
+      <c r="E95">
+        <v>0</v>
+      </c>
+      <c r="F95" t="str">
+        <v>0.03</v>
+      </c>
+      <c r="G95" t="str">
+        <v>↓↓</v>
+      </c>
+      <c r="H95">
+        <v>2</v>
+      </c>
+      <c r="I95">
+        <v>0</v>
+      </c>
+      <c r="J95" t="str">
+        <v>nessuna vendita 7gg (30gg: 2, scorta: 1)</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>SACHER TORTE</v>
+      </c>
+      <c r="B96">
+        <v>2</v>
+      </c>
+      <c r="C96">
+        <v>0</v>
+      </c>
+      <c r="D96">
+        <v>2</v>
+      </c>
+      <c r="E96">
+        <v>0</v>
+      </c>
+      <c r="F96" t="str">
+        <v>0.03</v>
+      </c>
+      <c r="G96" t="str">
+        <v>↓↓</v>
+      </c>
+      <c r="H96">
+        <v>2</v>
+      </c>
+      <c r="I96">
+        <v>0</v>
+      </c>
+      <c r="J96" t="str">
+        <v>nessuna vendita 7gg (30gg: 2, scorta: 2)</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>FRAGOLE CHAMP</v>
+      </c>
+      <c r="B97">
+        <v>3</v>
+      </c>
+      <c r="C97">
+        <v>0</v>
+      </c>
+      <c r="D97">
+        <v>1</v>
+      </c>
+      <c r="E97">
+        <v>0</v>
+      </c>
+      <c r="F97" t="str">
+        <v>0.01</v>
+      </c>
+      <c r="G97" t="str">
+        <v>↓↓</v>
+      </c>
+      <c r="H97">
+        <v>2</v>
+      </c>
+      <c r="I97">
+        <v>0</v>
+      </c>
+      <c r="J97" t="str">
+        <v>nessuna vendita 7gg (30gg: 1, scorta: 3)</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
         <v>ZABAIONE GELATO</v>
       </c>
-      <c r="B93">
-        <v>3</v>
-      </c>
-      <c r="C93">
-        <v>0</v>
-      </c>
-      <c r="D93">
-        <v>4</v>
-      </c>
-      <c r="E93">
+      <c r="B98">
+        <v>3</v>
+      </c>
+      <c r="C98">
+        <v>0</v>
+      </c>
+      <c r="D98">
+        <v>4</v>
+      </c>
+      <c r="E98">
         <v>127</v>
       </c>
-      <c r="F93" t="str">
+      <c r="F98" t="str">
         <v>0.05</v>
       </c>
-      <c r="G93" t="str">
+      <c r="G98" t="str">
         <v>↓↓</v>
       </c>
-      <c r="H93">
-        <v>2</v>
-      </c>
-      <c r="I93">
-        <v>0</v>
-      </c>
-      <c r="J93" t="str">
+      <c r="H98">
+        <v>2</v>
+      </c>
+      <c r="I98">
+        <v>0</v>
+      </c>
+      <c r="J98" t="str">
         <v>nessuna vendita 7gg (30gg: 4, scorta: 3)</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>SPRITZ</v>
+      </c>
+      <c r="B99">
+        <v>1</v>
+      </c>
+      <c r="C99">
+        <v>0</v>
+      </c>
+      <c r="D99">
+        <v>0</v>
+      </c>
+      <c r="E99">
+        <v>0</v>
+      </c>
+      <c r="F99" t="str">
+        <v>0.00</v>
+      </c>
+      <c r="G99" t="str">
+        <v>→</v>
+      </c>
+      <c r="H99">
+        <v>0</v>
+      </c>
+      <c r="I99">
+        <v>0</v>
+      </c>
+      <c r="J99" t="str">
+        <v>nessuna vendita 30gg</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J93"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J99"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>